<commit_message>
sync latest prices into docs/
</commit_message>
<xml_diff>
--- a/docs/herblore_top8.xlsx
+++ b/docs/herblore_top8.xlsx
@@ -97,7 +97,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Last price update: 2026-09-14 08:46 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
+          <t xml:space="preserve">Last price update: 2026-09-14 08:56 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
         </is>
       </c>
     </row>
@@ -3978,7 +3978,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4062,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4146,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -4209,7 +4209,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -4377,7 +4377,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4608,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4713,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -4734,7 +4734,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -4902,7 +4902,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -4923,7 +4923,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -4965,7 +4965,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -5238,7 +5238,7 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5259,7 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -5322,7 +5322,7 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -5406,7 +5406,7 @@
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -5427,7 +5427,7 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5469,7 @@
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -5553,7 +5553,7 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -5574,7 +5574,7 @@
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -5595,7 +5595,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5637,7 @@
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5679,7 @@
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -5763,7 +5763,7 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -5931,7 +5931,7 @@
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -5952,7 +5952,7 @@
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -5973,7 +5973,7 @@
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -5994,7 +5994,7 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -6015,7 +6015,7 @@
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -6057,7 +6057,7 @@
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6120,7 @@
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6141,7 @@
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -6162,7 +6162,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -6225,7 +6225,7 @@
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -6246,7 +6246,7 @@
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6267,7 @@
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6288,7 @@
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6372,7 @@
       </c>
       <c r="E116" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -6393,7 +6393,7 @@
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -6414,7 +6414,7 @@
       </c>
       <c r="E118" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -6456,7 +6456,7 @@
       </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="E121" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="E124" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -6582,7 +6582,7 @@
       </c>
       <c r="E126" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -6666,7 +6666,7 @@
       </c>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -6687,7 +6687,7 @@
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -6729,7 +6729,7 @@
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -6750,7 +6750,7 @@
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -6792,7 +6792,7 @@
       </c>
       <c r="E136" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -6813,7 +6813,7 @@
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -6834,7 +6834,7 @@
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="E140" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -6897,7 +6897,7 @@
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -6918,7 +6918,7 @@
       </c>
       <c r="E142" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -6939,7 +6939,7 @@
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -6960,7 +6960,7 @@
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -6981,7 +6981,7 @@
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -7002,7 +7002,7 @@
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7023,7 @@
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -7044,7 +7044,7 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -7086,7 +7086,7 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -7107,7 +7107,7 @@
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -7128,7 +7128,7 @@
       </c>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7149,7 @@
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -7170,7 +7170,7 @@
       </c>
       <c r="E154" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -7229,7 +7229,7 @@
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="E158" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -7292,7 +7292,7 @@
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -7355,7 +7355,7 @@
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="E164" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -7397,7 +7397,7 @@
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7418,7 @@
       </c>
       <c r="E166" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7439,7 @@
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -7460,7 +7460,7 @@
       </c>
       <c r="E168" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -7481,7 +7481,7 @@
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -7502,7 +7502,7 @@
       </c>
       <c r="E170" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -7523,7 +7523,7 @@
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -7544,7 +7544,7 @@
       </c>
       <c r="E172" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>
@@ -7586,7 +7586,7 @@
       </c>
       <c r="E174" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:46</t>
+          <t xml:space="preserve">2026-09-14 08:56</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
prices: 2026-09-14 15:59 UTC
</commit_message>
<xml_diff>
--- a/docs/herblore_top8.xlsx
+++ b/docs/herblore_top8.xlsx
@@ -97,7 +97,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Last price update: 2026-09-14 08:56 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
+          <t xml:space="preserve">Last price update: 2026-09-14 15:59 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
         </is>
       </c>
     </row>
@@ -3978,7 +3978,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4062,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4146,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -4209,7 +4209,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -4377,7 +4377,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4608,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4713,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -4734,7 +4734,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -4902,7 +4902,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -4923,7 +4923,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -4965,7 +4965,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -5238,7 +5238,7 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5259,7 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -5322,7 +5322,7 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -5406,7 +5406,7 @@
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -5427,7 +5427,7 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5469,7 @@
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -5553,7 +5553,7 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -5574,7 +5574,7 @@
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -5595,7 +5595,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5637,7 @@
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5679,7 @@
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -5763,7 +5763,7 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -5931,7 +5931,7 @@
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -5952,7 +5952,7 @@
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -5973,7 +5973,7 @@
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -5994,7 +5994,7 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -6015,7 +6015,7 @@
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -6057,7 +6057,7 @@
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6120,7 @@
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6141,7 @@
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -6162,7 +6162,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -6225,7 +6225,7 @@
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -6246,7 +6246,7 @@
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6267,7 @@
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6288,7 @@
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6372,7 @@
       </c>
       <c r="E116" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -6393,7 +6393,7 @@
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -6414,7 +6414,7 @@
       </c>
       <c r="E118" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -6456,7 +6456,7 @@
       </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="E121" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="E124" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -6582,7 +6582,7 @@
       </c>
       <c r="E126" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -6666,7 +6666,7 @@
       </c>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -6687,7 +6687,7 @@
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -6729,7 +6729,7 @@
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -6750,7 +6750,7 @@
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -6792,7 +6792,7 @@
       </c>
       <c r="E136" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -6813,7 +6813,7 @@
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -6834,7 +6834,7 @@
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="E140" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -6897,7 +6897,7 @@
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -6918,7 +6918,7 @@
       </c>
       <c r="E142" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -6939,7 +6939,7 @@
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -6960,7 +6960,7 @@
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -6981,7 +6981,7 @@
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -7002,7 +7002,7 @@
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7023,7 @@
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -7044,7 +7044,7 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -7086,7 +7086,7 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -7107,7 +7107,7 @@
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -7128,7 +7128,7 @@
       </c>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7149,7 @@
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -7170,7 +7170,7 @@
       </c>
       <c r="E154" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -7229,7 +7229,7 @@
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="E158" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -7292,7 +7292,7 @@
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -7355,7 +7355,7 @@
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="E164" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -7397,7 +7397,7 @@
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7418,7 @@
       </c>
       <c r="E166" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7439,7 @@
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -7460,7 +7460,7 @@
       </c>
       <c r="E168" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -7481,7 +7481,7 @@
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -7502,7 +7502,7 @@
       </c>
       <c r="E170" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -7523,7 +7523,7 @@
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -7544,7 +7544,7 @@
       </c>
       <c r="E172" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>
@@ -7586,7 +7586,7 @@
       </c>
       <c r="E174" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 08:56</t>
+          <t xml:space="preserve">2026-09-14 15:59</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
prices: 2026-09-14 17:29 UTC
</commit_message>
<xml_diff>
--- a/docs/herblore_top8.xlsx
+++ b/docs/herblore_top8.xlsx
@@ -97,7 +97,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Last price update: 2026-09-14 15:59 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
+          <t xml:space="preserve">Last price update: 2026-09-14 17:29 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
         </is>
       </c>
     </row>
@@ -3978,7 +3978,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4062,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4146,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -4209,7 +4209,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -4377,7 +4377,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4608,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4713,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -4734,7 +4734,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -4902,7 +4902,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -4923,7 +4923,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -4965,7 +4965,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -5238,7 +5238,7 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5259,7 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -5322,7 +5322,7 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -5406,7 +5406,7 @@
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -5427,7 +5427,7 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5469,7 @@
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -5553,7 +5553,7 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -5574,7 +5574,7 @@
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -5595,7 +5595,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5637,7 @@
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5679,7 @@
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -5763,7 +5763,7 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -5931,7 +5931,7 @@
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -5952,7 +5952,7 @@
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -5973,7 +5973,7 @@
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -5994,7 +5994,7 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -6015,7 +6015,7 @@
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -6057,7 +6057,7 @@
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6120,7 @@
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6141,7 @@
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -6162,7 +6162,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -6225,7 +6225,7 @@
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -6246,7 +6246,7 @@
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6267,7 @@
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6288,7 @@
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6372,7 @@
       </c>
       <c r="E116" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -6393,7 +6393,7 @@
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -6414,7 +6414,7 @@
       </c>
       <c r="E118" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -6456,7 +6456,7 @@
       </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="E121" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="E124" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -6582,7 +6582,7 @@
       </c>
       <c r="E126" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -6666,7 +6666,7 @@
       </c>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -6687,7 +6687,7 @@
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -6729,7 +6729,7 @@
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -6750,7 +6750,7 @@
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -6792,7 +6792,7 @@
       </c>
       <c r="E136" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -6813,7 +6813,7 @@
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -6834,7 +6834,7 @@
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="E140" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -6897,7 +6897,7 @@
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -6918,7 +6918,7 @@
       </c>
       <c r="E142" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -6939,7 +6939,7 @@
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -6960,7 +6960,7 @@
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -6981,7 +6981,7 @@
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -7002,7 +7002,7 @@
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7023,7 @@
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -7044,7 +7044,7 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -7086,7 +7086,7 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -7107,7 +7107,7 @@
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -7128,7 +7128,7 @@
       </c>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7149,7 @@
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -7170,7 +7170,7 @@
       </c>
       <c r="E154" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -7229,7 +7229,7 @@
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="E158" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -7292,7 +7292,7 @@
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -7355,7 +7355,7 @@
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="E164" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -7397,7 +7397,7 @@
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7418,7 @@
       </c>
       <c r="E166" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7439,7 @@
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -7460,7 +7460,7 @@
       </c>
       <c r="E168" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -7481,7 +7481,7 @@
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -7502,7 +7502,7 @@
       </c>
       <c r="E170" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -7523,7 +7523,7 @@
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -7544,7 +7544,7 @@
       </c>
       <c r="E172" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>
@@ -7586,7 +7586,7 @@
       </c>
       <c r="E174" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 15:59</t>
+          <t xml:space="preserve">2026-09-14 17:29</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
prices: 2026-09-14 20:10 UTC
</commit_message>
<xml_diff>
--- a/docs/herblore_top8.xlsx
+++ b/docs/herblore_top8.xlsx
@@ -97,7 +97,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Last price update: 2026-09-14 17:29 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
+          <t xml:space="preserve">Last price update: 2026-09-14 20:10 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
         </is>
       </c>
     </row>
@@ -3978,7 +3978,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4062,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4146,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -4209,7 +4209,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -4377,7 +4377,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4608,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4713,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -4734,7 +4734,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -4902,7 +4902,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -4923,7 +4923,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -4965,7 +4965,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -5238,7 +5238,7 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5259,7 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -5322,7 +5322,7 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -5406,7 +5406,7 @@
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -5427,7 +5427,7 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5469,7 @@
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -5553,7 +5553,7 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -5574,7 +5574,7 @@
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -5595,7 +5595,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5637,7 @@
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5679,7 @@
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -5763,7 +5763,7 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -5931,7 +5931,7 @@
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -5952,7 +5952,7 @@
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -5973,7 +5973,7 @@
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -5994,7 +5994,7 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -6015,7 +6015,7 @@
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -6057,7 +6057,7 @@
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6120,7 @@
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6141,7 @@
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -6162,7 +6162,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -6225,7 +6225,7 @@
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -6246,7 +6246,7 @@
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6267,7 @@
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6288,7 @@
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6372,7 @@
       </c>
       <c r="E116" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -6393,7 +6393,7 @@
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -6414,7 +6414,7 @@
       </c>
       <c r="E118" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -6456,7 +6456,7 @@
       </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="E121" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="E124" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -6582,7 +6582,7 @@
       </c>
       <c r="E126" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -6666,7 +6666,7 @@
       </c>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -6687,7 +6687,7 @@
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -6729,7 +6729,7 @@
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -6750,7 +6750,7 @@
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -6792,7 +6792,7 @@
       </c>
       <c r="E136" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -6813,7 +6813,7 @@
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -6834,7 +6834,7 @@
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="E140" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -6897,7 +6897,7 @@
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -6918,7 +6918,7 @@
       </c>
       <c r="E142" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -6939,7 +6939,7 @@
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -6960,7 +6960,7 @@
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -6981,7 +6981,7 @@
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -7002,7 +7002,7 @@
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7023,7 @@
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -7044,7 +7044,7 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -7086,7 +7086,7 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -7107,7 +7107,7 @@
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -7128,7 +7128,7 @@
       </c>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7149,7 @@
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -7170,7 +7170,7 @@
       </c>
       <c r="E154" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -7229,7 +7229,7 @@
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="E158" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -7292,7 +7292,7 @@
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -7355,7 +7355,7 @@
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="E164" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -7397,7 +7397,7 @@
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7418,7 @@
       </c>
       <c r="E166" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7439,7 @@
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -7460,7 +7460,7 @@
       </c>
       <c r="E168" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -7481,7 +7481,7 @@
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -7502,7 +7502,7 @@
       </c>
       <c r="E170" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -7523,7 +7523,7 @@
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -7544,7 +7544,7 @@
       </c>
       <c r="E172" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>
@@ -7586,7 +7586,7 @@
       </c>
       <c r="E174" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 17:29</t>
+          <t xml:space="preserve">2026-09-14 20:10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
prices: 2026-09-14 20:23 UTC
</commit_message>
<xml_diff>
--- a/docs/herblore_top8.xlsx
+++ b/docs/herblore_top8.xlsx
@@ -97,7 +97,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Last price update: 2026-09-14 20:10 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
+          <t xml:space="preserve">Last price update: 2026-09-14 20:23 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
         </is>
       </c>
     </row>
@@ -3978,7 +3978,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4062,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4146,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -4209,7 +4209,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -4377,7 +4377,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4608,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4713,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -4734,7 +4734,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -4902,7 +4902,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -4923,7 +4923,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -4965,7 +4965,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -5238,7 +5238,7 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5259,7 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -5322,7 +5322,7 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -5406,7 +5406,7 @@
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -5427,7 +5427,7 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5469,7 @@
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -5553,7 +5553,7 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -5574,7 +5574,7 @@
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -5595,7 +5595,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5637,7 @@
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5679,7 @@
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -5763,7 +5763,7 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -5931,7 +5931,7 @@
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -5952,7 +5952,7 @@
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -5973,7 +5973,7 @@
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -5994,7 +5994,7 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -6015,7 +6015,7 @@
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -6057,7 +6057,7 @@
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6120,7 @@
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6141,7 @@
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -6162,7 +6162,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -6225,7 +6225,7 @@
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -6246,7 +6246,7 @@
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6267,7 @@
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6288,7 @@
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6372,7 @@
       </c>
       <c r="E116" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -6393,7 +6393,7 @@
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -6414,7 +6414,7 @@
       </c>
       <c r="E118" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -6456,7 +6456,7 @@
       </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="E121" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="E124" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -6582,7 +6582,7 @@
       </c>
       <c r="E126" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -6666,7 +6666,7 @@
       </c>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -6687,7 +6687,7 @@
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -6729,7 +6729,7 @@
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -6750,7 +6750,7 @@
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -6792,7 +6792,7 @@
       </c>
       <c r="E136" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -6813,7 +6813,7 @@
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -6834,7 +6834,7 @@
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="E140" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -6897,7 +6897,7 @@
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -6918,7 +6918,7 @@
       </c>
       <c r="E142" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -6939,7 +6939,7 @@
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -6960,7 +6960,7 @@
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -6981,7 +6981,7 @@
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -7002,7 +7002,7 @@
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7023,7 @@
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -7044,7 +7044,7 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -7086,7 +7086,7 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -7107,7 +7107,7 @@
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -7128,7 +7128,7 @@
       </c>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7149,7 @@
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -7170,7 +7170,7 @@
       </c>
       <c r="E154" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -7229,7 +7229,7 @@
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="E158" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -7292,7 +7292,7 @@
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -7355,7 +7355,7 @@
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="E164" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -7397,7 +7397,7 @@
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7418,7 @@
       </c>
       <c r="E166" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7439,7 @@
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -7460,7 +7460,7 @@
       </c>
       <c r="E168" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -7481,7 +7481,7 @@
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -7502,7 +7502,7 @@
       </c>
       <c r="E170" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -7523,7 +7523,7 @@
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -7544,7 +7544,7 @@
       </c>
       <c r="E172" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>
@@ -7586,7 +7586,7 @@
       </c>
       <c r="E174" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:10</t>
+          <t xml:space="preserve">2026-09-14 20:23</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
prices: 2026-09-14 20:28 UTC
</commit_message>
<xml_diff>
--- a/docs/herblore_top8.xlsx
+++ b/docs/herblore_top8.xlsx
@@ -97,7 +97,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Last price update: 2026-09-14 20:23 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
+          <t xml:space="preserve">Last price update: 2026-09-14 20:28 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
         </is>
       </c>
     </row>
@@ -3978,7 +3978,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4062,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4146,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -4209,7 +4209,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -4377,7 +4377,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4608,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4713,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -4734,7 +4734,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -4902,7 +4902,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -4923,7 +4923,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -4965,7 +4965,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -5238,7 +5238,7 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5259,7 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -5322,7 +5322,7 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -5406,7 +5406,7 @@
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -5427,7 +5427,7 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5469,7 @@
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -5553,7 +5553,7 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -5574,7 +5574,7 @@
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -5595,7 +5595,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5637,7 @@
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5679,7 @@
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -5763,7 +5763,7 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -5931,7 +5931,7 @@
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -5952,7 +5952,7 @@
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -5973,7 +5973,7 @@
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -5994,7 +5994,7 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -6015,7 +6015,7 @@
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -6057,7 +6057,7 @@
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6120,7 @@
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6141,7 @@
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -6162,7 +6162,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -6225,7 +6225,7 @@
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -6246,7 +6246,7 @@
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6267,7 @@
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6288,7 @@
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6372,7 @@
       </c>
       <c r="E116" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -6393,7 +6393,7 @@
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -6414,7 +6414,7 @@
       </c>
       <c r="E118" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -6456,7 +6456,7 @@
       </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="E121" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="E124" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -6582,7 +6582,7 @@
       </c>
       <c r="E126" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -6666,7 +6666,7 @@
       </c>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -6687,7 +6687,7 @@
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -6729,7 +6729,7 @@
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -6750,7 +6750,7 @@
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -6792,7 +6792,7 @@
       </c>
       <c r="E136" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -6813,7 +6813,7 @@
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -6834,7 +6834,7 @@
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="E140" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -6897,7 +6897,7 @@
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -6918,7 +6918,7 @@
       </c>
       <c r="E142" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -6939,7 +6939,7 @@
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -6960,7 +6960,7 @@
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -6981,7 +6981,7 @@
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -7002,7 +7002,7 @@
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7023,7 @@
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -7044,7 +7044,7 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -7086,7 +7086,7 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -7107,7 +7107,7 @@
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -7128,7 +7128,7 @@
       </c>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7149,7 @@
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -7170,7 +7170,7 @@
       </c>
       <c r="E154" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -7229,7 +7229,7 @@
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="E158" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -7292,7 +7292,7 @@
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -7355,7 +7355,7 @@
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="E164" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -7397,7 +7397,7 @@
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7418,7 @@
       </c>
       <c r="E166" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7439,7 @@
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -7460,7 +7460,7 @@
       </c>
       <c r="E168" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -7481,7 +7481,7 @@
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -7502,7 +7502,7 @@
       </c>
       <c r="E170" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -7523,7 +7523,7 @@
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -7544,7 +7544,7 @@
       </c>
       <c r="E172" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>
@@ -7586,7 +7586,7 @@
       </c>
       <c r="E174" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:23</t>
+          <t xml:space="preserve">2026-09-14 20:28</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
prices: 2026-09-14 20:33 UTC
</commit_message>
<xml_diff>
--- a/docs/herblore_top8.xlsx
+++ b/docs/herblore_top8.xlsx
@@ -97,7 +97,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Last price update: 2026-09-14 20:28 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
+          <t xml:space="preserve">Last price update: 2026-09-14 20:33 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
         </is>
       </c>
     </row>
@@ -3978,7 +3978,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4062,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4146,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -4209,7 +4209,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -4377,7 +4377,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4608,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4713,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -4734,7 +4734,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -4902,7 +4902,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -4923,7 +4923,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -4965,7 +4965,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -5238,7 +5238,7 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5259,7 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -5322,7 +5322,7 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -5406,7 +5406,7 @@
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -5427,7 +5427,7 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5469,7 @@
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -5553,7 +5553,7 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -5574,7 +5574,7 @@
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -5595,7 +5595,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5637,7 @@
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5679,7 @@
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -5763,7 +5763,7 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -5931,7 +5931,7 @@
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -5952,7 +5952,7 @@
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -5973,7 +5973,7 @@
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -5994,7 +5994,7 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -6015,7 +6015,7 @@
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -6057,7 +6057,7 @@
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6120,7 @@
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6141,7 @@
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -6162,7 +6162,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -6225,7 +6225,7 @@
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -6246,7 +6246,7 @@
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6267,7 @@
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6288,7 @@
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6372,7 @@
       </c>
       <c r="E116" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -6393,7 +6393,7 @@
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -6414,7 +6414,7 @@
       </c>
       <c r="E118" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -6456,7 +6456,7 @@
       </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="E121" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="E124" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -6582,7 +6582,7 @@
       </c>
       <c r="E126" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -6666,7 +6666,7 @@
       </c>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -6687,7 +6687,7 @@
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -6729,7 +6729,7 @@
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -6750,7 +6750,7 @@
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -6792,7 +6792,7 @@
       </c>
       <c r="E136" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -6813,7 +6813,7 @@
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -6834,7 +6834,7 @@
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="E140" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -6897,7 +6897,7 @@
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -6918,7 +6918,7 @@
       </c>
       <c r="E142" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -6939,7 +6939,7 @@
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -6960,7 +6960,7 @@
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -6981,7 +6981,7 @@
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -7002,7 +7002,7 @@
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7023,7 @@
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -7044,7 +7044,7 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -7086,7 +7086,7 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -7107,7 +7107,7 @@
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -7128,7 +7128,7 @@
       </c>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7149,7 @@
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -7170,7 +7170,7 @@
       </c>
       <c r="E154" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -7229,7 +7229,7 @@
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="E158" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -7292,7 +7292,7 @@
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -7355,7 +7355,7 @@
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="E164" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -7397,7 +7397,7 @@
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7418,7 @@
       </c>
       <c r="E166" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7439,7 @@
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -7460,7 +7460,7 @@
       </c>
       <c r="E168" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -7481,7 +7481,7 @@
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -7502,7 +7502,7 @@
       </c>
       <c r="E170" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -7523,7 +7523,7 @@
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -7544,7 +7544,7 @@
       </c>
       <c r="E172" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>
@@ -7586,7 +7586,7 @@
       </c>
       <c r="E174" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:28</t>
+          <t xml:space="preserve">2026-09-14 20:33</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
prices: 2026-09-14 20:38 UTC
</commit_message>
<xml_diff>
--- a/docs/herblore_top8.xlsx
+++ b/docs/herblore_top8.xlsx
@@ -97,7 +97,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Last price update: 2026-09-14 20:33 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
+          <t xml:space="preserve">Last price update: 2026-09-14 20:38 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
         </is>
       </c>
     </row>
@@ -167,19 +167,19 @@
       </c>
       <c r="E4" s="2">
         <f>IF($G4="","",INDEX(Recipes!$L$2:$L$55,MATCH($G4,Recipes!$R$2:$R$55,0)))</f>
-        <v>59374</v>
+        <v>57078</v>
       </c>
       <c r="F4" s="2">
         <f>IF($G4="","",INDEX(Recipes!$M$2:$M$55,MATCH($G4,Recipes!$R$2:$R$55,0)))</f>
-        <v>68715</v>
+        <v>68159</v>
       </c>
       <c r="G4" s="2">
         <f>IFERROR(LARGE(Recipes!$R$2:$R$55,1),"")</f>
-        <v>941.7249999999985</v>
+        <v>2716.225000000006</v>
       </c>
       <c r="H4" s="2">
         <f>IF($G4="","",INDEX(Recipes!$Q$2:$Q$55,MATCH($G4,Recipes!$R$2:$R$55,0)))</f>
-        <v>2825174.999999996</v>
+        <v>8148675.000000018</v>
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
@@ -196,31 +196,31 @@
       </c>
       <c r="B5" s="0" t="str">
         <f>IF($G5="","",INDEX(Recipes!$A$2:$A$55,MATCH($G5,Recipes!$R$2:$R$55,0)))</f>
-        <v>Extended anti-venom+(4)</v>
+        <v>Goading potion(4)</v>
       </c>
       <c r="C5" s="2">
         <f>IF($G5="","",INDEX(Recipes!$B$2:$B$55,MATCH($G5,Recipes!$R$2:$R$55,0)))</f>
-        <v>94</v>
+        <v>54</v>
       </c>
       <c r="D5" s="4">
         <f>IF($G5="","",INDEX(Recipes!$C$2:$C$55,MATCH($G5,Recipes!$R$2:$R$55,0)))</f>
-        <v>80</v>
+        <v>132</v>
       </c>
       <c r="E5" s="2">
         <f>IF($G5="","",INDEX(Recipes!$L$2:$L$55,MATCH($G5,Recipes!$R$2:$R$55,0)))</f>
-        <v>14185.5</v>
+        <v>49560</v>
       </c>
       <c r="F5" s="2">
         <f>IF($G5="","",INDEX(Recipes!$M$2:$M$55,MATCH($G5,Recipes!$R$2:$R$55,0)))</f>
-        <v>18218</v>
+        <v>58337</v>
       </c>
       <c r="G5" s="2">
         <f>IFERROR(LARGE(Recipes!$R$2:$R$55,2),"")</f>
-        <v>867.1499999999996</v>
+        <v>2368.1500000000015</v>
       </c>
       <c r="H5" s="2">
         <f>IF($G5="","",INDEX(Recipes!$Q$2:$Q$55,MATCH($G5,Recipes!$R$2:$R$55,0)))</f>
-        <v>2601449.999999999</v>
+        <v>7104450.000000005</v>
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
@@ -272,31 +272,31 @@
       </c>
       <c r="B7" s="0" t="str">
         <f>IF($G7="","",INDEX(Recipes!$A$2:$A$55,MATCH($G7,Recipes!$R$2:$R$55,0)))</f>
-        <v>Goading potion(4)</v>
+        <v>Extended anti-venom+(4)</v>
       </c>
       <c r="C7" s="2">
         <f>IF($G7="","",INDEX(Recipes!$B$2:$B$55,MATCH($G7,Recipes!$R$2:$R$55,0)))</f>
-        <v>54</v>
+        <v>94</v>
       </c>
       <c r="D7" s="4">
         <f>IF($G7="","",INDEX(Recipes!$C$2:$C$55,MATCH($G7,Recipes!$R$2:$R$55,0)))</f>
-        <v>132</v>
+        <v>80</v>
       </c>
       <c r="E7" s="2">
         <f>IF($G7="","",INDEX(Recipes!$L$2:$L$55,MATCH($G7,Recipes!$R$2:$R$55,0)))</f>
-        <v>51856</v>
+        <v>14163.75</v>
       </c>
       <c r="F7" s="2">
         <f>IF($G7="","",INDEX(Recipes!$M$2:$M$55,MATCH($G7,Recipes!$R$2:$R$55,0)))</f>
-        <v>59655</v>
+        <v>18171</v>
       </c>
       <c r="G7" s="2">
         <f>IFERROR(LARGE(Recipes!$R$2:$R$55,4),"")</f>
-        <v>674.5</v>
+        <v>862.125</v>
       </c>
       <c r="H7" s="2">
         <f>IF($G7="","",INDEX(Recipes!$Q$2:$Q$55,MATCH($G7,Recipes!$R$2:$R$55,0)))</f>
-        <v>2023500</v>
+        <v>2586375</v>
       </c>
       <c r="I7" s="5"/>
       <c r="J7" s="2"/>
@@ -319,19 +319,19 @@
       </c>
       <c r="E8" s="2">
         <f>IF($G8="","",INDEX(Recipes!$L$2:$L$55,MATCH($G8,Recipes!$R$2:$R$55,0)))</f>
-        <v>11921</v>
+        <v>11896</v>
       </c>
       <c r="F8" s="2">
         <f>IF($G8="","",INDEX(Recipes!$M$2:$M$55,MATCH($G8,Recipes!$R$2:$R$55,0)))</f>
-        <v>12034</v>
+        <v>11968</v>
       </c>
       <c r="G8" s="2">
         <f>IFERROR(LARGE(Recipes!$R$2:$R$55,5),"")</f>
-        <v>482.7000000000007</v>
+        <v>445.7000000000007</v>
       </c>
       <c r="H8" s="2">
         <f>IF($G8="","",INDEX(Recipes!$Q$2:$Q$55,MATCH($G8,Recipes!$R$2:$R$55,0)))</f>
-        <v>1448100.000000002</v>
+        <v>1337100.000000002</v>
       </c>
       <c r="I8" s="5"/>
       <c r="J8" s="2"/>
@@ -354,19 +354,19 @@
       </c>
       <c r="E9" s="2">
         <f>IF($G9="","",INDEX(Recipes!$L$2:$L$55,MATCH($G9,Recipes!$R$2:$R$55,0)))</f>
-        <v>7126</v>
+        <v>7170</v>
       </c>
       <c r="F9" s="2">
         <f>IF($G9="","",INDEX(Recipes!$M$2:$M$55,MATCH($G9,Recipes!$R$2:$R$55,0)))</f>
-        <v>9351</v>
+        <v>9473</v>
       </c>
       <c r="G9" s="2">
         <f>IFERROR(LARGE(Recipes!$R$2:$R$55,6),"")</f>
-        <v>238.97500000000036</v>
+        <v>279.1749999999993</v>
       </c>
       <c r="H9" s="2">
         <f>IF($G9="","",INDEX(Recipes!$Q$2:$Q$55,MATCH($G9,Recipes!$R$2:$R$55,0)))</f>
-        <v>716925.000000001</v>
+        <v>837524.9999999978</v>
       </c>
       <c r="I9" s="5"/>
       <c r="J9" s="2"/>
@@ -377,31 +377,31 @@
       </c>
       <c r="B10" s="0" t="str">
         <f>IF($G10="","",INDEX(Recipes!$A$2:$A$55,MATCH($G10,Recipes!$R$2:$R$55,0)))</f>
-        <v>Guthix rest(4)</v>
+        <v>Guthix balance(4)</v>
       </c>
       <c r="C10" s="2">
         <f>IF($G10="","",INDEX(Recipes!$B$2:$B$55,MATCH($G10,Recipes!$R$2:$R$55,0)))</f>
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="D10" s="4">
         <f>IF($G10="","",INDEX(Recipes!$C$2:$C$55,MATCH($G10,Recipes!$R$2:$R$55,0)))</f>
-        <v>59</v>
+        <v>50</v>
       </c>
       <c r="E10" s="2">
         <f>IF($G10="","",INDEX(Recipes!$L$2:$L$55,MATCH($G10,Recipes!$R$2:$R$55,0)))</f>
-        <v>1915</v>
+        <v>826.75</v>
       </c>
       <c r="F10" s="2">
         <f>IF($G10="","",INDEX(Recipes!$M$2:$M$55,MATCH($G10,Recipes!$R$2:$R$55,0)))</f>
-        <v>2804</v>
+        <v>1124</v>
       </c>
       <c r="G10" s="2">
         <f>IFERROR(LARGE(Recipes!$R$2:$R$55,7),"")</f>
-        <v>160.5</v>
+        <v>110.55000000000007</v>
       </c>
       <c r="H10" s="2">
         <f>IF($G10="","",INDEX(Recipes!$Q$2:$Q$55,MATCH($G10,Recipes!$R$2:$R$55,0)))</f>
-        <v>963000</v>
+        <v>331650.00000000023</v>
       </c>
       <c r="I10" s="5"/>
       <c r="J10" s="2"/>
@@ -412,31 +412,31 @@
       </c>
       <c r="B11" s="0" t="str">
         <f>IF($G11="","",INDEX(Recipes!$A$2:$A$55,MATCH($G11,Recipes!$R$2:$R$55,0)))</f>
-        <v>Battlemage potion(4)</v>
+        <v>Guthix rest(4)</v>
       </c>
       <c r="C11" s="2">
         <f>IF($G11="","",INDEX(Recipes!$B$2:$B$55,MATCH($G11,Recipes!$R$2:$R$55,0)))</f>
-        <v>80</v>
+        <v>18</v>
       </c>
       <c r="D11" s="4">
         <f>IF($G11="","",INDEX(Recipes!$C$2:$C$55,MATCH($G11,Recipes!$R$2:$R$55,0)))</f>
-        <v>155</v>
+        <v>59</v>
       </c>
       <c r="E11" s="2">
         <f>IF($G11="","",INDEX(Recipes!$L$2:$L$55,MATCH($G11,Recipes!$R$2:$R$55,0)))</f>
-        <v>10848</v>
+        <v>1942</v>
       </c>
       <c r="F11" s="2">
         <f>IF($G11="","",INDEX(Recipes!$M$2:$M$55,MATCH($G11,Recipes!$R$2:$R$55,0)))</f>
-        <v>13198</v>
+        <v>2794</v>
       </c>
       <c r="G11" s="2">
         <f>IFERROR(LARGE(Recipes!$R$2:$R$55,8),"")</f>
-        <v>115.77499999999964</v>
+        <v>103.59999999999991</v>
       </c>
       <c r="H11" s="2">
         <f>IF($G11="","",INDEX(Recipes!$Q$2:$Q$55,MATCH($G11,Recipes!$R$2:$R$55,0)))</f>
-        <v>347324.9999999989</v>
+        <v>621599.9999999994</v>
       </c>
       <c r="I11" s="5"/>
       <c r="J11" s="2"/>
@@ -601,7 +601,7 @@
       <c r="K2" s="2"/>
       <c r="L2" s="2">
         <f>IFERROR((IF($D2="","",VLOOKUP($D2,Prices!$A$2:$D$174,3,0))*$E2)+(IF($F2="","",VLOOKUP($F2,Prices!$A$2:$D$174,3,0))*$G2),"")</f>
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="M2" s="2">
         <f>IFERROR(VLOOKUP($A2,Prices!$A$2:$D$174,4,0),"")</f>
@@ -613,19 +613,19 @@
       </c>
       <c r="O2" s="2">
         <f>IFERROR((IF($F2="","",VLOOKUP($F2,Prices!$A$2:$D$174,3,0))*$G2),"")</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P2" s="2">
         <f>IF(OR($L2="",$M2=""),"",(3+0.15*'Top 8'!$J$4)*($M2+$N2)/6-($L2-0.1*'Top 8'!$J$5*$O2))</f>
-        <v>-290.525</v>
+        <v>-289.625</v>
       </c>
       <c r="Q2" s="2">
         <f>IF($P2="","",$P2*3000)</f>
-        <v>-871574.9999999999</v>
+        <v>-868875</v>
       </c>
       <c r="R2" s="5">
         <f>IF($P2="","",$P2+ROW()/1000000)</f>
-        <v>-290.524997</v>
+        <v>-289.624997</v>
       </c>
     </row>
     <row r="3">
@@ -662,11 +662,11 @@
       <c r="K3" s="2"/>
       <c r="L3" s="2">
         <f>IFERROR((IF($D3="","",VLOOKUP($D3,Prices!$A$2:$D$174,3,0))*$E3)+(IF($F3="","",VLOOKUP($F3,Prices!$A$2:$D$174,3,0))*$G3),"")</f>
-        <v>933</v>
+        <v>938</v>
       </c>
       <c r="M3" s="2">
         <f>IFERROR(VLOOKUP($A3,Prices!$A$2:$D$174,4,0),"")</f>
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="N3" s="2">
         <f>IF(ISNUMBER(SEARCH("(4)",$A3)),IFERROR(VLOOKUP(SUBSTITUTE($A3,"(4)","(2)"),Prices!$A$2:$D$174,4,0),""),"")</f>
@@ -674,19 +674,19 @@
       </c>
       <c r="O3" s="2">
         <f>IFERROR((IF($F3="","",VLOOKUP($F3,Prices!$A$2:$D$174,3,0))*$G3),"")</f>
-        <v>694</v>
+        <v>699</v>
       </c>
       <c r="P3" s="2">
         <f>IF(OR($L3="",$M3=""),"",(3+0.15*'Top 8'!$J$4)*($M3+$N3)/6-($L3-0.1*'Top 8'!$J$5*$O3))</f>
-        <v>-507.65000000000003</v>
+        <v>-513.2</v>
       </c>
       <c r="Q3" s="2">
         <f>IF($P3="","",$P3*3000)</f>
-        <v>-1522950</v>
+        <v>-1539600.0000000002</v>
       </c>
       <c r="R3" s="5">
         <f>IF($P3="","",$P3+ROW()/1000000)</f>
-        <v>-507.64999600000004</v>
+        <v>-513.199996</v>
       </c>
     </row>
     <row r="4">
@@ -723,11 +723,11 @@
       <c r="K4" s="2"/>
       <c r="L4" s="2">
         <f>IFERROR((IF($D4="","",VLOOKUP($D4,Prices!$A$2:$D$174,3,0))*$E4)+(IF($F4="","",VLOOKUP($F4,Prices!$A$2:$D$174,3,0))*$G4),"")</f>
-        <v>708</v>
+        <v>705</v>
       </c>
       <c r="M4" s="2">
         <f>IFERROR(VLOOKUP($A4,Prices!$A$2:$D$174,4,0),"")</f>
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="N4" s="2">
         <f>IF(ISNUMBER(SEARCH("(4)",$A4)),IFERROR(VLOOKUP(SUBSTITUTE($A4,"(4)","(2)"),Prices!$A$2:$D$174,4,0),""),"")</f>
@@ -735,19 +735,19 @@
       </c>
       <c r="O4" s="2">
         <f>IFERROR((IF($F4="","",VLOOKUP($F4,Prices!$A$2:$D$174,3,0))*$G4),"")</f>
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="P4" s="2">
         <f>IF(OR($L4="",$M4=""),"",(3+0.15*'Top 8'!$J$4)*($M4+$N4)/6-($L4-0.1*'Top 8'!$J$5*$O4))</f>
-        <v>-606.85</v>
+        <v>-604.675</v>
       </c>
       <c r="Q4" s="2">
         <f>IF($P4="","",$P4*3000)</f>
-        <v>-1820550</v>
+        <v>-1814024.9999999998</v>
       </c>
       <c r="R4" s="5">
         <f>IF($P4="","",$P4+ROW()/1000000)</f>
-        <v>-606.849995</v>
+        <v>-604.674995</v>
       </c>
     </row>
     <row r="5">
@@ -784,7 +784,7 @@
       <c r="K5" s="2"/>
       <c r="L5" s="2">
         <f>IFERROR((IF($D5="","",VLOOKUP($D5,Prices!$A$2:$D$174,3,0))*$E5)+(IF($F5="","",VLOOKUP($F5,Prices!$A$2:$D$174,3,0))*$G5),"")</f>
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="M5" s="2">
         <f>IFERROR(VLOOKUP($A5,Prices!$A$2:$D$174,4,0),"")</f>
@@ -796,19 +796,19 @@
       </c>
       <c r="O5" s="2">
         <f>IFERROR((IF($F5="","",VLOOKUP($F5,Prices!$A$2:$D$174,3,0))*$G5),"")</f>
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="P5" s="2">
         <f>IF(OR($L5="",$M5=""),"",(3+0.15*'Top 8'!$J$4)*($M5+$N5)/6-($L5-0))</f>
-        <v>-495.425</v>
+        <v>-496.425</v>
       </c>
       <c r="Q5" s="2">
         <f>IF($P5="","",$P5*3000)</f>
-        <v>-1486275</v>
+        <v>-1489275</v>
       </c>
       <c r="R5" s="5">
         <f>IF($P5="","",$P5+ROW()/1000000)</f>
-        <v>-495.424994</v>
+        <v>-496.424994</v>
       </c>
     </row>
     <row r="6">
@@ -857,31 +857,31 @@
       </c>
       <c r="L6" s="2">
         <f>IFERROR((IF($D6="","",VLOOKUP($D6,Prices!$A$2:$D$174,3,0))*$E6)+(IF($F6="","",VLOOKUP($F6,Prices!$A$2:$D$174,3,0))*$G6)+(IF($H6="","",VLOOKUP($H6,Prices!$A$2:$D$174,3,0))*$I6)+(IF($J6="","",VLOOKUP($J6,Prices!$A$2:$D$174,3,0))*$K6),"")</f>
-        <v>1915</v>
+        <v>1942</v>
       </c>
       <c r="M6" s="2">
         <f>IFERROR(VLOOKUP($A6,Prices!$A$2:$D$174,4,0),"")</f>
-        <v>2804</v>
+        <v>2794</v>
       </c>
       <c r="N6" s="2">
         <f>IF(ISNUMBER(SEARCH("(4)",$A6)),IFERROR(VLOOKUP(SUBSTITUTE($A6,"(4)","(2)"),Prices!$A$2:$D$174,4,0),""),"")</f>
-        <v>1283</v>
+        <v>1231</v>
       </c>
       <c r="O6" s="2">
         <f>IFERROR((IF($J6="","",VLOOKUP($J6,Prices!$A$2:$D$174,3,0))*$K6),"")</f>
-        <v>320</v>
+        <v>331</v>
       </c>
       <c r="P6" s="2">
         <f>IF(OR($L6="",$M6=""),"",($M6+$N6)/2-($L6-0.1*'Top 8'!$J$5*$O6))</f>
-        <v>160.5</v>
+        <v>103.59999999999991</v>
       </c>
       <c r="Q6" s="2">
         <f>IF($P6="","",$P6*6000)</f>
-        <v>963000</v>
+        <v>621599.9999999994</v>
       </c>
       <c r="R6" s="5">
         <f>IF($P6="","",$P6+ROW()/1000000)</f>
-        <v>160.500007</v>
+        <v>103.6000069999999</v>
       </c>
     </row>
     <row r="7">
@@ -918,7 +918,7 @@
       <c r="K7" s="2"/>
       <c r="L7" s="2">
         <f>IFERROR((IF($D7="","",VLOOKUP($D7,Prices!$A$2:$D$174,3,0))*$E7)+(IF($F7="","",VLOOKUP($F7,Prices!$A$2:$D$174,3,0))*$G7),"")</f>
-        <v>700</v>
+        <v>707</v>
       </c>
       <c r="M7" s="2">
         <f>IFERROR(VLOOKUP($A7,Prices!$A$2:$D$174,4,0),"")</f>
@@ -930,19 +930,19 @@
       </c>
       <c r="O7" s="2">
         <f>IFERROR((IF($F7="","",VLOOKUP($F7,Prices!$A$2:$D$174,3,0))*$G7),"")</f>
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="P7" s="2">
         <f>IF(OR($L7="",$M7=""),"",(3+0.15*'Top 8'!$J$4)*($M7+$N7)/6-($L7-0.1*'Top 8'!$J$5*$O7))</f>
-        <v>-667.4000000000001</v>
+        <v>-673.7</v>
       </c>
       <c r="Q7" s="2">
         <f>IF($P7="","",$P7*3000)</f>
-        <v>-2002200.0000000002</v>
+        <v>-2021100.0000000002</v>
       </c>
       <c r="R7" s="5">
         <f>IF($P7="","",$P7+ROW()/1000000)</f>
-        <v>-667.3999920000001</v>
+        <v>-673.6999920000001</v>
       </c>
     </row>
     <row r="8">
@@ -979,11 +979,11 @@
       <c r="K8" s="2"/>
       <c r="L8" s="2">
         <f>IFERROR((IF($D8="","",VLOOKUP($D8,Prices!$A$2:$D$174,3,0))*$E8)+(IF($F8="","",VLOOKUP($F8,Prices!$A$2:$D$174,3,0))*$G8),"")</f>
-        <v>728</v>
+        <v>726</v>
       </c>
       <c r="M8" s="2">
         <f>IFERROR(VLOOKUP($A8,Prices!$A$2:$D$174,4,0),"")</f>
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="N8" s="2">
         <f>IF(ISNUMBER(SEARCH("(4)",$A8)),IFERROR(VLOOKUP(SUBSTITUTE($A8,"(4)","(2)"),Prices!$A$2:$D$174,4,0),""),"")</f>
@@ -991,19 +991,19 @@
       </c>
       <c r="O8" s="2">
         <f>IFERROR((IF($F8="","",VLOOKUP($F8,Prices!$A$2:$D$174,3,0))*$G8),"")</f>
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="P8" s="2">
         <f>IF(OR($L8="",$M8=""),"",(3+0.15*'Top 8'!$J$4)*($M8+$N8)/6-($L8-0.1*'Top 8'!$J$5*$O8))</f>
-        <v>-657.425</v>
+        <v>-655.1</v>
       </c>
       <c r="Q8" s="2">
         <f>IF($P8="","",$P8*3000)</f>
-        <v>-1972274.9999999998</v>
+        <v>-1965300</v>
       </c>
       <c r="R8" s="5">
         <f>IF($P8="","",$P8+ROW()/1000000)</f>
-        <v>-657.424991</v>
+        <v>-655.099991</v>
       </c>
     </row>
     <row r="9">
@@ -1046,11 +1046,11 @@
       <c r="K9" s="2"/>
       <c r="L9" s="2">
         <f>IFERROR((IF($D9="","",VLOOKUP($D9,Prices!$A$2:$D$174,3,0))*$E9)+(IF($F9="","",VLOOKUP($F9,Prices!$A$2:$D$174,3,0))*$G9)+(IF($H9="","",VLOOKUP($H9,Prices!$A$2:$D$174,3,0))*$I9)-0.25*((IF($D9="","",VLOOKUP($D9,Prices!$A$2:$D$174,3,0))*$E9)),"")</f>
-        <v>816</v>
+        <v>826.75</v>
       </c>
       <c r="M9" s="2">
         <f>IFERROR(VLOOKUP($A9,Prices!$A$2:$D$174,4,0),"")</f>
-        <v>1087</v>
+        <v>1124</v>
       </c>
       <c r="N9" s="2">
         <f>IF(ISNUMBER(SEARCH("(4)",$A9)),IFERROR(VLOOKUP(SUBSTITUTE($A9,"(4)","(2)"),Prices!$A$2:$D$174,4,0),""),"")</f>
@@ -1058,19 +1058,19 @@
       </c>
       <c r="O9" s="2">
         <f>IFERROR((IF($F9="","",VLOOKUP($F9,Prices!$A$2:$D$174,3,0))*$G9)+(IF($H9="","",VLOOKUP($H9,Prices!$A$2:$D$174,3,0))*$I9),"")</f>
-        <v>774</v>
+        <v>784</v>
       </c>
       <c r="P9" s="2">
         <f>IF(OR($L9="",$M9=""),"",(3+0.15*'Top 8'!$J$4)*($M9+$N9)/6-($L9-0.1*'Top 8'!$J$5*$O9))</f>
-        <v>100.875</v>
+        <v>110.55000000000007</v>
       </c>
       <c r="Q9" s="2">
         <f>IF($P9="","",$P9*3000)</f>
-        <v>302625</v>
+        <v>331650.00000000023</v>
       </c>
       <c r="R9" s="5">
         <f>IF($P9="","",$P9+ROW()/1000000)</f>
-        <v>100.87501</v>
+        <v>110.55001000000007</v>
       </c>
     </row>
     <row r="10">
@@ -1107,11 +1107,11 @@
       <c r="K10" s="2"/>
       <c r="L10" s="2">
         <f>IFERROR((IF($D10="","",VLOOKUP($D10,Prices!$A$2:$D$174,3,0))*$E10)+(IF($F10="","",VLOOKUP($F10,Prices!$A$2:$D$174,3,0))*$G10),"")</f>
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="M10" s="2">
         <f>IFERROR(VLOOKUP($A10,Prices!$A$2:$D$174,4,0),"")</f>
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="N10" s="2">
         <f>IF(ISNUMBER(SEARCH("(4)",$A10)),IFERROR(VLOOKUP(SUBSTITUTE($A10,"(4)","(2)"),Prices!$A$2:$D$174,4,0),""),"")</f>
@@ -1119,19 +1119,19 @@
       </c>
       <c r="O10" s="2">
         <f>IFERROR((IF($F10="","",VLOOKUP($F10,Prices!$A$2:$D$174,3,0))*$G10),"")</f>
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="P10" s="2">
         <f>IF(OR($L10="",$M10=""),"",(3+0.15*'Top 8'!$J$4)*($M10+$N10)/6-($L10-0.1*'Top 8'!$J$5*$O10))</f>
-        <v>-459.80000000000007</v>
+        <v>-458.525</v>
       </c>
       <c r="Q10" s="2">
         <f>IF($P10="","",$P10*3000)</f>
-        <v>-1379400.0000000002</v>
+        <v>-1375575</v>
       </c>
       <c r="R10" s="5">
         <f>IF($P10="","",$P10+ROW()/1000000)</f>
-        <v>-459.7999890000001</v>
+        <v>-458.524989</v>
       </c>
     </row>
     <row r="11">
@@ -1168,31 +1168,31 @@
       <c r="K11" s="2"/>
       <c r="L11" s="2">
         <f>IFERROR((IF($D11="","",VLOOKUP($D11,Prices!$A$2:$D$174,3,0))*$E11)+(IF($F11="","",VLOOKUP($F11,Prices!$A$2:$D$174,3,0))*$G11),"")</f>
-        <v>6854</v>
+        <v>6848</v>
       </c>
       <c r="M11" s="2">
         <f>IFERROR(VLOOKUP($A11,Prices!$A$2:$D$174,4,0),"")</f>
-        <v>552</v>
+        <v>571</v>
       </c>
       <c r="N11" s="2">
         <f>IF(ISNUMBER(SEARCH("(4)",$A11)),IFERROR(VLOOKUP(SUBSTITUTE($A11,"(4)","(2)"),Prices!$A$2:$D$174,4,0),""),"")</f>
-        <v>350</v>
+        <v>336</v>
       </c>
       <c r="O11" s="2">
         <f>IFERROR((IF($F11="","",VLOOKUP($F11,Prices!$A$2:$D$174,3,0))*$G11),"")</f>
-        <v>681</v>
+        <v>675</v>
       </c>
       <c r="P11" s="2">
         <f>IF(OR($L11="",$M11=""),"",(3+0.15*'Top 8'!$J$4)*($M11+$N11)/6-($L11-0.1*'Top 8'!$J$5*$O11))</f>
-        <v>-6312.349999999999</v>
+        <v>-6304.325</v>
       </c>
       <c r="Q11" s="2">
         <f>IF($P11="","",$P11*3000)</f>
-        <v>-18937050</v>
+        <v>-18912975</v>
       </c>
       <c r="R11" s="5">
         <f>IF($P11="","",$P11+ROW()/1000000)</f>
-        <v>-6312.349987999999</v>
+        <v>-6304.324987999999</v>
       </c>
     </row>
     <row r="12">
@@ -1229,11 +1229,11 @@
       <c r="K12" s="2"/>
       <c r="L12" s="2">
         <f>IFERROR((IF($D12="","",VLOOKUP($D12,Prices!$A$2:$D$174,3,0))*$E12)+(IF($F12="","",VLOOKUP($F12,Prices!$A$2:$D$174,3,0))*$G12),"")</f>
-        <v>2915</v>
+        <v>2917</v>
       </c>
       <c r="M12" s="2">
         <f>IFERROR(VLOOKUP($A12,Prices!$A$2:$D$174,4,0),"")</f>
-        <v>334</v>
+        <v>350</v>
       </c>
       <c r="N12" s="2">
         <f>IF(ISNUMBER(SEARCH("(4)",$A12)),IFERROR(VLOOKUP(SUBSTITUTE($A12,"(4)","(2)"),Prices!$A$2:$D$174,4,0),""),"")</f>
@@ -1241,19 +1241,19 @@
       </c>
       <c r="O12" s="2">
         <f>IFERROR((IF($F12="","",VLOOKUP($F12,Prices!$A$2:$D$174,3,0))*$G12),"")</f>
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="P12" s="2">
         <f>IF(OR($L12="",$M12=""),"",(3+0.15*'Top 8'!$J$4)*($M12+$N12)/6-($L12-0.1*'Top 8'!$J$5*$O12))</f>
-        <v>-2599</v>
+        <v>-2592.4</v>
       </c>
       <c r="Q12" s="2">
         <f>IF($P12="","",$P12*3000)</f>
-        <v>-7797000</v>
+        <v>-7777200</v>
       </c>
       <c r="R12" s="5">
         <f>IF($P12="","",$P12+ROW()/1000000)</f>
-        <v>-2598.999987</v>
+        <v>-2592.3999870000002</v>
       </c>
     </row>
     <row r="13">
@@ -1290,7 +1290,7 @@
       <c r="K13" s="2"/>
       <c r="L13" s="2">
         <f>IFERROR((IF($D13="","",VLOOKUP($D13,Prices!$A$2:$D$174,3,0))*$E13)+(IF($F13="","",VLOOKUP($F13,Prices!$A$2:$D$174,3,0))*$G13),"")</f>
-        <v>676</v>
+        <v>672</v>
       </c>
       <c r="M13" s="2">
         <f>IFERROR(VLOOKUP($A13,Prices!$A$2:$D$174,4,0),"")</f>
@@ -1298,23 +1298,23 @@
       </c>
       <c r="N13" s="2">
         <f>IF(ISNUMBER(SEARCH("(4)",$A13)),IFERROR(VLOOKUP(SUBSTITUTE($A13,"(4)","(2)"),Prices!$A$2:$D$174,4,0),""),"")</f>
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="O13" s="2">
         <f>IFERROR((IF($F13="","",VLOOKUP($F13,Prices!$A$2:$D$174,3,0))*$G13),"")</f>
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="P13" s="2">
         <f>IF(OR($L13="",$M13=""),"",(3+0.15*'Top 8'!$J$4)*($M13+$N13)/6-($L13-0.1*'Top 8'!$J$5*$O13))</f>
-        <v>-495.125</v>
+        <v>-494.15</v>
       </c>
       <c r="Q13" s="2">
         <f>IF($P13="","",$P13*3000)</f>
-        <v>-1485375</v>
+        <v>-1482450</v>
       </c>
       <c r="R13" s="5">
         <f>IF($P13="","",$P13+ROW()/1000000)</f>
-        <v>-495.124986</v>
+        <v>-494.14998599999996</v>
       </c>
     </row>
     <row r="14">
@@ -1351,31 +1351,31 @@
       <c r="K14" s="2"/>
       <c r="L14" s="2">
         <f>IFERROR((IF($D14="","",VLOOKUP($D14,Prices!$A$2:$D$174,3,0))*$E14)+(IF($F14="","",VLOOKUP($F14,Prices!$A$2:$D$174,3,0))*$G14),"")</f>
-        <v>7126</v>
+        <v>7170</v>
       </c>
       <c r="M14" s="2">
         <f>IFERROR(VLOOKUP($A14,Prices!$A$2:$D$174,4,0),"")</f>
-        <v>9351</v>
+        <v>9473</v>
       </c>
       <c r="N14" s="2">
         <f>IF(ISNUMBER(SEARCH("(4)",$A14)),IFERROR(VLOOKUP(SUBSTITUTE($A14,"(4)","(2)"),Prices!$A$2:$D$174,4,0),""),"")</f>
-        <v>4496</v>
+        <v>4526</v>
       </c>
       <c r="O14" s="2">
         <f>IFERROR((IF($F14="","",VLOOKUP($F14,Prices!$A$2:$D$174,3,0))*$G14),"")</f>
-        <v>953</v>
+        <v>997</v>
       </c>
       <c r="P14" s="2">
         <f>IF(OR($L14="",$M14=""),"",(3+0.15*'Top 8'!$J$4)*($M14+$N14)/6-($L14-0.1*'Top 8'!$J$5*$O14))</f>
-        <v>238.97500000000036</v>
+        <v>279.1749999999993</v>
       </c>
       <c r="Q14" s="2">
         <f>IF($P14="","",$P14*3000)</f>
-        <v>716925.000000001</v>
+        <v>837524.9999999978</v>
       </c>
       <c r="R14" s="5">
         <f>IF($P14="","",$P14+ROW()/1000000)</f>
-        <v>238.97501500000035</v>
+        <v>279.1750149999993</v>
       </c>
     </row>
     <row r="15">
@@ -1412,11 +1412,11 @@
       <c r="K15" s="2"/>
       <c r="L15" s="2">
         <f>IFERROR((IF($D15="","",VLOOKUP($D15,Prices!$A$2:$D$174,3,0))*$E15)+(IF($F15="","",VLOOKUP($F15,Prices!$A$2:$D$174,3,0))*$G15),"")</f>
-        <v>1736</v>
+        <v>1735</v>
       </c>
       <c r="M15" s="2">
         <f>IFERROR(VLOOKUP($A15,Prices!$A$2:$D$174,4,0),"")</f>
-        <v>1906</v>
+        <v>1885</v>
       </c>
       <c r="N15" s="2">
         <f>IF(ISNUMBER(SEARCH("(4)",$A15)),IFERROR(VLOOKUP(SUBSTITUTE($A15,"(4)","(2)"),Prices!$A$2:$D$174,4,0),""),"")</f>
@@ -1424,19 +1424,19 @@
       </c>
       <c r="O15" s="2">
         <f>IFERROR((IF($F15="","",VLOOKUP($F15,Prices!$A$2:$D$174,3,0))*$G15),"")</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P15" s="2">
         <f>IF(OR($L15="",$M15=""),"",(3+0.15*'Top 8'!$J$4)*($M15+$N15)/6-($L15-0.1*'Top 8'!$J$5*$O15))</f>
-        <v>-259.20000000000005</v>
+        <v>-269.3249999999998</v>
       </c>
       <c r="Q15" s="2">
         <f>IF($P15="","",$P15*3000)</f>
-        <v>-777600.0000000001</v>
+        <v>-807974.9999999994</v>
       </c>
       <c r="R15" s="5">
         <f>IF($P15="","",$P15+ROW()/1000000)</f>
-        <v>-259.19998400000003</v>
+        <v>-269.3249839999998</v>
       </c>
     </row>
     <row r="16">
@@ -1473,11 +1473,11 @@
       <c r="K16" s="2"/>
       <c r="L16" s="2">
         <f>IFERROR((IF($D16="","",VLOOKUP($D16,Prices!$A$2:$D$174,3,0))*$E16)+(IF($F16="","",VLOOKUP($F16,Prices!$A$2:$D$174,3,0))*$G16),"")</f>
-        <v>2425</v>
+        <v>2430</v>
       </c>
       <c r="M16" s="2">
         <f>IFERROR(VLOOKUP($A16,Prices!$A$2:$D$174,4,0),"")</f>
-        <v>1368</v>
+        <v>1352</v>
       </c>
       <c r="N16" s="2">
         <f>IF(ISNUMBER(SEARCH("(4)",$A16)),IFERROR(VLOOKUP(SUBSTITUTE($A16,"(4)","(2)"),Prices!$A$2:$D$174,4,0),""),"")</f>
@@ -1485,19 +1485,19 @@
       </c>
       <c r="O16" s="2">
         <f>IFERROR((IF($F16="","",VLOOKUP($F16,Prices!$A$2:$D$174,3,0))*$G16),"")</f>
-        <v>694</v>
+        <v>699</v>
       </c>
       <c r="P16" s="2">
         <f>IF(OR($L16="",$M16=""),"",(3+0.15*'Top 8'!$J$4)*($M16+$N16)/6-($L16-0.1*'Top 8'!$J$5*$O16))</f>
-        <v>-1283.55</v>
+        <v>-1296.4499999999998</v>
       </c>
       <c r="Q16" s="2">
         <f>IF($P16="","",$P16*3000)</f>
-        <v>-3850650</v>
+        <v>-3889349.9999999995</v>
       </c>
       <c r="R16" s="5">
         <f>IF($P16="","",$P16+ROW()/1000000)</f>
-        <v>-1283.5499829999999</v>
+        <v>-1296.4499829999997</v>
       </c>
     </row>
     <row r="17">
@@ -1534,7 +1534,7 @@
       <c r="K17" s="2"/>
       <c r="L17" s="2">
         <f>IFERROR((IF($D17="","",VLOOKUP($D17,Prices!$A$2:$D$174,3,0))*$E17)+(IF($F17="","",VLOOKUP($F17,Prices!$A$2:$D$174,3,0))*$G17),"")</f>
-        <v>3420</v>
+        <v>3464</v>
       </c>
       <c r="M17" s="2">
         <f>IFERROR(VLOOKUP($A17,Prices!$A$2:$D$174,4,0),"")</f>
@@ -1546,19 +1546,19 @@
       </c>
       <c r="O17" s="2">
         <f>IFERROR((IF($F17="","",VLOOKUP($F17,Prices!$A$2:$D$174,3,0))*$G17),"")</f>
-        <v>953</v>
+        <v>997</v>
       </c>
       <c r="P17" s="2">
         <f>IF(OR($L17="",$M17=""),"",(3+0.15*'Top 8'!$J$4)*($M17+$N17)/6-($L17-0.1*'Top 8'!$J$5*$O17))</f>
-        <v>-3241.75</v>
+        <v>-3281.3500000000004</v>
       </c>
       <c r="Q17" s="2">
         <f>IF($P17="","",$P17*3000)</f>
-        <v>-9725250</v>
+        <v>-9844050.000000002</v>
       </c>
       <c r="R17" s="5">
         <f>IF($P17="","",$P17+ROW()/1000000)</f>
-        <v>-3241.749982</v>
+        <v>-3281.349982</v>
       </c>
     </row>
     <row r="18">
@@ -1595,11 +1595,11 @@
       <c r="K18" s="2"/>
       <c r="L18" s="2">
         <f>IFERROR((IF($D18="","",VLOOKUP($D18,Prices!$A$2:$D$174,3,0))*$E18)+(IF($F18="","",VLOOKUP($F18,Prices!$A$2:$D$174,3,0))*$G18),"")</f>
-        <v>2694</v>
+        <v>2687</v>
       </c>
       <c r="M18" s="2">
         <f>IFERROR(VLOOKUP($A18,Prices!$A$2:$D$174,4,0),"")</f>
-        <v>2499</v>
+        <v>2566</v>
       </c>
       <c r="N18" s="2">
         <f>IF(ISNUMBER(SEARCH("(4)",$A18)),IFERROR(VLOOKUP(SUBSTITUTE($A18,"(4)","(2)"),Prices!$A$2:$D$174,4,0),""),"")</f>
@@ -1607,19 +1607,19 @@
       </c>
       <c r="O18" s="2">
         <f>IFERROR((IF($F18="","",VLOOKUP($F18,Prices!$A$2:$D$174,3,0))*$G18),"")</f>
-        <v>227</v>
+        <v>220</v>
       </c>
       <c r="P18" s="2">
         <f>IF(OR($L18="",$M18=""),"",(3+0.15*'Top 8'!$J$4)*($M18+$N18)/6-($L18-0.1*'Top 8'!$J$5*$O18))</f>
-        <v>-454.75000000000045</v>
+        <v>-413.2750000000001</v>
       </c>
       <c r="Q18" s="2">
         <f>IF($P18="","",$P18*3000)</f>
-        <v>-1364250.0000000014</v>
+        <v>-1239825.0000000002</v>
       </c>
       <c r="R18" s="5">
         <f>IF($P18="","",$P18+ROW()/1000000)</f>
-        <v>-454.74998100000045</v>
+        <v>-413.2749810000001</v>
       </c>
     </row>
     <row r="19">
@@ -1656,11 +1656,11 @@
       <c r="K19" s="2"/>
       <c r="L19" s="2">
         <f>IFERROR((IF($D19="","",VLOOKUP($D19,Prices!$A$2:$D$174,3,0))*$E19)+(IF($F19="","",VLOOKUP($F19,Prices!$A$2:$D$174,3,0))*$G19),"")</f>
-        <v>3251</v>
+        <v>3232</v>
       </c>
       <c r="M19" s="2">
         <f>IFERROR(VLOOKUP($A19,Prices!$A$2:$D$174,4,0),"")</f>
-        <v>547</v>
+        <v>560</v>
       </c>
       <c r="N19" s="2">
         <f>IF(ISNUMBER(SEARCH("(4)",$A19)),IFERROR(VLOOKUP(SUBSTITUTE($A19,"(4)","(2)"),Prices!$A$2:$D$174,4,0),""),"")</f>
@@ -1668,19 +1668,19 @@
       </c>
       <c r="O19" s="2">
         <f>IFERROR((IF($F19="","",VLOOKUP($F19,Prices!$A$2:$D$174,3,0))*$G19),"")</f>
-        <v>784</v>
+        <v>765</v>
       </c>
       <c r="P19" s="2">
         <f>IF(OR($L19="",$M19=""),"",(3+0.15*'Top 8'!$J$4)*($M19+$N19)/6-($L19-0.1*'Top 8'!$J$5*$O19))</f>
-        <v>-2279.575</v>
+        <v>-2255.65</v>
       </c>
       <c r="Q19" s="2">
         <f>IF($P19="","",$P19*3000)</f>
-        <v>-6838724.999999999</v>
+        <v>-6766950</v>
       </c>
       <c r="R19" s="5">
         <f>IF($P19="","",$P19+ROW()/1000000)</f>
-        <v>-2279.57498</v>
+        <v>-2255.64998</v>
       </c>
     </row>
     <row r="20">
@@ -1717,31 +1717,31 @@
       <c r="K20" s="2"/>
       <c r="L20" s="2">
         <f>IFERROR((IF($D20="","",VLOOKUP($D20,Prices!$A$2:$D$174,3,0))*$E20)+(IF($F20="","",VLOOKUP($F20,Prices!$A$2:$D$174,3,0))*$G20),"")</f>
-        <v>51856</v>
+        <v>49560</v>
       </c>
       <c r="M20" s="2">
         <f>IFERROR(VLOOKUP($A20,Prices!$A$2:$D$174,4,0),"")</f>
-        <v>59655</v>
+        <v>58337</v>
       </c>
       <c r="N20" s="2">
         <f>IF(ISNUMBER(SEARCH("(4)",$A20)),IFERROR(VLOOKUP(SUBSTITUTE($A20,"(4)","(2)"),Prices!$A$2:$D$174,4,0),""),"")</f>
-        <v>30629</v>
+        <v>31237</v>
       </c>
       <c r="O20" s="2">
         <f>IFERROR((IF($F20="","",VLOOKUP($F20,Prices!$A$2:$D$174,3,0))*$G20),"")</f>
-        <v>51314</v>
+        <v>49018</v>
       </c>
       <c r="P20" s="2">
         <f>IF(OR($L20="",$M20=""),"",(3+0.15*'Top 8'!$J$4)*($M20+$N20)/6-($L20-0.1*'Top 8'!$J$5*$O20))</f>
-        <v>674.5</v>
+        <v>2368.1500000000015</v>
       </c>
       <c r="Q20" s="2">
         <f>IF($P20="","",$P20*3000)</f>
-        <v>2023500</v>
+        <v>7104450.000000005</v>
       </c>
       <c r="R20" s="5">
         <f>IF($P20="","",$P20+ROW()/1000000)</f>
-        <v>674.500021</v>
+        <v>2368.1500210000013</v>
       </c>
     </row>
     <row r="21">
@@ -1778,11 +1778,11 @@
       <c r="K21" s="2"/>
       <c r="L21" s="2">
         <f>IFERROR((IF($D21="","",VLOOKUP($D21,Prices!$A$2:$D$174,3,0))*$E21)+(IF($F21="","",VLOOKUP($F21,Prices!$A$2:$D$174,3,0))*$G21),"")</f>
-        <v>2834</v>
+        <v>2831</v>
       </c>
       <c r="M21" s="2">
         <f>IFERROR(VLOOKUP($A21,Prices!$A$2:$D$174,4,0),"")</f>
-        <v>2990</v>
+        <v>3039</v>
       </c>
       <c r="N21" s="2">
         <f>IF(ISNUMBER(SEARCH("(4)",$A21)),IFERROR(VLOOKUP(SUBSTITUTE($A21,"(4)","(2)"),Prices!$A$2:$D$174,4,0),""),"")</f>
@@ -1790,19 +1790,19 @@
       </c>
       <c r="O21" s="2">
         <f>IFERROR((IF($F21="","",VLOOKUP($F21,Prices!$A$2:$D$174,3,0))*$G21),"")</f>
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="P21" s="2">
         <f>IF(OR($L21="",$M21=""),"",(3+0.15*'Top 8'!$J$4)*($M21+$N21)/6-($L21-0.1*'Top 8'!$J$5*$O21))</f>
-        <v>-480.0750000000003</v>
+        <v>-451.6500000000001</v>
       </c>
       <c r="Q21" s="2">
         <f>IF($P21="","",$P21*3000)</f>
-        <v>-1440225.000000001</v>
+        <v>-1354950.0000000002</v>
       </c>
       <c r="R21" s="5">
         <f>IF($P21="","",$P21+ROW()/1000000)</f>
-        <v>-480.07497800000027</v>
+        <v>-451.6499780000001</v>
       </c>
     </row>
     <row r="22">
@@ -1960,11 +1960,11 @@
       <c r="K24" s="2"/>
       <c r="L24" s="2">
         <f>IFERROR((IF($D24="","",VLOOKUP($D24,Prices!$A$2:$D$174,3,0))*$E24)+(IF($F24="","",VLOOKUP($F24,Prices!$A$2:$D$174,3,0))*$G24),"")</f>
-        <v>59374</v>
+        <v>57078</v>
       </c>
       <c r="M24" s="2">
         <f>IFERROR(VLOOKUP($A24,Prices!$A$2:$D$174,4,0),"")</f>
-        <v>68715</v>
+        <v>68159</v>
       </c>
       <c r="N24" s="2">
         <f>IF(ISNUMBER(SEARCH("(4)",$A24)),IFERROR(VLOOKUP(SUBSTITUTE($A24,"(4)","(2)"),Prices!$A$2:$D$174,4,0),""),"")</f>
@@ -1972,19 +1972,19 @@
       </c>
       <c r="O24" s="2">
         <f>IFERROR((IF($F24="","",VLOOKUP($F24,Prices!$A$2:$D$174,3,0))*$G24),"")</f>
-        <v>51314</v>
+        <v>49018</v>
       </c>
       <c r="P24" s="2">
         <f>IF(OR($L24="",$M24=""),"",(3+0.15*'Top 8'!$J$4)*($M24+$N24)/6-($L24-0.1*'Top 8'!$J$5*$O24))</f>
-        <v>941.7249999999985</v>
+        <v>2716.225000000006</v>
       </c>
       <c r="Q24" s="2">
         <f>IF($P24="","",$P24*3000)</f>
-        <v>2825174.999999996</v>
+        <v>8148675.000000018</v>
       </c>
       <c r="R24" s="5">
         <f>IF($P24="","",$P24+ROW()/1000000)</f>
-        <v>941.7250249999986</v>
+        <v>2716.2250250000056</v>
       </c>
     </row>
     <row r="25">
@@ -2021,30 +2021,30 @@
       <c r="K25" s="2"/>
       <c r="L25" s="2">
         <f>IFERROR((IF($D25="","",VLOOKUP($D25,Prices!$A$2:$D$174,3,0))*$E25)+(IF($F25="","",VLOOKUP($F25,Prices!$A$2:$D$174,3,0))*$G25),"")</f>
-        <v>2681</v>
+        <v>2680</v>
       </c>
       <c r="M25" s="2">
         <f>IFERROR(VLOOKUP($A25,Prices!$A$2:$D$174,4,0),"")</f>
-        <v>286</v>
+        <v>280</v>
       </c>
       <c r="N25" s="2">
         <f>IF(ISNUMBER(SEARCH("(4)",$A25)),IFERROR(VLOOKUP(SUBSTITUTE($A25,"(4)","(2)"),Prices!$A$2:$D$174,4,0),""),"")</f>
       </c>
       <c r="O25" s="2">
         <f>IFERROR((IF($F25="","",VLOOKUP($F25,Prices!$A$2:$D$174,3,0))*$G25),"")</f>
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="P25" s="2">
         <f>IF(OR($L25="",$M25=""),"",$M25-($L25-0.1*'Top 8'!$J$5*$O25))</f>
-        <v>-2387.9</v>
+        <v>-2393</v>
       </c>
       <c r="Q25" s="2">
         <f>IF($P25="","",$P25*3000)</f>
-        <v>-7163700</v>
+        <v>-7179000</v>
       </c>
       <c r="R25" s="5">
         <f>IF($P25="","",$P25+ROW()/1000000)</f>
-        <v>-2387.899974</v>
+        <v>-2392.999974</v>
       </c>
     </row>
     <row r="26">
@@ -2085,7 +2085,7 @@
       </c>
       <c r="M26" s="2">
         <f>IFERROR(VLOOKUP($A26,Prices!$A$2:$D$174,4,0),"")</f>
-        <v>1785</v>
+        <v>1875</v>
       </c>
       <c r="N26" s="2">
         <f>IF(ISNUMBER(SEARCH("(4)",$A26)),IFERROR(VLOOKUP(SUBSTITUTE($A26,"(4)","(2)"),Prices!$A$2:$D$174,4,0),""),"")</f>
@@ -2097,15 +2097,15 @@
       </c>
       <c r="P26" s="2">
         <f>IF(OR($L26="",$M26=""),"",(3+0.15*'Top 8'!$J$4)*($M26+$N26)/6-($L26-0.1*'Top 8'!$J$5*$O26))</f>
-        <v>-677.575</v>
+        <v>-630.3250000000003</v>
       </c>
       <c r="Q26" s="2">
         <f>IF($P26="","",$P26*3000)</f>
-        <v>-2032725.0000000002</v>
+        <v>-1890975.000000001</v>
       </c>
       <c r="R26" s="5">
         <f>IF($P26="","",$P26+ROW()/1000000)</f>
-        <v>-677.574973</v>
+        <v>-630.3249730000002</v>
       </c>
     </row>
     <row r="27">
@@ -2142,11 +2142,11 @@
       <c r="K27" s="2"/>
       <c r="L27" s="2">
         <f>IFERROR((IF($D27="","",VLOOKUP($D27,Prices!$A$2:$D$174,3,0))*$E27)+(IF($F27="","",VLOOKUP($F27,Prices!$A$2:$D$174,3,0))*$G27),"")</f>
-        <v>8086</v>
+        <v>8084</v>
       </c>
       <c r="M27" s="2">
         <f>IFERROR(VLOOKUP($A27,Prices!$A$2:$D$174,4,0),"")</f>
-        <v>9811</v>
+        <v>9810</v>
       </c>
       <c r="N27" s="2">
         <f>IF(ISNUMBER(SEARCH("(4)",$A27)),IFERROR(VLOOKUP(SUBSTITUTE($A27,"(4)","(2)"),Prices!$A$2:$D$174,4,0),""),"")</f>
@@ -2154,19 +2154,19 @@
       </c>
       <c r="O27" s="2">
         <f>IFERROR((IF($F27="","",VLOOKUP($F27,Prices!$A$2:$D$174,3,0))*$G27),"")</f>
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="P27" s="2">
         <f>IF(OR($L27="",$M27=""),"",(3+0.15*'Top 8'!$J$4)*($M27+$N27)/6-($L27-0.1*'Top 8'!$J$5*$O27))</f>
-        <v>-402.39999999999964</v>
+        <v>-401.1250000000009</v>
       </c>
       <c r="Q27" s="2">
         <f>IF($P27="","",$P27*3000)</f>
-        <v>-1207199.9999999988</v>
+        <v>-1203375.0000000028</v>
       </c>
       <c r="R27" s="5">
         <f>IF($P27="","",$P27+ROW()/1000000)</f>
-        <v>-402.39997199999965</v>
+        <v>-401.1249720000009</v>
       </c>
     </row>
     <row r="28">
@@ -2218,11 +2218,11 @@
       </c>
       <c r="M28" s="2">
         <f>IFERROR(VLOOKUP($A28,Prices!$A$2:$D$174,4,0),"")</f>
-        <v>18910</v>
+        <v>19090</v>
       </c>
       <c r="N28" s="2">
         <f>IF(ISNUMBER(SEARCH("(4)",$A28)),IFERROR(VLOOKUP(SUBSTITUTE($A28,"(4)","(2)"),Prices!$A$2:$D$174,4,0),""),"")</f>
-        <v>8259</v>
+        <v>8335</v>
       </c>
       <c r="O28" s="2">
         <f>IFERROR((IF($F28="","",VLOOKUP($F28,Prices!$A$2:$D$174,3,0))*$G28)+(IF($H28="","",VLOOKUP($H28,Prices!$A$2:$D$174,3,0))*$I28)+(IF($J28="","",VLOOKUP($J28,Prices!$A$2:$D$174,3,0))*$K28),"")</f>
@@ -2271,11 +2271,11 @@
       <c r="K29" s="2"/>
       <c r="L29" s="2">
         <f>IFERROR(0.75*((IF($D29="","",VLOOKUP($D29,Prices!$A$2:$D$174,3,0))*$E29)+(IF($F29="","",VLOOKUP($F29,Prices!$A$2:$D$174,3,0))*$G29)),"")</f>
-        <v>2472.75</v>
+        <v>2524.5</v>
       </c>
       <c r="M29" s="2">
         <f>IFERROR(VLOOKUP($A29,Prices!$A$2:$D$174,4,0),"")</f>
-        <v>2180</v>
+        <v>2250</v>
       </c>
       <c r="N29" s="2">
         <f>IF(ISNUMBER(SEARCH("(4)",$A29)),IFERROR(VLOOKUP(SUBSTITUTE($A29,"(4)","(2)"),Prices!$A$2:$D$174,4,0),""),"")</f>
@@ -2287,15 +2287,15 @@
       </c>
       <c r="P29" s="2">
         <f>IF(OR($L29="",$M29=""),"",(3+0.15*'Top 8'!$J$4)*($M29+$N29)/6-($L29-0.1*'Top 8'!$J$5*$O29))</f>
-        <v>-48.375</v>
+        <v>-63.375</v>
       </c>
       <c r="Q29" s="2">
         <f>IF($P29="","",$P29*3000)</f>
-        <v>-145125</v>
+        <v>-190125</v>
       </c>
       <c r="R29" s="5">
         <f>IF($P29="","",$P29+ROW()/1000000)</f>
-        <v>-48.37497</v>
+        <v>-63.37497</v>
       </c>
     </row>
     <row r="30">
@@ -2332,11 +2332,11 @@
       <c r="K30" s="2"/>
       <c r="L30" s="2">
         <f>IFERROR((IF($D30="","",VLOOKUP($D30,Prices!$A$2:$D$174,3,0))*$E30)+(IF($F30="","",VLOOKUP($F30,Prices!$A$2:$D$174,3,0))*$G30),"")</f>
-        <v>3251</v>
+        <v>3245</v>
       </c>
       <c r="M30" s="2">
         <f>IFERROR(VLOOKUP($A30,Prices!$A$2:$D$174,4,0),"")</f>
-        <v>3165</v>
+        <v>3073</v>
       </c>
       <c r="N30" s="2">
         <f>IF(ISNUMBER(SEARCH("(4)",$A30)),IFERROR(VLOOKUP(SUBSTITUTE($A30,"(4)","(2)"),Prices!$A$2:$D$174,4,0),""),"")</f>
@@ -2344,19 +2344,19 @@
       </c>
       <c r="O30" s="2">
         <f>IFERROR((IF($F30="","",VLOOKUP($F30,Prices!$A$2:$D$174,3,0))*$G30),"")</f>
-        <v>681</v>
+        <v>675</v>
       </c>
       <c r="P30" s="2">
         <f>IF(OR($L30="",$M30=""),"",(3+0.15*'Top 8'!$J$4)*($M30+$N30)/6-($L30-0.1*'Top 8'!$J$5*$O30))</f>
-        <v>-714.3500000000004</v>
+        <v>-757.25</v>
       </c>
       <c r="Q30" s="2">
         <f>IF($P30="","",$P30*3000)</f>
-        <v>-2143050.000000001</v>
+        <v>-2271750</v>
       </c>
       <c r="R30" s="5">
         <f>IF($P30="","",$P30+ROW()/1000000)</f>
-        <v>-714.3499690000003</v>
+        <v>-757.249969</v>
       </c>
     </row>
     <row r="31">
@@ -2460,7 +2460,7 @@
       <c r="K32" s="2"/>
       <c r="L32" s="2">
         <f>IFERROR((IF($D32="","",VLOOKUP($D32,Prices!$A$2:$D$174,3,0))*$E32)+(IF($F32="","",VLOOKUP($F32,Prices!$A$2:$D$174,3,0))*$G32)+(IF($H32="","",VLOOKUP($H32,Prices!$A$2:$D$174,3,0))*$I32),"")</f>
-        <v>2583</v>
+        <v>2619</v>
       </c>
       <c r="M32" s="2">
         <f>IFERROR(VLOOKUP($A32,Prices!$A$2:$D$174,4,0),"")</f>
@@ -2472,19 +2472,19 @@
       </c>
       <c r="O32" s="2">
         <f>IFERROR((IF($H32="","",VLOOKUP($H32,Prices!$A$2:$D$174,3,0))*$I32),"")</f>
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="P32" s="2">
         <f>IF(OR($L32="",$M32=""),"",$M32-($L32-0.1*'Top 8'!$J$5*$O32))</f>
-        <v>-967.8000000000002</v>
+        <v>-1003.9000000000001</v>
       </c>
       <c r="Q32" s="2">
         <f>IF($P32="","",$P32*3000)</f>
-        <v>-2903400.0000000005</v>
+        <v>-3011700.0000000005</v>
       </c>
       <c r="R32" s="5">
         <f>IF($P32="","",$P32+ROW()/1000000)</f>
-        <v>-967.7999670000002</v>
+        <v>-1003.8999670000001</v>
       </c>
     </row>
     <row r="33">
@@ -2521,11 +2521,11 @@
       <c r="K33" s="2"/>
       <c r="L33" s="2">
         <f>IFERROR((IF($D33="","",VLOOKUP($D33,Prices!$A$2:$D$174,3,0))*$E33)+(IF($F33="","",VLOOKUP($F33,Prices!$A$2:$D$174,3,0))*$G33),"")</f>
-        <v>1755</v>
+        <v>1754</v>
       </c>
       <c r="M33" s="2">
         <f>IFERROR(VLOOKUP($A33,Prices!$A$2:$D$174,4,0),"")</f>
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="N33" s="2">
         <f>IF(ISNUMBER(SEARCH("(4)",$A33)),IFERROR(VLOOKUP(SUBSTITUTE($A33,"(4)","(2)"),Prices!$A$2:$D$174,4,0),""),"")</f>
@@ -2533,19 +2533,19 @@
       </c>
       <c r="O33" s="2">
         <f>IFERROR((IF($F33="","",VLOOKUP($F33,Prices!$A$2:$D$174,3,0))*$G33),"")</f>
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="P33" s="2">
         <f>IF(OR($L33="",$M33=""),"",(3+0.15*'Top 8'!$J$4)*($M33+$N33)/6-($L33-0.1*'Top 8'!$J$5*$O33))</f>
-        <v>-1025.5</v>
+        <v>-1025.125</v>
       </c>
       <c r="Q33" s="2">
         <f>IF($P33="","",$P33*3000)</f>
-        <v>-3076500</v>
+        <v>-3075375</v>
       </c>
       <c r="R33" s="5">
         <f>IF($P33="","",$P33+ROW()/1000000)</f>
-        <v>-1025.499966</v>
+        <v>-1025.124966</v>
       </c>
     </row>
     <row r="34">
@@ -2582,31 +2582,31 @@
       <c r="K34" s="2"/>
       <c r="L34" s="2">
         <f>IFERROR((IF($D34="","",VLOOKUP($D34,Prices!$A$2:$D$174,3,0))*$E34)+(IF($F34="","",VLOOKUP($F34,Prices!$A$2:$D$174,3,0))*$G34),"")</f>
-        <v>2597</v>
+        <v>2604</v>
       </c>
       <c r="M34" s="2">
         <f>IFERROR(VLOOKUP($A34,Prices!$A$2:$D$174,4,0),"")</f>
-        <v>1693</v>
+        <v>1718</v>
       </c>
       <c r="N34" s="2">
         <f>IF(ISNUMBER(SEARCH("(4)",$A34)),IFERROR(VLOOKUP(SUBSTITUTE($A34,"(4)","(2)"),Prices!$A$2:$D$174,4,0),""),"")</f>
-        <v>903</v>
+        <v>908</v>
       </c>
       <c r="O34" s="2">
         <f>IFERROR((IF($F34="","",VLOOKUP($F34,Prices!$A$2:$D$174,3,0))*$G34),"")</f>
-        <v>917</v>
+        <v>924</v>
       </c>
       <c r="P34" s="2">
         <f>IF(OR($L34="",$M34=""),"",(3+0.15*'Top 8'!$J$4)*($M34+$N34)/6-($L34-0.1*'Top 8'!$J$5*$O34))</f>
-        <v>-1142.4</v>
+        <v>-1132.9499999999998</v>
       </c>
       <c r="Q34" s="2">
         <f>IF($P34="","",$P34*3000)</f>
-        <v>-3427200.0000000005</v>
+        <v>-3398849.9999999995</v>
       </c>
       <c r="R34" s="5">
         <f>IF($P34="","",$P34+ROW()/1000000)</f>
-        <v>-1142.399965</v>
+        <v>-1132.9499649999998</v>
       </c>
     </row>
     <row r="35">
@@ -2649,7 +2649,7 @@
       <c r="K35" s="2"/>
       <c r="L35" s="2">
         <f>IFERROR((IF($D35="","",VLOOKUP($D35,Prices!$A$2:$D$174,3,0))*$E35)+(IF($F35="","",VLOOKUP($F35,Prices!$A$2:$D$174,3,0))*$G35)+(IF($H35="","",VLOOKUP($H35,Prices!$A$2:$D$174,3,0))*$I35),"")</f>
-        <v>2074</v>
+        <v>2056</v>
       </c>
       <c r="M35" s="2">
         <f>IFERROR(VLOOKUP($A35,Prices!$A$2:$D$174,4,0),"")</f>
@@ -2660,19 +2660,19 @@
       </c>
       <c r="O35" s="2">
         <f>IFERROR((IF($H35="","",VLOOKUP($H35,Prices!$A$2:$D$174,3,0))*$I35),"")</f>
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="P35" s="2">
         <f>IF(OR($L35="",$M35=""),"",$M35-($L35-0.1*'Top 8'!$J$5*$O35))</f>
-        <v>-1157.4</v>
+        <v>-1139.6</v>
       </c>
       <c r="Q35" s="2">
         <f>IF($P35="","",$P35*3000)</f>
-        <v>-3472200.0000000005</v>
+        <v>-3418799.9999999995</v>
       </c>
       <c r="R35" s="5">
         <f>IF($P35="","",$P35+ROW()/1000000)</f>
-        <v>-1157.3999640000002</v>
+        <v>-1139.599964</v>
       </c>
     </row>
     <row r="36">
@@ -2713,7 +2713,7 @@
       </c>
       <c r="M36" s="2">
         <f>IFERROR(VLOOKUP($A36,Prices!$A$2:$D$174,4,0),"")</f>
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="N36" s="2">
         <f>IF(ISNUMBER(SEARCH("(4)",$A36)),IFERROR(VLOOKUP(SUBSTITUTE($A36,"(4)","(2)"),Prices!$A$2:$D$174,4,0),""),"")</f>
@@ -2725,15 +2725,15 @@
       </c>
       <c r="P36" s="2">
         <f>IF(OR($L36="",$M36=""),"",(3+0.15*'Top 8'!$J$4)*($M36+$N36)/6-($L36-0.1*'Top 8'!$J$5*$O36))</f>
-        <v>-1642.225</v>
+        <v>-1644.325</v>
       </c>
       <c r="Q36" s="2">
         <f>IF($P36="","",$P36*3000)</f>
-        <v>-4926675</v>
+        <v>-4932975</v>
       </c>
       <c r="R36" s="5">
         <f>IF($P36="","",$P36+ROW()/1000000)</f>
-        <v>-1642.224963</v>
+        <v>-1644.324963</v>
       </c>
     </row>
     <row r="37">
@@ -2770,11 +2770,11 @@
       <c r="K37" s="2"/>
       <c r="L37" s="2">
         <f>IFERROR(0.75*((IF($D37="","",VLOOKUP($D37,Prices!$A$2:$D$174,3,0))*$E37)+(IF($F37="","",VLOOKUP($F37,Prices!$A$2:$D$174,3,0))*$G37)),"")</f>
-        <v>3441.75</v>
+        <v>3484.5</v>
       </c>
       <c r="M37" s="2">
         <f>IFERROR(VLOOKUP($A37,Prices!$A$2:$D$174,4,0),"")</f>
-        <v>3855</v>
+        <v>3990</v>
       </c>
       <c r="N37" s="2">
         <f>IF(ISNUMBER(SEARCH("(4)",$A37)),IFERROR(VLOOKUP(SUBSTITUTE($A37,"(4)","(2)"),Prices!$A$2:$D$174,4,0),""),"")</f>
@@ -2782,19 +2782,19 @@
       </c>
       <c r="O37" s="2">
         <f>IFERROR(0.75*((IF($F37="","",VLOOKUP($F37,Prices!$A$2:$D$174,3,0))*$G37)),"")</f>
-        <v>1530</v>
+        <v>1521</v>
       </c>
       <c r="P37" s="2">
         <f>IF(OR($L37="",$M37=""),"",(3+0.15*'Top 8'!$J$4)*($M37+$N37)/6-($L37-0.1*'Top 8'!$J$5*$O37))</f>
-        <v>-306.2249999999999</v>
+        <v>-279</v>
       </c>
       <c r="Q37" s="2">
         <f>IF($P37="","",$P37*3000)</f>
-        <v>-918674.9999999998</v>
+        <v>-837000</v>
       </c>
       <c r="R37" s="5">
         <f>IF($P37="","",$P37+ROW()/1000000)</f>
-        <v>-306.2249619999999</v>
+        <v>-278.999962</v>
       </c>
     </row>
     <row r="38">
@@ -2831,7 +2831,7 @@
       <c r="K38" s="2"/>
       <c r="L38" s="2">
         <f>IFERROR((IF($D38="","",VLOOKUP($D38,Prices!$A$2:$D$174,3,0))*$E38)+(IF($F38="","",VLOOKUP($F38,Prices!$A$2:$D$174,3,0))*$G38),"")</f>
-        <v>4244</v>
+        <v>4248</v>
       </c>
       <c r="M38" s="2">
         <f>IFERROR(VLOOKUP($A38,Prices!$A$2:$D$174,4,0),"")</f>
@@ -2839,23 +2839,23 @@
       </c>
       <c r="N38" s="2">
         <f>IF(ISNUMBER(SEARCH("(4)",$A38)),IFERROR(VLOOKUP(SUBSTITUTE($A38,"(4)","(2)"),Prices!$A$2:$D$174,4,0),""),"")</f>
-        <v>533</v>
+        <v>506</v>
       </c>
       <c r="O38" s="2">
         <f>IFERROR((IF($F38="","",VLOOKUP($F38,Prices!$A$2:$D$174,3,0))*$G38),"")</f>
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="P38" s="2">
         <f>IF(OR($L38="",$M38=""),"",(3+0.15*'Top 8'!$J$4)*($M38+$N38)/6-($L38-0.1*'Top 8'!$J$5*$O38))</f>
-        <v>-3617.2</v>
+        <v>-3634.9750000000004</v>
       </c>
       <c r="Q38" s="2">
         <f>IF($P38="","",$P38*3000)</f>
-        <v>-10851600</v>
+        <v>-10904925.000000002</v>
       </c>
       <c r="R38" s="5">
         <f>IF($P38="","",$P38+ROW()/1000000)</f>
-        <v>-3617.199961</v>
+        <v>-3634.9749610000003</v>
       </c>
     </row>
     <row r="39">
@@ -2898,11 +2898,11 @@
       <c r="K39" s="2"/>
       <c r="L39" s="2">
         <f>IFERROR((IF($D39="","",VLOOKUP($D39,Prices!$A$2:$D$174,3,0))*$E39)+(IF($F39="","",VLOOKUP($F39,Prices!$A$2:$D$174,3,0))*$G39)+(IF($H39="","",VLOOKUP($H39,Prices!$A$2:$D$174,3,0))*$I39),"")</f>
-        <v>9728</v>
+        <v>9783</v>
       </c>
       <c r="M39" s="2">
         <f>IFERROR(VLOOKUP($A39,Prices!$A$2:$D$174,4,0),"")</f>
-        <v>8899</v>
+        <v>8583</v>
       </c>
       <c r="N39" s="2">
         <f>IF(ISNUMBER(SEARCH("(4)",$A39)),IFERROR(VLOOKUP(SUBSTITUTE($A39,"(4)","(2)"),Prices!$A$2:$D$174,4,0),""),"")</f>
@@ -2910,19 +2910,19 @@
       </c>
       <c r="O39" s="2">
         <f>IFERROR((IF($H39="","",VLOOKUP($H39,Prices!$A$2:$D$174,3,0))*$I39),"")</f>
-        <v>7963</v>
+        <v>8034</v>
       </c>
       <c r="P39" s="2">
         <f>IF(OR($L39="",$M39=""),"",$M39-($L39-0.1*'Top 8'!$J$5*$O39))</f>
-        <v>-32.70000000000073</v>
+        <v>-396.60000000000036</v>
       </c>
       <c r="Q39" s="2">
         <f>IF($P39="","",$P39*3000)</f>
-        <v>-98100.00000000218</v>
+        <v>-1189800.0000000012</v>
       </c>
       <c r="R39" s="5">
         <f>IF($P39="","",$P39+ROW()/1000000)</f>
-        <v>-32.69996000000073</v>
+        <v>-396.59996000000035</v>
       </c>
     </row>
     <row r="40">
@@ -2965,11 +2965,11 @@
       <c r="K40" s="2"/>
       <c r="L40" s="2">
         <f>IFERROR((IF($D40="","",VLOOKUP($D40,Prices!$A$2:$D$174,3,0))*$E40)+(IF($F40="","",VLOOKUP($F40,Prices!$A$2:$D$174,3,0))*$G40)+(IF($H40="","",VLOOKUP($H40,Prices!$A$2:$D$174,3,0))*$I40),"")</f>
-        <v>11700</v>
+        <v>11830</v>
       </c>
       <c r="M40" s="2">
         <f>IFERROR(VLOOKUP($A40,Prices!$A$2:$D$174,4,0),"")</f>
-        <v>15100</v>
+        <v>15294</v>
       </c>
       <c r="N40" s="2">
         <f>IF(ISNUMBER(SEARCH("(4)",$A40)),IFERROR(VLOOKUP(SUBSTITUTE($A40,"(4)","(2)"),Prices!$A$2:$D$174,4,0),""),"")</f>
@@ -2977,19 +2977,19 @@
       </c>
       <c r="O40" s="2">
         <f>IFERROR((IF($H40="","",VLOOKUP($H40,Prices!$A$2:$D$174,3,0))*$I40),"")</f>
-        <v>917</v>
+        <v>924</v>
       </c>
       <c r="P40" s="2">
         <f>IF(OR($L40="",$M40=""),"",(3+0.15*'Top 8'!$J$4)*($M40+$N40)/6-($L40-0.1*'Top 8'!$J$5*$O40))</f>
-        <v>-185.875</v>
+        <v>-213.32500000000073</v>
       </c>
       <c r="Q40" s="2">
         <f>IF($P40="","",$P40*3000)</f>
-        <v>-557625</v>
+        <v>-639975.0000000022</v>
       </c>
       <c r="R40" s="5">
         <f>IF($P40="","",$P40+ROW()/1000000)</f>
-        <v>-185.874959</v>
+        <v>-213.32495900000072</v>
       </c>
     </row>
     <row r="41">
@@ -3032,7 +3032,7 @@
       <c r="K41" s="2"/>
       <c r="L41" s="2">
         <f>IFERROR((IF($D41="","",VLOOKUP($D41,Prices!$A$2:$D$174,3,0))*$E41)+(IF($F41="","",VLOOKUP($F41,Prices!$A$2:$D$174,3,0))*$G41)+(IF($H41="","",VLOOKUP($H41,Prices!$A$2:$D$174,3,0))*$I41),"")</f>
-        <v>10848</v>
+        <v>10971</v>
       </c>
       <c r="M41" s="2">
         <f>IFERROR(VLOOKUP($A41,Prices!$A$2:$D$174,4,0),"")</f>
@@ -3048,15 +3048,15 @@
       </c>
       <c r="P41" s="2">
         <f>IF(OR($L41="",$M41=""),"",(3+0.15*'Top 8'!$J$4)*($M41+$N41)/6-($L41-0.1*'Top 8'!$J$5*$O41))</f>
-        <v>115.77499999999964</v>
+        <v>-7.225000000000364</v>
       </c>
       <c r="Q41" s="2">
         <f>IF($P41="","",$P41*3000)</f>
-        <v>347324.9999999989</v>
+        <v>-21675.00000000109</v>
       </c>
       <c r="R41" s="5">
         <f>IF($P41="","",$P41+ROW()/1000000)</f>
-        <v>115.77504199999963</v>
+        <v>-7.224958000000364</v>
       </c>
     </row>
     <row r="42">
@@ -3093,11 +3093,11 @@
       <c r="K42" s="2"/>
       <c r="L42" s="2">
         <f>IFERROR((IF($D42="","",VLOOKUP($D42,Prices!$A$2:$D$174,3,0))*$E42)+(IF($F42="","",VLOOKUP($F42,Prices!$A$2:$D$174,3,0))*$G42),"")</f>
-        <v>6981</v>
+        <v>6966</v>
       </c>
       <c r="M42" s="2">
         <f>IFERROR(VLOOKUP($A42,Prices!$A$2:$D$174,4,0),"")</f>
-        <v>6773</v>
+        <v>6784</v>
       </c>
       <c r="N42" s="2">
         <f>IF(ISNUMBER(SEARCH("(4)",$A42)),IFERROR(VLOOKUP(SUBSTITUTE($A42,"(4)","(2)"),Prices!$A$2:$D$174,4,0),""),"")</f>
@@ -3105,19 +3105,19 @@
       </c>
       <c r="O42" s="2">
         <f>IFERROR((IF($F42="","",VLOOKUP($F42,Prices!$A$2:$D$174,3,0))*$G42),"")</f>
-        <v>4391</v>
+        <v>4376</v>
       </c>
       <c r="P42" s="2">
         <f>IF(OR($L42="",$M42=""),"",(3+0.15*'Top 8'!$J$4)*($M42+$N42)/6-($L42-0.1*'Top 8'!$J$5*$O42))</f>
-        <v>-1283.5</v>
+        <v>-1264.2249999999995</v>
       </c>
       <c r="Q42" s="2">
         <f>IF($P42="","",$P42*3000)</f>
-        <v>-3850500</v>
+        <v>-3792674.999999998</v>
       </c>
       <c r="R42" s="5">
         <f>IF($P42="","",$P42+ROW()/1000000)</f>
-        <v>-1283.499957</v>
+        <v>-1264.2249569999994</v>
       </c>
     </row>
     <row r="43">
@@ -3210,11 +3210,11 @@
       <c r="K44" s="2"/>
       <c r="L44" s="2">
         <f>IFERROR(0.75*((IF($D44="","",VLOOKUP($D44,Prices!$A$2:$D$174,3,0))*$E44)+(IF($F44="","",VLOOKUP($F44,Prices!$A$2:$D$174,3,0))*$G44)),"")</f>
-        <v>927</v>
+        <v>926.25</v>
       </c>
       <c r="M44" s="2">
         <f>IFERROR(VLOOKUP($A44,Prices!$A$2:$D$174,4,0),"")</f>
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="N44" s="2">
         <f>IF(ISNUMBER(SEARCH("(4)",$A44)),IFERROR(VLOOKUP(SUBSTITUTE($A44,"(4)","(2)"),Prices!$A$2:$D$174,4,0),""),"")</f>
@@ -3226,15 +3226,15 @@
       </c>
       <c r="P44" s="2">
         <f>IF(OR($L44="",$M44=""),"",(3+0.15*'Top 8'!$J$4)*($M44+$N44)/6-($L44-0.1*'Top 8'!$J$5*$O44))</f>
-        <v>-646.275</v>
+        <v>-650.25</v>
       </c>
       <c r="Q44" s="2">
         <f>IF($P44="","",$P44*3000)</f>
-        <v>-1938825</v>
+        <v>-1950750</v>
       </c>
       <c r="R44" s="5">
         <f>IF($P44="","",$P44+ROW()/1000000)</f>
-        <v>-646.274955</v>
+        <v>-650.249955</v>
       </c>
     </row>
     <row r="45">
@@ -3332,15 +3332,15 @@
       <c r="K46" s="2"/>
       <c r="L46" s="2">
         <f>IFERROR(0.75*((IF($D46="","",VLOOKUP($D46,Prices!$A$2:$D$174,3,0))*$E46)+(IF($F46="","",VLOOKUP($F46,Prices!$A$2:$D$174,3,0))*$G46)),"")</f>
-        <v>6423.75</v>
+        <v>6527.25</v>
       </c>
       <c r="M46" s="2">
         <f>IFERROR(VLOOKUP($A46,Prices!$A$2:$D$174,4,0),"")</f>
-        <v>7622</v>
+        <v>7599</v>
       </c>
       <c r="N46" s="2">
         <f>IF(ISNUMBER(SEARCH("(4)",$A46)),IFERROR(VLOOKUP(SUBSTITUTE($A46,"(4)","(2)"),Prices!$A$2:$D$174,4,0),""),"")</f>
-        <v>3600</v>
+        <v>3601</v>
       </c>
       <c r="O46" s="2">
         <f>IFERROR(0.75*((IF($F46="","",VLOOKUP($F46,Prices!$A$2:$D$174,3,0))*$G46)),"")</f>
@@ -3348,15 +3348,15 @@
       </c>
       <c r="P46" s="2">
         <f>IF(OR($L46="",$M46=""),"",(3+0.15*'Top 8'!$J$4)*($M46+$N46)/6-($L46-0.1*'Top 8'!$J$5*$O46))</f>
-        <v>-184.8000000000011</v>
+        <v>-299.85000000000036</v>
       </c>
       <c r="Q46" s="2">
         <f>IF($P46="","",$P46*3000)</f>
-        <v>-554400.0000000033</v>
+        <v>-899550.000000001</v>
       </c>
       <c r="R46" s="5">
         <f>IF($P46="","",$P46+ROW()/1000000)</f>
-        <v>-184.7999530000011</v>
+        <v>-299.84995300000037</v>
       </c>
     </row>
     <row r="47">
@@ -3393,11 +3393,11 @@
       <c r="K47" s="2"/>
       <c r="L47" s="2">
         <f>IFERROR(0.75*((IF($D47="","",VLOOKUP($D47,Prices!$A$2:$D$174,3,0))*$E47)+(IF($F47="","",VLOOKUP($F47,Prices!$A$2:$D$174,3,0))*$G47)),"")</f>
-        <v>9105</v>
+        <v>8863.5</v>
       </c>
       <c r="M47" s="2">
         <f>IFERROR(VLOOKUP($A47,Prices!$A$2:$D$174,4,0),"")</f>
-        <v>10907</v>
+        <v>10787</v>
       </c>
       <c r="N47" s="2">
         <f>IF(ISNUMBER(SEARCH("(4)",$A47)),IFERROR(VLOOKUP(SUBSTITUTE($A47,"(4)","(2)"),Prices!$A$2:$D$174,4,0),""),"")</f>
@@ -3409,15 +3409,15 @@
       </c>
       <c r="P47" s="2">
         <f>IF(OR($L47="",$M47=""),"",(3+0.15*'Top 8'!$J$4)*($M47+$N47)/6-($L47-0.1*'Top 8'!$J$5*$O47))</f>
-        <v>-504.375</v>
+        <v>-325.875</v>
       </c>
       <c r="Q47" s="2">
         <f>IF($P47="","",$P47*3000)</f>
-        <v>-1513125</v>
+        <v>-977625</v>
       </c>
       <c r="R47" s="5">
         <f>IF($P47="","",$P47+ROW()/1000000)</f>
-        <v>-504.374952</v>
+        <v>-325.874952</v>
       </c>
     </row>
     <row r="48">
@@ -3454,7 +3454,7 @@
       <c r="K48" s="2"/>
       <c r="L48" s="2">
         <f>IFERROR((IF($D48="","",VLOOKUP($D48,Prices!$A$2:$D$174,3,0))*$E48)+(IF($F48="","",VLOOKUP($F48,Prices!$A$2:$D$174,3,0))*$G48),"")</f>
-        <v>3543</v>
+        <v>3575</v>
       </c>
       <c r="M48" s="2">
         <f>IFERROR(VLOOKUP($A48,Prices!$A$2:$D$174,4,0),"")</f>
@@ -3466,19 +3466,19 @@
       </c>
       <c r="O48" s="2">
         <f>IFERROR((IF($F48="","",VLOOKUP($F48,Prices!$A$2:$D$174,3,0))*$G48),"")</f>
-        <v>1863</v>
+        <v>1895</v>
       </c>
       <c r="P48" s="2">
         <f>IF(OR($L48="",$M48=""),"",(3+0.15*'Top 8'!$J$4)*($M48+$N48)/6-($L48-0.1*'Top 8'!$J$5*$O48))</f>
-        <v>-1837.35</v>
+        <v>-1866.15</v>
       </c>
       <c r="Q48" s="2">
         <f>IF($P48="","",$P48*3000)</f>
-        <v>-5512050</v>
+        <v>-5598450</v>
       </c>
       <c r="R48" s="5">
         <f>IF($P48="","",$P48+ROW()/1000000)</f>
-        <v>-1837.349951</v>
+        <v>-1866.149951</v>
       </c>
     </row>
     <row r="49">
@@ -3588,31 +3588,31 @@
       </c>
       <c r="L50" s="2">
         <f>IFERROR((IF($D50="","",VLOOKUP($D50,Prices!$A$2:$D$174,3,0))*$E50)+(IF($F50="","",VLOOKUP($F50,Prices!$A$2:$D$174,3,0))*$G50)+(IF($H50="","",VLOOKUP($H50,Prices!$A$2:$D$174,3,0))*$I50)+(IF($J50="","",VLOOKUP($J50,Prices!$A$2:$D$174,3,0))*$K50),"")</f>
-        <v>11921</v>
+        <v>11896</v>
       </c>
       <c r="M50" s="2">
         <f>IFERROR(VLOOKUP($A50,Prices!$A$2:$D$174,4,0),"")</f>
-        <v>12034</v>
+        <v>11968</v>
       </c>
       <c r="N50" s="2">
         <f>IF(ISNUMBER(SEARCH("(4)",$A50)),IFERROR(VLOOKUP(SUBSTITUTE($A50,"(4)","(2)"),Prices!$A$2:$D$174,4,0),""),"")</f>
-        <v>6102</v>
+        <v>6130</v>
       </c>
       <c r="O50" s="2">
         <f>IFERROR((IF($J50="","",VLOOKUP($J50,Prices!$A$2:$D$174,3,0))*$K50),"")</f>
-        <v>3697</v>
+        <v>3737</v>
       </c>
       <c r="P50" s="2">
         <f>IF(OR($L50="",$M50=""),"",$M50-($L50-0.1*'Top 8'!$J$5*$O50))</f>
-        <v>482.7000000000007</v>
+        <v>445.7000000000007</v>
       </c>
       <c r="Q50" s="2">
         <f>IF($P50="","",$P50*3000)</f>
-        <v>1448100.000000002</v>
+        <v>1337100.000000002</v>
       </c>
       <c r="R50" s="5">
         <f>IF($P50="","",$P50+ROW()/1000000)</f>
-        <v>482.7000510000007</v>
+        <v>445.7000510000007</v>
       </c>
     </row>
     <row r="51">
@@ -3653,7 +3653,7 @@
       </c>
       <c r="M51" s="2">
         <f>IFERROR(VLOOKUP($A51,Prices!$A$2:$D$174,4,0),"")</f>
-        <v>3768</v>
+        <v>3770</v>
       </c>
       <c r="N51" s="2">
         <f>IF(ISNUMBER(SEARCH("(4)",$A51)),IFERROR(VLOOKUP(SUBSTITUTE($A51,"(4)","(2)"),Prices!$A$2:$D$174,4,0),""),"")</f>
@@ -3665,15 +3665,15 @@
       </c>
       <c r="P51" s="2">
         <f>IF(OR($L51="",$M51=""),"",(3+0.15*'Top 8'!$J$4)*($M51+$N51)/6-($L51-0.1*'Top 8'!$J$5*$O51))</f>
-        <v>86.77499999999964</v>
+        <v>87.82500000000027</v>
       </c>
       <c r="Q51" s="2">
         <f>IF($P51="","",$P51*3000)</f>
-        <v>260324.9999999989</v>
+        <v>263475.0000000008</v>
       </c>
       <c r="R51" s="5">
         <f>IF($P51="","",$P51+ROW()/1000000)</f>
-        <v>86.77505199999963</v>
+        <v>87.82505200000027</v>
       </c>
     </row>
     <row r="52">
@@ -3710,11 +3710,11 @@
       <c r="K52" s="2"/>
       <c r="L52" s="2">
         <f>IFERROR((IF($D52="","",VLOOKUP($D52,Prices!$A$2:$D$174,3,0))*$E52)+(IF($F52="","",VLOOKUP($F52,Prices!$A$2:$D$174,3,0))*$G52),"")</f>
-        <v>21214</v>
+        <v>21213</v>
       </c>
       <c r="M52" s="2">
         <f>IFERROR(VLOOKUP($A52,Prices!$A$2:$D$174,4,0),"")</f>
-        <v>19006</v>
+        <v>18960</v>
       </c>
       <c r="N52" s="2">
         <f>IF(ISNUMBER(SEARCH("(4)",$A52)),IFERROR(VLOOKUP(SUBSTITUTE($A52,"(4)","(2)"),Prices!$A$2:$D$174,4,0),""),"")</f>
@@ -3726,15 +3726,15 @@
       </c>
       <c r="P52" s="2">
         <f>IF(OR($L52="",$M52=""),"",$M52-($L52-0.1*'Top 8'!$J$5*$O52))</f>
-        <v>-175.40000000000146</v>
+        <v>-220.40000000000146</v>
       </c>
       <c r="Q52" s="2">
         <f>IF($P52="","",$P52*3000)</f>
-        <v>-526200.0000000044</v>
+        <v>-661200.0000000044</v>
       </c>
       <c r="R52" s="5">
         <f>IF($P52="","",$P52+ROW()/1000000)</f>
-        <v>-175.39994700000145</v>
+        <v>-220.39994700000145</v>
       </c>
     </row>
     <row r="53">
@@ -3771,31 +3771,31 @@
       <c r="K53" s="2"/>
       <c r="L53" s="2">
         <f>IFERROR((IF($D53="","",VLOOKUP($D53,Prices!$A$2:$D$174,3,0))*$E53)+(IF($F53="","",VLOOKUP($F53,Prices!$A$2:$D$174,3,0))*$G53),"")</f>
-        <v>14826</v>
+        <v>14744</v>
       </c>
       <c r="M53" s="2">
         <f>IFERROR(VLOOKUP($A53,Prices!$A$2:$D$174,4,0),"")</f>
-        <v>14326</v>
+        <v>14325</v>
       </c>
       <c r="N53" s="2">
         <f>IF(ISNUMBER(SEARCH("(4)",$A53)),IFERROR(VLOOKUP(SUBSTITUTE($A53,"(4)","(2)"),Prices!$A$2:$D$174,4,0),""),"")</f>
-        <v>7144</v>
+        <v>7338</v>
       </c>
       <c r="O53" s="2">
         <f>IFERROR((IF($F53="","",VLOOKUP($F53,Prices!$A$2:$D$174,3,0))*$G53),"")</f>
-        <v>3697</v>
+        <v>3737</v>
       </c>
       <c r="P53" s="2">
         <f>IF(OR($L53="",$M53=""),"",$M53-($L53-0.1*'Top 8'!$J$5*$O53))</f>
-        <v>-130.29999999999927</v>
+        <v>-45.29999999999927</v>
       </c>
       <c r="Q53" s="2">
         <f>IF($P53="","",$P53*3000)</f>
-        <v>-390899.9999999978</v>
+        <v>-135899.99999999782</v>
       </c>
       <c r="R53" s="5">
         <f>IF($P53="","",$P53+ROW()/1000000)</f>
-        <v>-130.29994599999927</v>
+        <v>-45.299945999999274</v>
       </c>
     </row>
     <row r="54">
@@ -3832,11 +3832,11 @@
       <c r="K54" s="2"/>
       <c r="L54" s="2">
         <f>IFERROR(0.75*((IF($D54="","",VLOOKUP($D54,Prices!$A$2:$D$174,3,0))*$E54)+(IF($F54="","",VLOOKUP($F54,Prices!$A$2:$D$174,3,0))*$G54)),"")</f>
-        <v>14185.5</v>
+        <v>14163.75</v>
       </c>
       <c r="M54" s="2">
         <f>IFERROR(VLOOKUP($A54,Prices!$A$2:$D$174,4,0),"")</f>
-        <v>18218</v>
+        <v>18171</v>
       </c>
       <c r="N54" s="2">
         <f>IF(ISNUMBER(SEARCH("(4)",$A54)),IFERROR(VLOOKUP(SUBSTITUTE($A54,"(4)","(2)"),Prices!$A$2:$D$174,4,0),""),"")</f>
@@ -3844,19 +3844,19 @@
       </c>
       <c r="O54" s="2">
         <f>IFERROR(0.75*((IF($F54="","",VLOOKUP($F54,Prices!$A$2:$D$174,3,0))*$G54)),"")</f>
-        <v>3222</v>
+        <v>3201</v>
       </c>
       <c r="P54" s="2">
         <f>IF(OR($L54="",$M54=""),"",(3+0.15*'Top 8'!$J$4)*($M54+$N54)/6-($L54-0.1*'Top 8'!$J$5*$O54))</f>
-        <v>867.1499999999996</v>
+        <v>862.125</v>
       </c>
       <c r="Q54" s="2">
         <f>IF($P54="","",$P54*3000)</f>
-        <v>2601449.999999999</v>
+        <v>2586375</v>
       </c>
       <c r="R54" s="5">
         <f>IF($P54="","",$P54+ROW()/1000000)</f>
-        <v>867.1500549999996</v>
+        <v>862.125055</v>
       </c>
     </row>
     <row r="55">
@@ -3893,11 +3893,11 @@
       <c r="K55" s="2"/>
       <c r="L55" s="2">
         <f>IFERROR(0.75*((IF($D55="","",VLOOKUP($D55,Prices!$A$2:$D$174,3,0))*$E55)+(IF($F55="","",VLOOKUP($F55,Prices!$A$2:$D$174,3,0))*$G55)),"")</f>
-        <v>14805.75</v>
+        <v>14770.5</v>
       </c>
       <c r="M55" s="2">
         <f>IFERROR(VLOOKUP($A55,Prices!$A$2:$D$174,4,0),"")</f>
-        <v>17667</v>
+        <v>17330</v>
       </c>
       <c r="N55" s="2">
         <f>IF(ISNUMBER(SEARCH("(4)",$A55)),IFERROR(VLOOKUP(SUBSTITUTE($A55,"(4)","(2)"),Prices!$A$2:$D$174,4,0),""),"")</f>
@@ -3909,15 +3909,15 @@
       </c>
       <c r="P55" s="2">
         <f>IF(OR($L55="",$M55=""),"",(3+0.15*'Top 8'!$J$4)*($M55+$N55)/6-($L55-0.1*'Top 8'!$J$5*$O55))</f>
-        <v>-650.3250000000007</v>
+        <v>-792.0000000000018</v>
       </c>
       <c r="Q55" s="2">
         <f>IF($P55="","",$P55*3000)</f>
-        <v>-1950975.000000002</v>
+        <v>-2376000.0000000056</v>
       </c>
       <c r="R55" s="5">
         <f>IF($P55="","",$P55+ROW()/1000000)</f>
-        <v>-650.3249440000008</v>
+        <v>-791.9999440000018</v>
       </c>
     </row>
   </sheetData>
@@ -3978,7 +3978,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -3992,14 +3992,14 @@
         <v>3032</v>
       </c>
       <c r="C3" s="2">
-        <v>340</v>
+        <v>357</v>
       </c>
       <c r="D3" s="2">
-        <v>334</v>
+        <v>350</v>
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -4013,14 +4013,14 @@
         <v>29993</v>
       </c>
       <c r="C4" s="2">
-        <v>51314</v>
+        <v>49018</v>
       </c>
       <c r="D4" s="2">
-        <v>50288</v>
+        <v>48038</v>
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -4034,14 +4034,14 @@
         <v>12640</v>
       </c>
       <c r="C5" s="2">
-        <v>510</v>
+        <v>507</v>
       </c>
       <c r="D5" s="2">
-        <v>500</v>
+        <v>497</v>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4062,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -4139,14 +4139,14 @@
         <v>12905</v>
       </c>
       <c r="C10" s="2">
-        <v>11129</v>
+        <v>11007</v>
       </c>
       <c r="D10" s="2">
-        <v>10907</v>
+        <v>10787</v>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -4160,14 +4160,14 @@
         <v>12917</v>
       </c>
       <c r="C11" s="2">
-        <v>7289</v>
+        <v>7487</v>
       </c>
       <c r="D11" s="2">
-        <v>7144</v>
+        <v>7338</v>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -4181,14 +4181,14 @@
         <v>12913</v>
       </c>
       <c r="C12" s="2">
-        <v>14618</v>
+        <v>14617</v>
       </c>
       <c r="D12" s="2">
-        <v>14326</v>
+        <v>14325</v>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -4209,7 +4209,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -4265,14 +4265,14 @@
         <v>5952</v>
       </c>
       <c r="C16" s="2">
-        <v>9080</v>
+        <v>8758</v>
       </c>
       <c r="D16" s="2">
-        <v>8899</v>
+        <v>8583</v>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -4307,14 +4307,14 @@
         <v>2452</v>
       </c>
       <c r="C18" s="2">
-        <v>888</v>
+        <v>887</v>
       </c>
       <c r="D18" s="2">
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -4349,14 +4349,14 @@
         <v>2446</v>
       </c>
       <c r="C20" s="2">
-        <v>455</v>
+        <v>453</v>
       </c>
       <c r="D20" s="2">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -4370,14 +4370,14 @@
         <v>29784</v>
       </c>
       <c r="C21" s="2">
-        <v>1074</v>
+        <v>1067</v>
       </c>
       <c r="D21" s="2">
-        <v>1053</v>
+        <v>1046</v>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -4433,14 +4433,14 @@
         <v>592</v>
       </c>
       <c r="C24" s="2">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D24" s="2">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -4538,14 +4538,14 @@
         <v>22461</v>
       </c>
       <c r="C29" s="2">
-        <v>15408</v>
+        <v>15606</v>
       </c>
       <c r="D29" s="2">
-        <v>15100</v>
+        <v>15294</v>
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -4601,14 +4601,14 @@
         <v>6016</v>
       </c>
       <c r="C32" s="2">
-        <v>1640</v>
+        <v>1613</v>
       </c>
       <c r="D32" s="2">
-        <v>1608</v>
+        <v>1581</v>
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -4622,14 +4622,14 @@
         <v>265</v>
       </c>
       <c r="C33" s="2">
-        <v>2244</v>
+        <v>2267</v>
       </c>
       <c r="D33" s="2">
-        <v>2200</v>
+        <v>2222</v>
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -4664,14 +4664,14 @@
         <v>1975</v>
       </c>
       <c r="C35" s="2">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D35" s="2">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -4685,14 +4685,14 @@
         <v>5935</v>
       </c>
       <c r="C36" s="2">
-        <v>248</v>
+        <v>259</v>
       </c>
       <c r="D36" s="2">
-        <v>244</v>
+        <v>254</v>
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -4706,14 +4706,14 @@
         <v>9743</v>
       </c>
       <c r="C37" s="2">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="D37" s="2">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -4734,7 +4734,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -4832,14 +4832,14 @@
         <v>6693</v>
       </c>
       <c r="C43" s="2">
-        <v>4391</v>
+        <v>4376</v>
       </c>
       <c r="D43" s="2">
-        <v>4304</v>
+        <v>4289</v>
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -4895,14 +4895,14 @@
         <v>135</v>
       </c>
       <c r="C46" s="2">
-        <v>357</v>
+        <v>342</v>
       </c>
       <c r="D46" s="2">
-        <v>350</v>
+        <v>336</v>
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -4916,14 +4916,14 @@
         <v>2432</v>
       </c>
       <c r="C47" s="2">
-        <v>563</v>
+        <v>582</v>
       </c>
       <c r="D47" s="2">
-        <v>552</v>
+        <v>571</v>
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -4958,14 +4958,14 @@
         <v>241</v>
       </c>
       <c r="C49" s="2">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D49" s="2">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -5042,14 +5042,14 @@
         <v>3008</v>
       </c>
       <c r="C53" s="2">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D53" s="2">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -5084,14 +5084,14 @@
         <v>29824</v>
       </c>
       <c r="C55" s="2">
-        <v>18589</v>
+        <v>18541</v>
       </c>
       <c r="D55" s="2">
-        <v>18218</v>
+        <v>18171</v>
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -5126,14 +5126,14 @@
         <v>11951</v>
       </c>
       <c r="C57" s="2">
-        <v>277</v>
+        <v>268</v>
       </c>
       <c r="D57" s="2">
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -5147,14 +5147,14 @@
         <v>31644</v>
       </c>
       <c r="C58" s="2">
-        <v>3673</v>
+        <v>3674</v>
       </c>
       <c r="D58" s="2">
-        <v>3600</v>
+        <v>3601</v>
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -5168,14 +5168,14 @@
         <v>31638</v>
       </c>
       <c r="C59" s="2">
-        <v>7777</v>
+        <v>7754</v>
       </c>
       <c r="D59" s="2">
-        <v>7622</v>
+        <v>7599</v>
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -5210,14 +5210,14 @@
         <v>22209</v>
       </c>
       <c r="C61" s="2">
-        <v>18027</v>
+        <v>17683</v>
       </c>
       <c r="D61" s="2">
-        <v>17667</v>
+        <v>17330</v>
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -5238,7 +5238,7 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -5252,14 +5252,14 @@
         <v>31614</v>
       </c>
       <c r="C63" s="2">
-        <v>2224</v>
+        <v>2295</v>
       </c>
       <c r="D63" s="2">
-        <v>2180</v>
+        <v>2250</v>
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -5273,14 +5273,14 @@
         <v>221</v>
       </c>
       <c r="C64" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D64" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -5322,7 +5322,7 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -5357,14 +5357,14 @@
         <v>27629</v>
       </c>
       <c r="C68" s="2">
-        <v>3844</v>
+        <v>3846</v>
       </c>
       <c r="D68" s="2">
-        <v>3768</v>
+        <v>3770</v>
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -5378,14 +5378,14 @@
         <v>1550</v>
       </c>
       <c r="C69" s="2">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D69" s="2">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -5399,14 +5399,14 @@
         <v>30143</v>
       </c>
       <c r="C70" s="2">
-        <v>31254</v>
+        <v>31874</v>
       </c>
       <c r="D70" s="2">
-        <v>30629</v>
+        <v>31237</v>
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -5420,14 +5420,14 @@
         <v>30137</v>
       </c>
       <c r="C71" s="2">
-        <v>60872</v>
+        <v>59527</v>
       </c>
       <c r="D71" s="2">
-        <v>59655</v>
+        <v>58337</v>
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -5441,14 +5441,14 @@
         <v>9736</v>
       </c>
       <c r="C72" s="2">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="D72" s="2">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -5462,14 +5462,14 @@
         <v>249</v>
       </c>
       <c r="C73" s="2">
-        <v>368</v>
+        <v>371</v>
       </c>
       <c r="D73" s="2">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -5525,14 +5525,14 @@
         <v>7660</v>
       </c>
       <c r="C76" s="2">
-        <v>1109</v>
+        <v>1146</v>
       </c>
       <c r="D76" s="2">
-        <v>1087</v>
+        <v>1124</v>
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -5546,14 +5546,14 @@
         <v>4421</v>
       </c>
       <c r="C77" s="2">
-        <v>1309</v>
+        <v>1256</v>
       </c>
       <c r="D77" s="2">
-        <v>1283</v>
+        <v>1231</v>
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -5567,14 +5567,14 @@
         <v>4417</v>
       </c>
       <c r="C78" s="2">
-        <v>2861</v>
+        <v>2851</v>
       </c>
       <c r="D78" s="2">
-        <v>2804</v>
+        <v>2794</v>
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -5595,7 +5595,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5637,7 @@
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -5672,14 +5672,14 @@
         <v>255</v>
       </c>
       <c r="C83" s="2">
-        <v>428</v>
+        <v>438</v>
       </c>
       <c r="D83" s="2">
-        <v>420</v>
+        <v>430</v>
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -5756,14 +5756,14 @@
         <v>9998</v>
       </c>
       <c r="C87" s="2">
-        <v>558</v>
+        <v>571</v>
       </c>
       <c r="D87" s="2">
-        <v>547</v>
+        <v>560</v>
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -5777,14 +5777,14 @@
         <v>259</v>
       </c>
       <c r="C88" s="2">
-        <v>1517</v>
+        <v>1490</v>
       </c>
       <c r="D88" s="2">
-        <v>1487</v>
+        <v>1461</v>
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -5819,14 +5819,14 @@
         <v>247</v>
       </c>
       <c r="C90" s="2">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="D90" s="2">
-        <v>319</v>
+        <v>323</v>
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -5840,14 +5840,14 @@
         <v>10111</v>
       </c>
       <c r="C91" s="2">
-        <v>784</v>
+        <v>765</v>
       </c>
       <c r="D91" s="2">
-        <v>769</v>
+        <v>750</v>
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -5924,14 +5924,14 @@
         <v>27272</v>
       </c>
       <c r="C95" s="2">
-        <v>1863</v>
+        <v>1895</v>
       </c>
       <c r="D95" s="2">
-        <v>1826</v>
+        <v>1858</v>
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -5945,14 +5945,14 @@
         <v>225</v>
       </c>
       <c r="C96" s="2">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="D96" s="2">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -5973,7 +5973,7 @@
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -5987,14 +5987,14 @@
         <v>3040</v>
       </c>
       <c r="C98" s="2">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="D98" s="2">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -6008,14 +6008,14 @@
         <v>6051</v>
       </c>
       <c r="C99" s="2">
-        <v>7963</v>
+        <v>8034</v>
       </c>
       <c r="D99" s="2">
-        <v>7804</v>
+        <v>7874</v>
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -6050,14 +6050,14 @@
         <v>251</v>
       </c>
       <c r="C101" s="2">
-        <v>320</v>
+        <v>331</v>
       </c>
       <c r="D101" s="2">
-        <v>314</v>
+        <v>325</v>
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6120,7 @@
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -6134,14 +6134,14 @@
         <v>2970</v>
       </c>
       <c r="C105" s="2">
-        <v>227</v>
+        <v>220</v>
       </c>
       <c r="D105" s="2">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -6155,14 +6155,14 @@
         <v>10937</v>
       </c>
       <c r="C106" s="2">
-        <v>811</v>
+        <v>803</v>
       </c>
       <c r="D106" s="2">
-        <v>795</v>
+        <v>787</v>
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -6225,7 +6225,7 @@
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -6239,14 +6239,14 @@
         <v>141</v>
       </c>
       <c r="C110" s="2">
-        <v>4587</v>
+        <v>4618</v>
       </c>
       <c r="D110" s="2">
-        <v>4496</v>
+        <v>4526</v>
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -6260,14 +6260,14 @@
         <v>2434</v>
       </c>
       <c r="C111" s="2">
-        <v>9541</v>
+        <v>9666</v>
       </c>
       <c r="D111" s="2">
-        <v>9351</v>
+        <v>9473</v>
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6288,7 @@
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -6302,14 +6302,14 @@
         <v>30125</v>
       </c>
       <c r="C113" s="2">
-        <v>70117</v>
+        <v>69550</v>
       </c>
       <c r="D113" s="2">
-        <v>68715</v>
+        <v>68159</v>
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -6365,14 +6365,14 @@
         <v>171</v>
       </c>
       <c r="C116" s="2">
-        <v>921</v>
+        <v>926</v>
       </c>
       <c r="D116" s="2">
-        <v>903</v>
+        <v>908</v>
       </c>
       <c r="E116" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -6386,14 +6386,14 @@
         <v>2444</v>
       </c>
       <c r="C117" s="2">
-        <v>1727</v>
+        <v>1753</v>
       </c>
       <c r="D117" s="2">
-        <v>1693</v>
+        <v>1718</v>
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -6407,14 +6407,14 @@
         <v>223</v>
       </c>
       <c r="C118" s="2">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="D118" s="2">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="E118" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -6449,14 +6449,14 @@
         <v>2430</v>
       </c>
       <c r="C120" s="2">
+        <v>57</v>
+      </c>
+      <c r="D120" s="2">
         <v>56</v>
       </c>
-      <c r="D120" s="2">
-        <v>55</v>
-      </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -6470,14 +6470,14 @@
         <v>10929</v>
       </c>
       <c r="C121" s="2">
-        <v>8427</v>
+        <v>8505</v>
       </c>
       <c r="D121" s="2">
-        <v>8259</v>
+        <v>8335</v>
       </c>
       <c r="E121" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -6491,14 +6491,14 @@
         <v>10925</v>
       </c>
       <c r="C122" s="2">
-        <v>19295</v>
+        <v>19479</v>
       </c>
       <c r="D122" s="2">
-        <v>18910</v>
+        <v>19090</v>
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -6533,14 +6533,14 @@
         <v>6685</v>
       </c>
       <c r="C124" s="2">
-        <v>6911</v>
+        <v>6922</v>
       </c>
       <c r="D124" s="2">
-        <v>6773</v>
+        <v>6784</v>
       </c>
       <c r="E124" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -6582,7 +6582,7 @@
       </c>
       <c r="E126" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -6596,14 +6596,14 @@
         <v>7650</v>
       </c>
       <c r="C127" s="2">
-        <v>750</v>
+        <v>762</v>
       </c>
       <c r="D127" s="2">
-        <v>735</v>
+        <v>747</v>
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -6638,14 +6638,14 @@
         <v>231</v>
       </c>
       <c r="C129" s="2">
-        <v>953</v>
+        <v>997</v>
       </c>
       <c r="D129" s="2">
-        <v>934</v>
+        <v>978</v>
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -6666,7 +6666,7 @@
       </c>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -6687,7 +6687,7 @@
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -6701,14 +6701,14 @@
         <v>12625</v>
       </c>
       <c r="C132" s="2">
-        <v>3933</v>
+        <v>4071</v>
       </c>
       <c r="D132" s="2">
-        <v>3855</v>
+        <v>3990</v>
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -6729,7 +6729,7 @@
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -6743,14 +6743,14 @@
         <v>113</v>
       </c>
       <c r="C134" s="2">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D134" s="2">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -6785,14 +6785,14 @@
         <v>21978</v>
       </c>
       <c r="C136" s="2">
-        <v>19393</v>
+        <v>19346</v>
       </c>
       <c r="D136" s="2">
-        <v>19006</v>
+        <v>18960</v>
       </c>
       <c r="E136" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -6813,7 +6813,7 @@
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -6827,14 +6827,14 @@
         <v>2436</v>
       </c>
       <c r="C138" s="2">
-        <v>1944</v>
+        <v>1923</v>
       </c>
       <c r="D138" s="2">
-        <v>1906</v>
+        <v>1885</v>
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -6848,14 +6848,14 @@
         <v>12699</v>
       </c>
       <c r="C139" s="2">
-        <v>6226</v>
+        <v>6255</v>
       </c>
       <c r="D139" s="2">
-        <v>6102</v>
+        <v>6130</v>
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -6869,14 +6869,14 @@
         <v>12695</v>
       </c>
       <c r="C140" s="2">
-        <v>12279</v>
+        <v>12212</v>
       </c>
       <c r="D140" s="2">
-        <v>12034</v>
+        <v>11968</v>
       </c>
       <c r="E140" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -6897,7 +6897,7 @@
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -6911,14 +6911,14 @@
         <v>2442</v>
       </c>
       <c r="C142" s="2">
-        <v>3229</v>
+        <v>3135</v>
       </c>
       <c r="D142" s="2">
-        <v>3165</v>
+        <v>3073</v>
       </c>
       <c r="E142" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -6939,7 +6939,7 @@
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -6953,14 +6953,14 @@
         <v>3016</v>
       </c>
       <c r="C144" s="2">
-        <v>2549</v>
+        <v>2618</v>
       </c>
       <c r="D144" s="2">
-        <v>2499</v>
+        <v>2566</v>
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -6981,7 +6981,7 @@
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -6995,14 +6995,14 @@
         <v>31602</v>
       </c>
       <c r="C146" s="2">
-        <v>1821</v>
+        <v>1913</v>
       </c>
       <c r="D146" s="2">
-        <v>1785</v>
+        <v>1875</v>
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7023,7 @@
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -7044,7 +7044,7 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -7079,14 +7079,14 @@
         <v>3024</v>
       </c>
       <c r="C150" s="2">
-        <v>10011</v>
+        <v>10010</v>
       </c>
       <c r="D150" s="2">
-        <v>9811</v>
+        <v>9810</v>
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -7107,7 +7107,7 @@
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -7121,14 +7121,14 @@
         <v>2440</v>
       </c>
       <c r="C152" s="2">
-        <v>3051</v>
+        <v>3101</v>
       </c>
       <c r="D152" s="2">
-        <v>2990</v>
+        <v>3039</v>
       </c>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7149,7 @@
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -7163,14 +7163,14 @@
         <v>2448</v>
       </c>
       <c r="C154" s="2">
-        <v>1395</v>
+        <v>1379</v>
       </c>
       <c r="D154" s="2">
-        <v>1368</v>
+        <v>1352</v>
       </c>
       <c r="E154" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -7222,14 +7222,14 @@
         <v>2152</v>
       </c>
       <c r="C157" s="2">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="D157" s="2">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -7243,14 +7243,14 @@
         <v>2998</v>
       </c>
       <c r="C158" s="2">
-        <v>2263</v>
+        <v>2289</v>
       </c>
       <c r="D158" s="2">
-        <v>2218</v>
+        <v>2244</v>
       </c>
       <c r="E158" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -7285,14 +7285,14 @@
         <v>269</v>
       </c>
       <c r="C160" s="2">
-        <v>3697</v>
+        <v>3737</v>
       </c>
       <c r="D160" s="2">
-        <v>3624</v>
+        <v>3663</v>
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -7348,14 +7348,14 @@
         <v>235</v>
       </c>
       <c r="C163" s="2">
-        <v>694</v>
+        <v>699</v>
       </c>
       <c r="D163" s="2">
-        <v>681</v>
+        <v>686</v>
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -7369,14 +7369,14 @@
         <v>22446</v>
       </c>
       <c r="C164" s="2">
-        <v>8539</v>
+        <v>8639</v>
       </c>
       <c r="D164" s="2">
-        <v>8369</v>
+        <v>8467</v>
       </c>
       <c r="E164" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -7390,14 +7390,14 @@
         <v>21622</v>
       </c>
       <c r="C165" s="2">
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="D165" s="2">
-        <v>155</v>
+        <v>162</v>
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -7411,14 +7411,14 @@
         <v>187</v>
       </c>
       <c r="C166" s="2">
-        <v>291</v>
+        <v>285</v>
       </c>
       <c r="D166" s="2">
-        <v>286</v>
+        <v>280</v>
       </c>
       <c r="E166" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7439,7 @@
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -7453,14 +7453,14 @@
         <v>239</v>
       </c>
       <c r="C168" s="2">
-        <v>681</v>
+        <v>675</v>
       </c>
       <c r="D168" s="2">
-        <v>668</v>
+        <v>662</v>
       </c>
       <c r="E168" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -7474,14 +7474,14 @@
         <v>245</v>
       </c>
       <c r="C169" s="2">
-        <v>917</v>
+        <v>924</v>
       </c>
       <c r="D169" s="2">
-        <v>899</v>
+        <v>906</v>
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -7502,7 +7502,7 @@
       </c>
       <c r="E170" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -7516,14 +7516,14 @@
         <v>6049</v>
       </c>
       <c r="C171" s="2">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D171" s="2">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -7537,14 +7537,14 @@
         <v>191</v>
       </c>
       <c r="C172" s="2">
-        <v>543</v>
+        <v>516</v>
       </c>
       <c r="D172" s="2">
-        <v>533</v>
+        <v>506</v>
       </c>
       <c r="E172" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>
@@ -7586,7 +7586,7 @@
       </c>
       <c r="E174" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:33</t>
+          <t xml:space="preserve">2026-09-14 20:38</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
prices: 2026-09-14 20:43 UTC
</commit_message>
<xml_diff>
--- a/docs/herblore_top8.xlsx
+++ b/docs/herblore_top8.xlsx
@@ -97,7 +97,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Last price update: 2026-09-14 20:38 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
+          <t xml:space="preserve">Last price update: 2026-09-14 20:43 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
         </is>
       </c>
     </row>
@@ -3978,7 +3978,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4062,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4146,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -4209,7 +4209,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -4377,7 +4377,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4608,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4713,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -4734,7 +4734,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -4902,7 +4902,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -4923,7 +4923,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -4965,7 +4965,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -5238,7 +5238,7 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5259,7 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -5322,7 +5322,7 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -5406,7 +5406,7 @@
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -5427,7 +5427,7 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5469,7 @@
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -5553,7 +5553,7 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -5574,7 +5574,7 @@
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -5595,7 +5595,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5637,7 @@
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5679,7 @@
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -5763,7 +5763,7 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -5931,7 +5931,7 @@
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -5952,7 +5952,7 @@
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -5973,7 +5973,7 @@
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -5994,7 +5994,7 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -6015,7 +6015,7 @@
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -6057,7 +6057,7 @@
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6120,7 @@
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6141,7 @@
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -6162,7 +6162,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -6225,7 +6225,7 @@
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -6246,7 +6246,7 @@
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6267,7 @@
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6288,7 @@
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6372,7 @@
       </c>
       <c r="E116" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -6393,7 +6393,7 @@
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -6414,7 +6414,7 @@
       </c>
       <c r="E118" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -6456,7 +6456,7 @@
       </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="E121" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="E124" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -6582,7 +6582,7 @@
       </c>
       <c r="E126" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -6666,7 +6666,7 @@
       </c>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -6687,7 +6687,7 @@
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -6729,7 +6729,7 @@
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -6750,7 +6750,7 @@
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -6792,7 +6792,7 @@
       </c>
       <c r="E136" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -6813,7 +6813,7 @@
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -6834,7 +6834,7 @@
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="E140" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -6897,7 +6897,7 @@
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -6918,7 +6918,7 @@
       </c>
       <c r="E142" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -6939,7 +6939,7 @@
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -6960,7 +6960,7 @@
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -6981,7 +6981,7 @@
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -7002,7 +7002,7 @@
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7023,7 @@
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -7044,7 +7044,7 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -7086,7 +7086,7 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -7107,7 +7107,7 @@
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -7128,7 +7128,7 @@
       </c>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7149,7 @@
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -7170,7 +7170,7 @@
       </c>
       <c r="E154" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -7229,7 +7229,7 @@
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="E158" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -7292,7 +7292,7 @@
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -7355,7 +7355,7 @@
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="E164" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -7397,7 +7397,7 @@
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7418,7 @@
       </c>
       <c r="E166" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7439,7 @@
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -7460,7 +7460,7 @@
       </c>
       <c r="E168" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -7481,7 +7481,7 @@
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -7502,7 +7502,7 @@
       </c>
       <c r="E170" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -7523,7 +7523,7 @@
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -7544,7 +7544,7 @@
       </c>
       <c r="E172" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>
@@ -7586,7 +7586,7 @@
       </c>
       <c r="E174" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:38</t>
+          <t xml:space="preserve">2026-09-14 20:43</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
prices: 2026-09-14 20:48 UTC
</commit_message>
<xml_diff>
--- a/docs/herblore_top8.xlsx
+++ b/docs/herblore_top8.xlsx
@@ -97,7 +97,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Last price update: 2026-09-14 20:43 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
+          <t xml:space="preserve">Last price update: 2026-09-14 20:48 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
         </is>
       </c>
     </row>
@@ -3978,7 +3978,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4062,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4146,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -4209,7 +4209,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -4377,7 +4377,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4608,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4713,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -4734,7 +4734,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -4902,7 +4902,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -4923,7 +4923,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -4965,7 +4965,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -5238,7 +5238,7 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5259,7 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -5322,7 +5322,7 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -5406,7 +5406,7 @@
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -5427,7 +5427,7 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5469,7 @@
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -5553,7 +5553,7 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -5574,7 +5574,7 @@
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -5595,7 +5595,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5637,7 @@
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5679,7 @@
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -5763,7 +5763,7 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -5931,7 +5931,7 @@
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -5952,7 +5952,7 @@
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -5973,7 +5973,7 @@
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -5994,7 +5994,7 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -6015,7 +6015,7 @@
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -6057,7 +6057,7 @@
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6120,7 @@
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6141,7 @@
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -6162,7 +6162,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -6225,7 +6225,7 @@
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -6246,7 +6246,7 @@
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6267,7 @@
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6288,7 @@
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6372,7 @@
       </c>
       <c r="E116" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -6393,7 +6393,7 @@
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -6414,7 +6414,7 @@
       </c>
       <c r="E118" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -6456,7 +6456,7 @@
       </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="E121" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="E124" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -6582,7 +6582,7 @@
       </c>
       <c r="E126" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -6666,7 +6666,7 @@
       </c>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -6687,7 +6687,7 @@
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -6729,7 +6729,7 @@
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -6750,7 +6750,7 @@
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -6792,7 +6792,7 @@
       </c>
       <c r="E136" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -6813,7 +6813,7 @@
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -6834,7 +6834,7 @@
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="E140" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -6897,7 +6897,7 @@
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -6918,7 +6918,7 @@
       </c>
       <c r="E142" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -6939,7 +6939,7 @@
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -6960,7 +6960,7 @@
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -6981,7 +6981,7 @@
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -7002,7 +7002,7 @@
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7023,7 @@
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -7044,7 +7044,7 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -7086,7 +7086,7 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -7107,7 +7107,7 @@
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -7128,7 +7128,7 @@
       </c>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7149,7 @@
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -7170,7 +7170,7 @@
       </c>
       <c r="E154" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -7229,7 +7229,7 @@
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="E158" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -7292,7 +7292,7 @@
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -7355,7 +7355,7 @@
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="E164" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -7397,7 +7397,7 @@
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7418,7 @@
       </c>
       <c r="E166" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7439,7 @@
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -7460,7 +7460,7 @@
       </c>
       <c r="E168" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -7481,7 +7481,7 @@
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -7502,7 +7502,7 @@
       </c>
       <c r="E170" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -7523,7 +7523,7 @@
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -7544,7 +7544,7 @@
       </c>
       <c r="E172" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>
@@ -7586,7 +7586,7 @@
       </c>
       <c r="E174" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:43</t>
+          <t xml:space="preserve">2026-09-14 20:48</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
prices: 2026-09-14 20:53 UTC
</commit_message>
<xml_diff>
--- a/docs/herblore_top8.xlsx
+++ b/docs/herblore_top8.xlsx
@@ -97,7 +97,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Last price update: 2026-09-14 20:48 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
+          <t xml:space="preserve">Last price update: 2026-09-14 20:53 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
         </is>
       </c>
     </row>
@@ -3978,7 +3978,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4062,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4146,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -4209,7 +4209,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -4377,7 +4377,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4608,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4713,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -4734,7 +4734,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -4902,7 +4902,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -4923,7 +4923,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -4965,7 +4965,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -5238,7 +5238,7 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5259,7 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -5322,7 +5322,7 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -5406,7 +5406,7 @@
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -5427,7 +5427,7 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5469,7 @@
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -5553,7 +5553,7 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -5574,7 +5574,7 @@
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -5595,7 +5595,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5637,7 @@
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5679,7 @@
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -5763,7 +5763,7 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -5931,7 +5931,7 @@
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -5952,7 +5952,7 @@
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -5973,7 +5973,7 @@
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -5994,7 +5994,7 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -6015,7 +6015,7 @@
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -6057,7 +6057,7 @@
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6120,7 @@
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6141,7 @@
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -6162,7 +6162,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -6225,7 +6225,7 @@
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -6246,7 +6246,7 @@
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6267,7 @@
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6288,7 @@
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6372,7 @@
       </c>
       <c r="E116" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -6393,7 +6393,7 @@
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -6414,7 +6414,7 @@
       </c>
       <c r="E118" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -6456,7 +6456,7 @@
       </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="E121" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="E124" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -6582,7 +6582,7 @@
       </c>
       <c r="E126" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -6666,7 +6666,7 @@
       </c>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -6687,7 +6687,7 @@
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -6729,7 +6729,7 @@
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -6750,7 +6750,7 @@
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -6792,7 +6792,7 @@
       </c>
       <c r="E136" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -6813,7 +6813,7 @@
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -6834,7 +6834,7 @@
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="E140" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -6897,7 +6897,7 @@
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -6918,7 +6918,7 @@
       </c>
       <c r="E142" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -6939,7 +6939,7 @@
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -6960,7 +6960,7 @@
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -6981,7 +6981,7 @@
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -7002,7 +7002,7 @@
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7023,7 @@
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -7044,7 +7044,7 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -7086,7 +7086,7 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -7107,7 +7107,7 @@
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -7128,7 +7128,7 @@
       </c>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7149,7 @@
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -7170,7 +7170,7 @@
       </c>
       <c r="E154" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -7229,7 +7229,7 @@
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="E158" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -7292,7 +7292,7 @@
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -7355,7 +7355,7 @@
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="E164" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -7397,7 +7397,7 @@
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7418,7 @@
       </c>
       <c r="E166" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7439,7 @@
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -7460,7 +7460,7 @@
       </c>
       <c r="E168" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -7481,7 +7481,7 @@
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -7502,7 +7502,7 @@
       </c>
       <c r="E170" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -7523,7 +7523,7 @@
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -7544,7 +7544,7 @@
       </c>
       <c r="E172" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>
@@ -7586,7 +7586,7 @@
       </c>
       <c r="E174" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:48</t>
+          <t xml:space="preserve">2026-09-14 20:53</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
prices: 2026-09-14 20:58 UTC
</commit_message>
<xml_diff>
--- a/docs/herblore_top8.xlsx
+++ b/docs/herblore_top8.xlsx
@@ -97,7 +97,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Last price update: 2026-09-14 20:53 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
+          <t xml:space="preserve">Last price update: 2026-09-14 20:58 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
         </is>
       </c>
     </row>
@@ -3978,7 +3978,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4062,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4146,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -4209,7 +4209,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -4377,7 +4377,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4608,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4713,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -4734,7 +4734,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -4902,7 +4902,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -4923,7 +4923,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -4965,7 +4965,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -5238,7 +5238,7 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5259,7 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -5322,7 +5322,7 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -5406,7 +5406,7 @@
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -5427,7 +5427,7 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5469,7 @@
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -5553,7 +5553,7 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -5574,7 +5574,7 @@
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -5595,7 +5595,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5637,7 @@
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5679,7 @@
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -5763,7 +5763,7 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -5931,7 +5931,7 @@
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -5952,7 +5952,7 @@
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -5973,7 +5973,7 @@
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -5994,7 +5994,7 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -6015,7 +6015,7 @@
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -6057,7 +6057,7 @@
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6120,7 @@
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6141,7 @@
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -6162,7 +6162,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -6225,7 +6225,7 @@
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -6246,7 +6246,7 @@
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6267,7 @@
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6288,7 @@
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6372,7 @@
       </c>
       <c r="E116" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -6393,7 +6393,7 @@
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -6414,7 +6414,7 @@
       </c>
       <c r="E118" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -6456,7 +6456,7 @@
       </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="E121" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="E124" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -6582,7 +6582,7 @@
       </c>
       <c r="E126" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -6666,7 +6666,7 @@
       </c>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -6687,7 +6687,7 @@
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -6729,7 +6729,7 @@
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -6750,7 +6750,7 @@
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -6792,7 +6792,7 @@
       </c>
       <c r="E136" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -6813,7 +6813,7 @@
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -6834,7 +6834,7 @@
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="E140" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -6897,7 +6897,7 @@
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -6918,7 +6918,7 @@
       </c>
       <c r="E142" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -6939,7 +6939,7 @@
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -6960,7 +6960,7 @@
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -6981,7 +6981,7 @@
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -7002,7 +7002,7 @@
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7023,7 @@
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -7044,7 +7044,7 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -7086,7 +7086,7 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -7107,7 +7107,7 @@
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -7128,7 +7128,7 @@
       </c>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7149,7 @@
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -7170,7 +7170,7 @@
       </c>
       <c r="E154" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -7229,7 +7229,7 @@
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="E158" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -7292,7 +7292,7 @@
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -7355,7 +7355,7 @@
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="E164" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -7397,7 +7397,7 @@
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7418,7 @@
       </c>
       <c r="E166" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7439,7 @@
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -7460,7 +7460,7 @@
       </c>
       <c r="E168" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -7481,7 +7481,7 @@
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -7502,7 +7502,7 @@
       </c>
       <c r="E170" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -7523,7 +7523,7 @@
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -7544,7 +7544,7 @@
       </c>
       <c r="E172" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>
@@ -7586,7 +7586,7 @@
       </c>
       <c r="E174" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:53</t>
+          <t xml:space="preserve">2026-09-14 20:58</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
prices: 2026-09-14 21:03 UTC
</commit_message>
<xml_diff>
--- a/docs/herblore_top8.xlsx
+++ b/docs/herblore_top8.xlsx
@@ -97,7 +97,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Last price update: 2026-09-14 20:58 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
+          <t xml:space="preserve">Last price update: 2026-09-14 21:03 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
         </is>
       </c>
     </row>
@@ -3978,7 +3978,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4062,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4146,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -4209,7 +4209,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -4377,7 +4377,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4608,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4713,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -4734,7 +4734,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -4902,7 +4902,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -4923,7 +4923,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -4965,7 +4965,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -5238,7 +5238,7 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5259,7 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -5322,7 +5322,7 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -5406,7 +5406,7 @@
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -5427,7 +5427,7 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5469,7 @@
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -5553,7 +5553,7 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -5574,7 +5574,7 @@
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -5595,7 +5595,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5637,7 @@
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5679,7 @@
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -5763,7 +5763,7 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -5931,7 +5931,7 @@
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -5952,7 +5952,7 @@
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -5973,7 +5973,7 @@
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -5994,7 +5994,7 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -6015,7 +6015,7 @@
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -6057,7 +6057,7 @@
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6120,7 @@
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6141,7 @@
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -6162,7 +6162,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -6225,7 +6225,7 @@
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -6246,7 +6246,7 @@
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6267,7 @@
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6288,7 @@
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6372,7 @@
       </c>
       <c r="E116" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -6393,7 +6393,7 @@
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -6414,7 +6414,7 @@
       </c>
       <c r="E118" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -6456,7 +6456,7 @@
       </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="E121" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="E124" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -6582,7 +6582,7 @@
       </c>
       <c r="E126" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -6666,7 +6666,7 @@
       </c>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -6687,7 +6687,7 @@
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -6729,7 +6729,7 @@
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -6750,7 +6750,7 @@
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -6792,7 +6792,7 @@
       </c>
       <c r="E136" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -6813,7 +6813,7 @@
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -6834,7 +6834,7 @@
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="E140" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -6897,7 +6897,7 @@
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -6918,7 +6918,7 @@
       </c>
       <c r="E142" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -6939,7 +6939,7 @@
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -6960,7 +6960,7 @@
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -6981,7 +6981,7 @@
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -7002,7 +7002,7 @@
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7023,7 @@
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -7044,7 +7044,7 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -7086,7 +7086,7 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -7107,7 +7107,7 @@
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -7128,7 +7128,7 @@
       </c>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7149,7 @@
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -7170,7 +7170,7 @@
       </c>
       <c r="E154" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -7229,7 +7229,7 @@
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="E158" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -7292,7 +7292,7 @@
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -7355,7 +7355,7 @@
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="E164" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -7397,7 +7397,7 @@
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7418,7 @@
       </c>
       <c r="E166" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7439,7 @@
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -7460,7 +7460,7 @@
       </c>
       <c r="E168" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -7481,7 +7481,7 @@
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -7502,7 +7502,7 @@
       </c>
       <c r="E170" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -7523,7 +7523,7 @@
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -7544,7 +7544,7 @@
       </c>
       <c r="E172" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>
@@ -7586,7 +7586,7 @@
       </c>
       <c r="E174" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 20:58</t>
+          <t xml:space="preserve">2026-09-14 21:03</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
prices: 2026-09-14 21:08 UTC
</commit_message>
<xml_diff>
--- a/docs/herblore_top8.xlsx
+++ b/docs/herblore_top8.xlsx
@@ -97,7 +97,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Last price update: 2026-09-14 21:03 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
+          <t xml:space="preserve">Last price update: 2026-09-14 21:08 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
         </is>
       </c>
     </row>
@@ -3978,7 +3978,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4062,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4146,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -4209,7 +4209,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -4377,7 +4377,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4608,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4713,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -4734,7 +4734,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -4902,7 +4902,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -4923,7 +4923,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -4965,7 +4965,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -5238,7 +5238,7 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5259,7 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -5322,7 +5322,7 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -5406,7 +5406,7 @@
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -5427,7 +5427,7 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5469,7 @@
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -5553,7 +5553,7 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -5574,7 +5574,7 @@
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -5595,7 +5595,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5637,7 @@
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5679,7 @@
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -5763,7 +5763,7 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -5931,7 +5931,7 @@
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -5952,7 +5952,7 @@
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -5973,7 +5973,7 @@
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -5994,7 +5994,7 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -6015,7 +6015,7 @@
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -6057,7 +6057,7 @@
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6120,7 @@
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6141,7 @@
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -6162,7 +6162,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -6225,7 +6225,7 @@
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -6246,7 +6246,7 @@
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6267,7 @@
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6288,7 @@
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6372,7 @@
       </c>
       <c r="E116" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -6393,7 +6393,7 @@
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -6414,7 +6414,7 @@
       </c>
       <c r="E118" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -6456,7 +6456,7 @@
       </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="E121" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="E124" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -6582,7 +6582,7 @@
       </c>
       <c r="E126" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -6666,7 +6666,7 @@
       </c>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -6687,7 +6687,7 @@
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -6729,7 +6729,7 @@
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -6750,7 +6750,7 @@
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -6792,7 +6792,7 @@
       </c>
       <c r="E136" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -6813,7 +6813,7 @@
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -6834,7 +6834,7 @@
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="E140" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -6897,7 +6897,7 @@
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -6918,7 +6918,7 @@
       </c>
       <c r="E142" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -6939,7 +6939,7 @@
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -6960,7 +6960,7 @@
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -6981,7 +6981,7 @@
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -7002,7 +7002,7 @@
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7023,7 @@
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -7044,7 +7044,7 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -7086,7 +7086,7 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -7107,7 +7107,7 @@
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -7128,7 +7128,7 @@
       </c>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7149,7 @@
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -7170,7 +7170,7 @@
       </c>
       <c r="E154" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -7229,7 +7229,7 @@
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="E158" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -7292,7 +7292,7 @@
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -7355,7 +7355,7 @@
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="E164" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -7397,7 +7397,7 @@
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7418,7 @@
       </c>
       <c r="E166" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7439,7 @@
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -7460,7 +7460,7 @@
       </c>
       <c r="E168" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -7481,7 +7481,7 @@
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -7502,7 +7502,7 @@
       </c>
       <c r="E170" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -7523,7 +7523,7 @@
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -7544,7 +7544,7 @@
       </c>
       <c r="E172" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>
@@ -7586,7 +7586,7 @@
       </c>
       <c r="E174" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:03</t>
+          <t xml:space="preserve">2026-09-14 21:08</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
prices: 2026-09-14 21:13 UTC
</commit_message>
<xml_diff>
--- a/docs/herblore_top8.xlsx
+++ b/docs/herblore_top8.xlsx
@@ -97,7 +97,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Last price update: 2026-09-14 21:08 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
+          <t xml:space="preserve">Last price update: 2026-09-14 21:13 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
         </is>
       </c>
     </row>
@@ -3978,7 +3978,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4062,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4146,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -4209,7 +4209,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -4377,7 +4377,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4608,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4713,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -4734,7 +4734,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -4902,7 +4902,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -4923,7 +4923,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -4965,7 +4965,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -5238,7 +5238,7 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5259,7 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -5322,7 +5322,7 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -5406,7 +5406,7 @@
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -5427,7 +5427,7 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5469,7 @@
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -5553,7 +5553,7 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -5574,7 +5574,7 @@
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -5595,7 +5595,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5637,7 @@
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5679,7 @@
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -5763,7 +5763,7 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -5931,7 +5931,7 @@
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -5952,7 +5952,7 @@
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -5973,7 +5973,7 @@
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -5994,7 +5994,7 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -6015,7 +6015,7 @@
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -6057,7 +6057,7 @@
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6120,7 @@
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6141,7 @@
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -6162,7 +6162,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -6225,7 +6225,7 @@
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -6246,7 +6246,7 @@
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6267,7 @@
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6288,7 @@
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6372,7 @@
       </c>
       <c r="E116" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -6393,7 +6393,7 @@
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -6414,7 +6414,7 @@
       </c>
       <c r="E118" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -6456,7 +6456,7 @@
       </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="E121" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="E124" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -6582,7 +6582,7 @@
       </c>
       <c r="E126" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -6666,7 +6666,7 @@
       </c>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -6687,7 +6687,7 @@
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -6729,7 +6729,7 @@
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -6750,7 +6750,7 @@
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -6792,7 +6792,7 @@
       </c>
       <c r="E136" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -6813,7 +6813,7 @@
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -6834,7 +6834,7 @@
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="E140" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -6897,7 +6897,7 @@
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -6918,7 +6918,7 @@
       </c>
       <c r="E142" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -6939,7 +6939,7 @@
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -6960,7 +6960,7 @@
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -6981,7 +6981,7 @@
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -7002,7 +7002,7 @@
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7023,7 @@
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -7044,7 +7044,7 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -7086,7 +7086,7 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -7107,7 +7107,7 @@
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -7128,7 +7128,7 @@
       </c>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7149,7 @@
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -7170,7 +7170,7 @@
       </c>
       <c r="E154" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -7229,7 +7229,7 @@
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="E158" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -7292,7 +7292,7 @@
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -7355,7 +7355,7 @@
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="E164" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -7397,7 +7397,7 @@
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7418,7 @@
       </c>
       <c r="E166" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7439,7 @@
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -7460,7 +7460,7 @@
       </c>
       <c r="E168" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -7481,7 +7481,7 @@
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -7502,7 +7502,7 @@
       </c>
       <c r="E170" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -7523,7 +7523,7 @@
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -7544,7 +7544,7 @@
       </c>
       <c r="E172" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>
@@ -7586,7 +7586,7 @@
       </c>
       <c r="E174" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:08</t>
+          <t xml:space="preserve">2026-09-14 21:13</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
prices: 2026-09-14 21:18 UTC
</commit_message>
<xml_diff>
--- a/docs/herblore_top8.xlsx
+++ b/docs/herblore_top8.xlsx
@@ -97,7 +97,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Last price update: 2026-09-14 21:13 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
+          <t xml:space="preserve">Last price update: 2026-09-14 21:18 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
         </is>
       </c>
     </row>
@@ -3978,7 +3978,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4062,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4146,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -4209,7 +4209,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -4377,7 +4377,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4608,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4713,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -4734,7 +4734,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -4902,7 +4902,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -4923,7 +4923,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -4965,7 +4965,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -5238,7 +5238,7 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5259,7 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -5322,7 +5322,7 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -5406,7 +5406,7 @@
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -5427,7 +5427,7 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5469,7 @@
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -5553,7 +5553,7 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -5574,7 +5574,7 @@
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -5595,7 +5595,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5637,7 @@
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5679,7 @@
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -5763,7 +5763,7 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -5931,7 +5931,7 @@
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -5952,7 +5952,7 @@
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -5973,7 +5973,7 @@
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -5994,7 +5994,7 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -6015,7 +6015,7 @@
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -6057,7 +6057,7 @@
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6120,7 @@
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6141,7 @@
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -6162,7 +6162,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -6225,7 +6225,7 @@
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -6246,7 +6246,7 @@
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6267,7 @@
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6288,7 @@
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6372,7 @@
       </c>
       <c r="E116" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -6393,7 +6393,7 @@
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -6414,7 +6414,7 @@
       </c>
       <c r="E118" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -6456,7 +6456,7 @@
       </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="E121" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="E124" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -6582,7 +6582,7 @@
       </c>
       <c r="E126" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -6666,7 +6666,7 @@
       </c>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -6687,7 +6687,7 @@
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -6729,7 +6729,7 @@
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -6750,7 +6750,7 @@
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -6792,7 +6792,7 @@
       </c>
       <c r="E136" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -6813,7 +6813,7 @@
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -6834,7 +6834,7 @@
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="E140" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -6897,7 +6897,7 @@
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -6918,7 +6918,7 @@
       </c>
       <c r="E142" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -6939,7 +6939,7 @@
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -6960,7 +6960,7 @@
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -6981,7 +6981,7 @@
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -7002,7 +7002,7 @@
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7023,7 @@
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -7044,7 +7044,7 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -7086,7 +7086,7 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -7107,7 +7107,7 @@
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -7128,7 +7128,7 @@
       </c>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7149,7 @@
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -7170,7 +7170,7 @@
       </c>
       <c r="E154" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -7229,7 +7229,7 @@
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="E158" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -7292,7 +7292,7 @@
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -7355,7 +7355,7 @@
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="E164" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -7397,7 +7397,7 @@
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7418,7 @@
       </c>
       <c r="E166" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7439,7 @@
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -7460,7 +7460,7 @@
       </c>
       <c r="E168" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -7481,7 +7481,7 @@
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -7502,7 +7502,7 @@
       </c>
       <c r="E170" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -7523,7 +7523,7 @@
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -7544,7 +7544,7 @@
       </c>
       <c r="E172" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>
@@ -7586,7 +7586,7 @@
       </c>
       <c r="E174" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:13</t>
+          <t xml:space="preserve">2026-09-14 21:18</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
prices: 2026-09-14 21:23 UTC
</commit_message>
<xml_diff>
--- a/docs/herblore_top8.xlsx
+++ b/docs/herblore_top8.xlsx
@@ -97,7 +97,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Last price update: 2026-09-14 21:18 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
+          <t xml:space="preserve">Last price update: 2026-09-14 21:23 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
         </is>
       </c>
     </row>
@@ -3978,7 +3978,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4062,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4146,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -4209,7 +4209,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -4377,7 +4377,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4608,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4713,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -4734,7 +4734,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -4902,7 +4902,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -4923,7 +4923,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -4965,7 +4965,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -5238,7 +5238,7 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5259,7 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -5322,7 +5322,7 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -5406,7 +5406,7 @@
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -5427,7 +5427,7 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5469,7 @@
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -5553,7 +5553,7 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -5574,7 +5574,7 @@
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -5595,7 +5595,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5637,7 @@
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5679,7 @@
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -5763,7 +5763,7 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -5931,7 +5931,7 @@
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -5952,7 +5952,7 @@
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -5973,7 +5973,7 @@
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -5994,7 +5994,7 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -6015,7 +6015,7 @@
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -6057,7 +6057,7 @@
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6120,7 @@
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6141,7 @@
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -6162,7 +6162,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -6225,7 +6225,7 @@
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -6246,7 +6246,7 @@
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6267,7 @@
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6288,7 @@
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6372,7 @@
       </c>
       <c r="E116" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -6393,7 +6393,7 @@
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -6414,7 +6414,7 @@
       </c>
       <c r="E118" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -6456,7 +6456,7 @@
       </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="E121" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="E124" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -6582,7 +6582,7 @@
       </c>
       <c r="E126" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -6666,7 +6666,7 @@
       </c>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -6687,7 +6687,7 @@
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -6729,7 +6729,7 @@
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -6750,7 +6750,7 @@
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -6792,7 +6792,7 @@
       </c>
       <c r="E136" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -6813,7 +6813,7 @@
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -6834,7 +6834,7 @@
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="E140" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -6897,7 +6897,7 @@
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -6918,7 +6918,7 @@
       </c>
       <c r="E142" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -6939,7 +6939,7 @@
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -6960,7 +6960,7 @@
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -6981,7 +6981,7 @@
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -7002,7 +7002,7 @@
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7023,7 @@
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -7044,7 +7044,7 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -7086,7 +7086,7 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -7107,7 +7107,7 @@
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -7128,7 +7128,7 @@
       </c>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7149,7 @@
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -7170,7 +7170,7 @@
       </c>
       <c r="E154" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -7229,7 +7229,7 @@
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="E158" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -7292,7 +7292,7 @@
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -7355,7 +7355,7 @@
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="E164" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -7397,7 +7397,7 @@
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7418,7 @@
       </c>
       <c r="E166" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7439,7 @@
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -7460,7 +7460,7 @@
       </c>
       <c r="E168" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -7481,7 +7481,7 @@
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -7502,7 +7502,7 @@
       </c>
       <c r="E170" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -7523,7 +7523,7 @@
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -7544,7 +7544,7 @@
       </c>
       <c r="E172" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>
@@ -7586,7 +7586,7 @@
       </c>
       <c r="E174" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:18</t>
+          <t xml:space="preserve">2026-09-14 21:23</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
prices: 2026-09-14 21:28 UTC
</commit_message>
<xml_diff>
--- a/docs/herblore_top8.xlsx
+++ b/docs/herblore_top8.xlsx
@@ -97,7 +97,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Last price update: 2026-09-14 21:23 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
+          <t xml:space="preserve">Last price update: 2026-09-14 21:28 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
         </is>
       </c>
     </row>
@@ -3978,7 +3978,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4062,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4146,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -4209,7 +4209,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -4377,7 +4377,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4608,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4713,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -4734,7 +4734,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -4902,7 +4902,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -4923,7 +4923,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -4965,7 +4965,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -5238,7 +5238,7 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5259,7 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -5322,7 +5322,7 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -5406,7 +5406,7 @@
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -5427,7 +5427,7 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5469,7 @@
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -5553,7 +5553,7 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -5574,7 +5574,7 @@
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -5595,7 +5595,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5637,7 @@
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5679,7 @@
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -5763,7 +5763,7 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -5931,7 +5931,7 @@
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -5952,7 +5952,7 @@
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -5973,7 +5973,7 @@
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -5994,7 +5994,7 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -6015,7 +6015,7 @@
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -6057,7 +6057,7 @@
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6120,7 @@
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6141,7 @@
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -6162,7 +6162,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -6225,7 +6225,7 @@
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -6246,7 +6246,7 @@
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6267,7 @@
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6288,7 @@
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6372,7 @@
       </c>
       <c r="E116" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -6393,7 +6393,7 @@
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -6414,7 +6414,7 @@
       </c>
       <c r="E118" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -6456,7 +6456,7 @@
       </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="E121" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="E124" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -6582,7 +6582,7 @@
       </c>
       <c r="E126" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -6666,7 +6666,7 @@
       </c>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -6687,7 +6687,7 @@
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -6729,7 +6729,7 @@
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -6750,7 +6750,7 @@
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -6792,7 +6792,7 @@
       </c>
       <c r="E136" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -6813,7 +6813,7 @@
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -6834,7 +6834,7 @@
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="E140" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -6897,7 +6897,7 @@
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -6918,7 +6918,7 @@
       </c>
       <c r="E142" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -6939,7 +6939,7 @@
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -6960,7 +6960,7 @@
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -6981,7 +6981,7 @@
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -7002,7 +7002,7 @@
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7023,7 @@
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -7044,7 +7044,7 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -7086,7 +7086,7 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -7107,7 +7107,7 @@
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -7128,7 +7128,7 @@
       </c>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7149,7 @@
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -7170,7 +7170,7 @@
       </c>
       <c r="E154" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -7229,7 +7229,7 @@
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="E158" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -7292,7 +7292,7 @@
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -7355,7 +7355,7 @@
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="E164" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -7397,7 +7397,7 @@
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7418,7 @@
       </c>
       <c r="E166" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7439,7 @@
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -7460,7 +7460,7 @@
       </c>
       <c r="E168" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -7481,7 +7481,7 @@
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -7502,7 +7502,7 @@
       </c>
       <c r="E170" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -7523,7 +7523,7 @@
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -7544,7 +7544,7 @@
       </c>
       <c r="E172" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>
@@ -7586,7 +7586,7 @@
       </c>
       <c r="E174" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:23</t>
+          <t xml:space="preserve">2026-09-14 21:28</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
prices: 2026-09-14 21:33 UTC
</commit_message>
<xml_diff>
--- a/docs/herblore_top8.xlsx
+++ b/docs/herblore_top8.xlsx
@@ -97,7 +97,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Last price update: 2026-09-14 21:28 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
+          <t xml:space="preserve">Last price update: 2026-09-14 21:33 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
         </is>
       </c>
     </row>
@@ -3978,7 +3978,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4062,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4146,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -4209,7 +4209,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -4377,7 +4377,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4608,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4713,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -4734,7 +4734,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -4902,7 +4902,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -4923,7 +4923,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -4965,7 +4965,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -5238,7 +5238,7 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5259,7 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -5322,7 +5322,7 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -5406,7 +5406,7 @@
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -5427,7 +5427,7 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5469,7 @@
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -5553,7 +5553,7 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -5574,7 +5574,7 @@
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -5595,7 +5595,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5637,7 @@
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5679,7 @@
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -5763,7 +5763,7 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -5931,7 +5931,7 @@
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -5952,7 +5952,7 @@
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -5973,7 +5973,7 @@
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -5994,7 +5994,7 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -6015,7 +6015,7 @@
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -6057,7 +6057,7 @@
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6120,7 @@
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6141,7 @@
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -6162,7 +6162,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -6225,7 +6225,7 @@
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -6246,7 +6246,7 @@
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6267,7 @@
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6288,7 @@
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6372,7 @@
       </c>
       <c r="E116" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -6393,7 +6393,7 @@
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -6414,7 +6414,7 @@
       </c>
       <c r="E118" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -6456,7 +6456,7 @@
       </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="E121" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="E124" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -6582,7 +6582,7 @@
       </c>
       <c r="E126" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -6666,7 +6666,7 @@
       </c>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -6687,7 +6687,7 @@
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -6729,7 +6729,7 @@
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -6750,7 +6750,7 @@
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -6792,7 +6792,7 @@
       </c>
       <c r="E136" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -6813,7 +6813,7 @@
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -6834,7 +6834,7 @@
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="E140" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -6897,7 +6897,7 @@
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -6918,7 +6918,7 @@
       </c>
       <c r="E142" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -6939,7 +6939,7 @@
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -6960,7 +6960,7 @@
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -6981,7 +6981,7 @@
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -7002,7 +7002,7 @@
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7023,7 @@
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -7044,7 +7044,7 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -7086,7 +7086,7 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -7107,7 +7107,7 @@
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -7128,7 +7128,7 @@
       </c>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7149,7 @@
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -7170,7 +7170,7 @@
       </c>
       <c r="E154" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -7229,7 +7229,7 @@
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="E158" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -7292,7 +7292,7 @@
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -7355,7 +7355,7 @@
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="E164" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -7397,7 +7397,7 @@
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7418,7 @@
       </c>
       <c r="E166" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7439,7 @@
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -7460,7 +7460,7 @@
       </c>
       <c r="E168" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -7481,7 +7481,7 @@
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -7502,7 +7502,7 @@
       </c>
       <c r="E170" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -7523,7 +7523,7 @@
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -7544,7 +7544,7 @@
       </c>
       <c r="E172" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>
@@ -7586,7 +7586,7 @@
       </c>
       <c r="E174" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:28</t>
+          <t xml:space="preserve">2026-09-14 21:33</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
prices: 2026-09-14 21:38 UTC
</commit_message>
<xml_diff>
--- a/docs/herblore_top8.xlsx
+++ b/docs/herblore_top8.xlsx
@@ -97,7 +97,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Last price update: 2026-09-14 21:33 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
+          <t xml:space="preserve">Last price update: 2026-09-14 21:38 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
         </is>
       </c>
     </row>
@@ -3978,7 +3978,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4062,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4146,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -4209,7 +4209,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -4377,7 +4377,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4608,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4713,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -4734,7 +4734,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -4902,7 +4902,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -4923,7 +4923,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -4965,7 +4965,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -5238,7 +5238,7 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5259,7 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -5322,7 +5322,7 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -5406,7 +5406,7 @@
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -5427,7 +5427,7 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5469,7 @@
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -5553,7 +5553,7 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -5574,7 +5574,7 @@
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -5595,7 +5595,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5637,7 @@
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5679,7 @@
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -5763,7 +5763,7 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -5931,7 +5931,7 @@
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -5952,7 +5952,7 @@
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -5973,7 +5973,7 @@
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -5994,7 +5994,7 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -6015,7 +6015,7 @@
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -6057,7 +6057,7 @@
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6120,7 @@
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6141,7 @@
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -6162,7 +6162,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -6225,7 +6225,7 @@
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -6246,7 +6246,7 @@
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6267,7 @@
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6288,7 @@
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6372,7 @@
       </c>
       <c r="E116" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -6393,7 +6393,7 @@
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -6414,7 +6414,7 @@
       </c>
       <c r="E118" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -6456,7 +6456,7 @@
       </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="E121" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="E124" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -6582,7 +6582,7 @@
       </c>
       <c r="E126" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -6666,7 +6666,7 @@
       </c>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -6687,7 +6687,7 @@
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -6729,7 +6729,7 @@
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -6750,7 +6750,7 @@
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -6792,7 +6792,7 @@
       </c>
       <c r="E136" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -6813,7 +6813,7 @@
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -6834,7 +6834,7 @@
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="E140" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -6897,7 +6897,7 @@
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -6918,7 +6918,7 @@
       </c>
       <c r="E142" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -6939,7 +6939,7 @@
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -6960,7 +6960,7 @@
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -6981,7 +6981,7 @@
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -7002,7 +7002,7 @@
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7023,7 @@
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -7044,7 +7044,7 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -7086,7 +7086,7 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -7107,7 +7107,7 @@
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -7128,7 +7128,7 @@
       </c>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7149,7 @@
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -7170,7 +7170,7 @@
       </c>
       <c r="E154" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -7229,7 +7229,7 @@
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="E158" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -7292,7 +7292,7 @@
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -7355,7 +7355,7 @@
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="E164" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -7397,7 +7397,7 @@
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7418,7 @@
       </c>
       <c r="E166" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7439,7 @@
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -7460,7 +7460,7 @@
       </c>
       <c r="E168" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -7481,7 +7481,7 @@
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -7502,7 +7502,7 @@
       </c>
       <c r="E170" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -7523,7 +7523,7 @@
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -7544,7 +7544,7 @@
       </c>
       <c r="E172" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>
@@ -7586,7 +7586,7 @@
       </c>
       <c r="E174" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:33</t>
+          <t xml:space="preserve">2026-09-14 21:38</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
prices: 2026-09-14 21:43 UTC
</commit_message>
<xml_diff>
--- a/docs/herblore_top8.xlsx
+++ b/docs/herblore_top8.xlsx
@@ -97,7 +97,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Last price update: 2026-09-14 21:38 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
+          <t xml:space="preserve">Last price update: 2026-09-14 21:43 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
         </is>
       </c>
     </row>
@@ -3978,7 +3978,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4062,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4146,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -4209,7 +4209,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -4377,7 +4377,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4608,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4713,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -4734,7 +4734,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -4902,7 +4902,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -4923,7 +4923,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -4965,7 +4965,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -5238,7 +5238,7 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5259,7 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -5322,7 +5322,7 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -5406,7 +5406,7 @@
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -5427,7 +5427,7 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5469,7 @@
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -5553,7 +5553,7 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -5574,7 +5574,7 @@
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -5595,7 +5595,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5637,7 @@
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5679,7 @@
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -5763,7 +5763,7 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -5931,7 +5931,7 @@
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -5952,7 +5952,7 @@
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -5973,7 +5973,7 @@
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -5994,7 +5994,7 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -6015,7 +6015,7 @@
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -6057,7 +6057,7 @@
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6120,7 @@
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6141,7 @@
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -6162,7 +6162,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -6225,7 +6225,7 @@
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -6246,7 +6246,7 @@
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6267,7 @@
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6288,7 @@
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6372,7 @@
       </c>
       <c r="E116" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -6393,7 +6393,7 @@
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -6414,7 +6414,7 @@
       </c>
       <c r="E118" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -6456,7 +6456,7 @@
       </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="E121" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="E124" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -6582,7 +6582,7 @@
       </c>
       <c r="E126" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -6666,7 +6666,7 @@
       </c>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -6687,7 +6687,7 @@
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -6729,7 +6729,7 @@
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -6750,7 +6750,7 @@
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -6792,7 +6792,7 @@
       </c>
       <c r="E136" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -6813,7 +6813,7 @@
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -6834,7 +6834,7 @@
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="E140" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -6897,7 +6897,7 @@
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -6918,7 +6918,7 @@
       </c>
       <c r="E142" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -6939,7 +6939,7 @@
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -6960,7 +6960,7 @@
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -6981,7 +6981,7 @@
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -7002,7 +7002,7 @@
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7023,7 @@
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -7044,7 +7044,7 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -7086,7 +7086,7 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -7107,7 +7107,7 @@
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -7128,7 +7128,7 @@
       </c>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7149,7 @@
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -7170,7 +7170,7 @@
       </c>
       <c r="E154" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -7229,7 +7229,7 @@
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="E158" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -7292,7 +7292,7 @@
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -7355,7 +7355,7 @@
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="E164" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -7397,7 +7397,7 @@
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7418,7 @@
       </c>
       <c r="E166" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7439,7 @@
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -7460,7 +7460,7 @@
       </c>
       <c r="E168" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -7481,7 +7481,7 @@
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -7502,7 +7502,7 @@
       </c>
       <c r="E170" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -7523,7 +7523,7 @@
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -7544,7 +7544,7 @@
       </c>
       <c r="E172" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>
@@ -7586,7 +7586,7 @@
       </c>
       <c r="E174" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:38</t>
+          <t xml:space="preserve">2026-09-14 21:43</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
prices: 2026-09-14 21:48 UTC
</commit_message>
<xml_diff>
--- a/docs/herblore_top8.xlsx
+++ b/docs/herblore_top8.xlsx
@@ -97,7 +97,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Last price update: 2026-09-14 21:43 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
+          <t xml:space="preserve">Last price update: 2026-09-14 21:48 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
         </is>
       </c>
     </row>
@@ -3978,7 +3978,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4062,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4146,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -4209,7 +4209,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -4377,7 +4377,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4608,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4713,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -4734,7 +4734,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -4902,7 +4902,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -4923,7 +4923,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -4965,7 +4965,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -5238,7 +5238,7 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5259,7 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -5322,7 +5322,7 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -5406,7 +5406,7 @@
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -5427,7 +5427,7 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5469,7 @@
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -5553,7 +5553,7 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -5574,7 +5574,7 @@
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -5595,7 +5595,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5637,7 @@
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5679,7 @@
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -5763,7 +5763,7 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -5931,7 +5931,7 @@
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -5952,7 +5952,7 @@
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -5973,7 +5973,7 @@
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -5994,7 +5994,7 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -6015,7 +6015,7 @@
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -6057,7 +6057,7 @@
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6120,7 @@
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6141,7 @@
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -6162,7 +6162,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -6225,7 +6225,7 @@
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -6246,7 +6246,7 @@
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6267,7 @@
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6288,7 @@
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6372,7 @@
       </c>
       <c r="E116" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -6393,7 +6393,7 @@
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -6414,7 +6414,7 @@
       </c>
       <c r="E118" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -6456,7 +6456,7 @@
       </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="E121" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="E124" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -6582,7 +6582,7 @@
       </c>
       <c r="E126" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -6666,7 +6666,7 @@
       </c>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -6687,7 +6687,7 @@
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -6729,7 +6729,7 @@
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -6750,7 +6750,7 @@
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -6792,7 +6792,7 @@
       </c>
       <c r="E136" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -6813,7 +6813,7 @@
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -6834,7 +6834,7 @@
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="E140" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -6897,7 +6897,7 @@
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -6918,7 +6918,7 @@
       </c>
       <c r="E142" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -6939,7 +6939,7 @@
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -6960,7 +6960,7 @@
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -6981,7 +6981,7 @@
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -7002,7 +7002,7 @@
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7023,7 @@
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -7044,7 +7044,7 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -7086,7 +7086,7 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -7107,7 +7107,7 @@
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -7128,7 +7128,7 @@
       </c>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7149,7 @@
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -7170,7 +7170,7 @@
       </c>
       <c r="E154" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -7229,7 +7229,7 @@
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="E158" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -7292,7 +7292,7 @@
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -7355,7 +7355,7 @@
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="E164" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -7397,7 +7397,7 @@
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7418,7 @@
       </c>
       <c r="E166" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7439,7 @@
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -7460,7 +7460,7 @@
       </c>
       <c r="E168" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -7481,7 +7481,7 @@
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -7502,7 +7502,7 @@
       </c>
       <c r="E170" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -7523,7 +7523,7 @@
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -7544,7 +7544,7 @@
       </c>
       <c r="E172" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>
@@ -7586,7 +7586,7 @@
       </c>
       <c r="E174" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:43</t>
+          <t xml:space="preserve">2026-09-14 21:48</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
prices: 2026-09-14 21:53 UTC
</commit_message>
<xml_diff>
--- a/docs/herblore_top8.xlsx
+++ b/docs/herblore_top8.xlsx
@@ -97,7 +97,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Last price update: 2026-09-14 21:48 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
+          <t xml:space="preserve">Last price update: 2026-09-14 21:53 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
         </is>
       </c>
     </row>
@@ -3978,7 +3978,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4062,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4146,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -4209,7 +4209,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -4377,7 +4377,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4608,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4713,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -4734,7 +4734,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -4902,7 +4902,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -4923,7 +4923,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -4965,7 +4965,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -5238,7 +5238,7 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5259,7 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -5322,7 +5322,7 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -5406,7 +5406,7 @@
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -5427,7 +5427,7 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5469,7 @@
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -5553,7 +5553,7 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -5574,7 +5574,7 @@
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -5595,7 +5595,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5637,7 @@
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5679,7 @@
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -5763,7 +5763,7 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -5931,7 +5931,7 @@
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -5952,7 +5952,7 @@
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -5973,7 +5973,7 @@
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -5994,7 +5994,7 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -6015,7 +6015,7 @@
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -6057,7 +6057,7 @@
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6120,7 @@
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6141,7 @@
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -6162,7 +6162,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -6225,7 +6225,7 @@
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -6246,7 +6246,7 @@
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6267,7 @@
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6288,7 @@
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6372,7 @@
       </c>
       <c r="E116" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -6393,7 +6393,7 @@
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -6414,7 +6414,7 @@
       </c>
       <c r="E118" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -6456,7 +6456,7 @@
       </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="E121" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="E124" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -6582,7 +6582,7 @@
       </c>
       <c r="E126" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -6666,7 +6666,7 @@
       </c>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -6687,7 +6687,7 @@
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -6729,7 +6729,7 @@
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -6750,7 +6750,7 @@
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -6792,7 +6792,7 @@
       </c>
       <c r="E136" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -6813,7 +6813,7 @@
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -6834,7 +6834,7 @@
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="E140" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -6897,7 +6897,7 @@
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -6918,7 +6918,7 @@
       </c>
       <c r="E142" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -6939,7 +6939,7 @@
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -6960,7 +6960,7 @@
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -6981,7 +6981,7 @@
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -7002,7 +7002,7 @@
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7023,7 @@
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -7044,7 +7044,7 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -7086,7 +7086,7 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -7107,7 +7107,7 @@
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -7128,7 +7128,7 @@
       </c>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7149,7 @@
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -7170,7 +7170,7 @@
       </c>
       <c r="E154" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -7229,7 +7229,7 @@
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="E158" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -7292,7 +7292,7 @@
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -7355,7 +7355,7 @@
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="E164" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -7397,7 +7397,7 @@
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7418,7 @@
       </c>
       <c r="E166" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7439,7 @@
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -7460,7 +7460,7 @@
       </c>
       <c r="E168" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -7481,7 +7481,7 @@
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -7502,7 +7502,7 @@
       </c>
       <c r="E170" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -7523,7 +7523,7 @@
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -7544,7 +7544,7 @@
       </c>
       <c r="E172" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>
@@ -7586,7 +7586,7 @@
       </c>
       <c r="E174" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:48</t>
+          <t xml:space="preserve">2026-09-14 21:53</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
prices: 2026-09-14 21:58 UTC
</commit_message>
<xml_diff>
--- a/docs/herblore_top8.xlsx
+++ b/docs/herblore_top8.xlsx
@@ -97,7 +97,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Last price update: 2026-09-14 21:53 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
+          <t xml:space="preserve">Last price update: 2026-09-14 21:58 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
         </is>
       </c>
     </row>
@@ -3978,7 +3978,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4062,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4146,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -4209,7 +4209,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -4377,7 +4377,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4608,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4713,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -4734,7 +4734,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -4902,7 +4902,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -4923,7 +4923,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -4965,7 +4965,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -5238,7 +5238,7 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5259,7 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -5322,7 +5322,7 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -5406,7 +5406,7 @@
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -5427,7 +5427,7 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5469,7 @@
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -5553,7 +5553,7 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -5574,7 +5574,7 @@
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -5595,7 +5595,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5637,7 @@
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5679,7 @@
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -5763,7 +5763,7 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -5931,7 +5931,7 @@
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -5952,7 +5952,7 @@
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -5973,7 +5973,7 @@
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -5994,7 +5994,7 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -6015,7 +6015,7 @@
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -6057,7 +6057,7 @@
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6120,7 @@
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6141,7 @@
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -6162,7 +6162,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -6225,7 +6225,7 @@
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -6246,7 +6246,7 @@
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6267,7 @@
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6288,7 @@
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6372,7 @@
       </c>
       <c r="E116" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -6393,7 +6393,7 @@
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -6414,7 +6414,7 @@
       </c>
       <c r="E118" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -6456,7 +6456,7 @@
       </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="E121" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="E124" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -6582,7 +6582,7 @@
       </c>
       <c r="E126" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -6666,7 +6666,7 @@
       </c>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -6687,7 +6687,7 @@
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -6729,7 +6729,7 @@
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -6750,7 +6750,7 @@
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -6792,7 +6792,7 @@
       </c>
       <c r="E136" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -6813,7 +6813,7 @@
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -6834,7 +6834,7 @@
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="E140" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -6897,7 +6897,7 @@
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -6918,7 +6918,7 @@
       </c>
       <c r="E142" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -6939,7 +6939,7 @@
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -6960,7 +6960,7 @@
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -6981,7 +6981,7 @@
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -7002,7 +7002,7 @@
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7023,7 @@
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -7044,7 +7044,7 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -7086,7 +7086,7 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -7107,7 +7107,7 @@
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -7128,7 +7128,7 @@
       </c>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7149,7 @@
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -7170,7 +7170,7 @@
       </c>
       <c r="E154" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -7229,7 +7229,7 @@
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="E158" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -7292,7 +7292,7 @@
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -7355,7 +7355,7 @@
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="E164" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -7397,7 +7397,7 @@
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7418,7 @@
       </c>
       <c r="E166" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7439,7 @@
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -7460,7 +7460,7 @@
       </c>
       <c r="E168" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -7481,7 +7481,7 @@
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -7502,7 +7502,7 @@
       </c>
       <c r="E170" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -7523,7 +7523,7 @@
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -7544,7 +7544,7 @@
       </c>
       <c r="E172" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>
@@ -7586,7 +7586,7 @@
       </c>
       <c r="E174" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:53</t>
+          <t xml:space="preserve">2026-09-14 21:58</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
prices: 2026-09-14 22:03 UTC
</commit_message>
<xml_diff>
--- a/docs/herblore_top8.xlsx
+++ b/docs/herblore_top8.xlsx
@@ -97,7 +97,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Last price update: 2026-09-14 21:58 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
+          <t xml:space="preserve">Last price update: 2026-09-14 22:03 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
         </is>
       </c>
     </row>
@@ -3978,7 +3978,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4062,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4146,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -4209,7 +4209,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -4377,7 +4377,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4608,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4713,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -4734,7 +4734,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -4902,7 +4902,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -4923,7 +4923,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -4965,7 +4965,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -5238,7 +5238,7 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5259,7 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -5322,7 +5322,7 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -5406,7 +5406,7 @@
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -5427,7 +5427,7 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5469,7 @@
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -5553,7 +5553,7 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -5574,7 +5574,7 @@
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -5595,7 +5595,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5637,7 @@
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5679,7 @@
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -5763,7 +5763,7 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -5931,7 +5931,7 @@
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -5952,7 +5952,7 @@
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -5973,7 +5973,7 @@
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -5994,7 +5994,7 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -6015,7 +6015,7 @@
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -6057,7 +6057,7 @@
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6120,7 @@
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6141,7 @@
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -6162,7 +6162,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -6225,7 +6225,7 @@
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -6246,7 +6246,7 @@
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6267,7 @@
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6288,7 @@
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6372,7 @@
       </c>
       <c r="E116" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -6393,7 +6393,7 @@
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -6414,7 +6414,7 @@
       </c>
       <c r="E118" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -6456,7 +6456,7 @@
       </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="E121" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="E124" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -6582,7 +6582,7 @@
       </c>
       <c r="E126" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -6666,7 +6666,7 @@
       </c>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -6687,7 +6687,7 @@
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -6729,7 +6729,7 @@
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -6750,7 +6750,7 @@
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -6792,7 +6792,7 @@
       </c>
       <c r="E136" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -6813,7 +6813,7 @@
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -6834,7 +6834,7 @@
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="E140" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -6897,7 +6897,7 @@
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -6918,7 +6918,7 @@
       </c>
       <c r="E142" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -6939,7 +6939,7 @@
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -6960,7 +6960,7 @@
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -6981,7 +6981,7 @@
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -7002,7 +7002,7 @@
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7023,7 @@
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -7044,7 +7044,7 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -7086,7 +7086,7 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -7107,7 +7107,7 @@
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -7128,7 +7128,7 @@
       </c>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7149,7 @@
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -7170,7 +7170,7 @@
       </c>
       <c r="E154" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -7229,7 +7229,7 @@
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="E158" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -7292,7 +7292,7 @@
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -7355,7 +7355,7 @@
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="E164" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -7397,7 +7397,7 @@
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7418,7 @@
       </c>
       <c r="E166" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7439,7 @@
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -7460,7 +7460,7 @@
       </c>
       <c r="E168" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -7481,7 +7481,7 @@
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -7502,7 +7502,7 @@
       </c>
       <c r="E170" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -7523,7 +7523,7 @@
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -7544,7 +7544,7 @@
       </c>
       <c r="E172" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>
@@ -7586,7 +7586,7 @@
       </c>
       <c r="E174" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 21:58</t>
+          <t xml:space="preserve">2026-09-14 22:03</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
prices: 2026-09-14 22:08 UTC
</commit_message>
<xml_diff>
--- a/docs/herblore_top8.xlsx
+++ b/docs/herblore_top8.xlsx
@@ -97,7 +97,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Last price update: 2026-09-14 22:03 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
+          <t xml:space="preserve">Last price update: 2026-09-14 22:08 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
         </is>
       </c>
     </row>
@@ -3978,7 +3978,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4062,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4146,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -4209,7 +4209,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -4377,7 +4377,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4608,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4713,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -4734,7 +4734,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -4902,7 +4902,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -4923,7 +4923,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -4965,7 +4965,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -5238,7 +5238,7 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5259,7 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -5322,7 +5322,7 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -5406,7 +5406,7 @@
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -5427,7 +5427,7 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5469,7 @@
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -5553,7 +5553,7 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -5574,7 +5574,7 @@
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -5595,7 +5595,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5637,7 @@
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5679,7 @@
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -5763,7 +5763,7 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -5931,7 +5931,7 @@
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -5952,7 +5952,7 @@
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -5973,7 +5973,7 @@
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -5994,7 +5994,7 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -6015,7 +6015,7 @@
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -6057,7 +6057,7 @@
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6120,7 @@
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6141,7 @@
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -6162,7 +6162,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -6225,7 +6225,7 @@
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -6246,7 +6246,7 @@
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6267,7 @@
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6288,7 @@
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6372,7 @@
       </c>
       <c r="E116" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -6393,7 +6393,7 @@
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -6414,7 +6414,7 @@
       </c>
       <c r="E118" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -6456,7 +6456,7 @@
       </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="E121" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="E124" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -6582,7 +6582,7 @@
       </c>
       <c r="E126" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -6666,7 +6666,7 @@
       </c>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -6687,7 +6687,7 @@
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -6729,7 +6729,7 @@
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -6750,7 +6750,7 @@
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -6792,7 +6792,7 @@
       </c>
       <c r="E136" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -6813,7 +6813,7 @@
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -6834,7 +6834,7 @@
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="E140" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -6897,7 +6897,7 @@
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -6918,7 +6918,7 @@
       </c>
       <c r="E142" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -6939,7 +6939,7 @@
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -6960,7 +6960,7 @@
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -6981,7 +6981,7 @@
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -7002,7 +7002,7 @@
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7023,7 @@
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -7044,7 +7044,7 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -7086,7 +7086,7 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -7107,7 +7107,7 @@
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -7128,7 +7128,7 @@
       </c>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7149,7 @@
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -7170,7 +7170,7 @@
       </c>
       <c r="E154" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -7229,7 +7229,7 @@
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="E158" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -7292,7 +7292,7 @@
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -7355,7 +7355,7 @@
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="E164" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -7397,7 +7397,7 @@
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7418,7 @@
       </c>
       <c r="E166" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7439,7 @@
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -7460,7 +7460,7 @@
       </c>
       <c r="E168" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -7481,7 +7481,7 @@
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -7502,7 +7502,7 @@
       </c>
       <c r="E170" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -7523,7 +7523,7 @@
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -7544,7 +7544,7 @@
       </c>
       <c r="E172" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>
@@ -7586,7 +7586,7 @@
       </c>
       <c r="E174" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:03</t>
+          <t xml:space="preserve">2026-09-14 22:08</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
prices: 2026-09-14 22:13 UTC
</commit_message>
<xml_diff>
--- a/docs/herblore_top8.xlsx
+++ b/docs/herblore_top8.xlsx
@@ -97,7 +97,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Last price update: 2026-09-14 22:08 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
+          <t xml:space="preserve">Last price update: 2026-09-14 22:13 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
         </is>
       </c>
     </row>
@@ -3978,7 +3978,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4062,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4146,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -4209,7 +4209,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -4377,7 +4377,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4608,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4713,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -4734,7 +4734,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -4902,7 +4902,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -4923,7 +4923,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -4965,7 +4965,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -5238,7 +5238,7 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5259,7 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -5322,7 +5322,7 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -5406,7 +5406,7 @@
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -5427,7 +5427,7 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5469,7 @@
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -5553,7 +5553,7 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -5574,7 +5574,7 @@
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -5595,7 +5595,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5637,7 @@
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5679,7 @@
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -5763,7 +5763,7 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -5931,7 +5931,7 @@
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -5952,7 +5952,7 @@
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -5973,7 +5973,7 @@
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -5994,7 +5994,7 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -6015,7 +6015,7 @@
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -6057,7 +6057,7 @@
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6120,7 @@
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6141,7 @@
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -6162,7 +6162,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -6225,7 +6225,7 @@
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -6246,7 +6246,7 @@
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6267,7 @@
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6288,7 @@
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6372,7 @@
       </c>
       <c r="E116" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -6393,7 +6393,7 @@
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -6414,7 +6414,7 @@
       </c>
       <c r="E118" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -6456,7 +6456,7 @@
       </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="E121" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="E124" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -6582,7 +6582,7 @@
       </c>
       <c r="E126" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -6666,7 +6666,7 @@
       </c>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -6687,7 +6687,7 @@
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -6729,7 +6729,7 @@
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -6750,7 +6750,7 @@
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -6792,7 +6792,7 @@
       </c>
       <c r="E136" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -6813,7 +6813,7 @@
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -6834,7 +6834,7 @@
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="E140" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -6897,7 +6897,7 @@
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -6918,7 +6918,7 @@
       </c>
       <c r="E142" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -6939,7 +6939,7 @@
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -6960,7 +6960,7 @@
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -6981,7 +6981,7 @@
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -7002,7 +7002,7 @@
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7023,7 @@
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -7044,7 +7044,7 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -7086,7 +7086,7 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -7107,7 +7107,7 @@
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -7128,7 +7128,7 @@
       </c>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7149,7 @@
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -7170,7 +7170,7 @@
       </c>
       <c r="E154" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -7229,7 +7229,7 @@
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="E158" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -7292,7 +7292,7 @@
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -7355,7 +7355,7 @@
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="E164" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -7397,7 +7397,7 @@
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7418,7 @@
       </c>
       <c r="E166" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7439,7 @@
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -7460,7 +7460,7 @@
       </c>
       <c r="E168" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -7481,7 +7481,7 @@
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -7502,7 +7502,7 @@
       </c>
       <c r="E170" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -7523,7 +7523,7 @@
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -7544,7 +7544,7 @@
       </c>
       <c r="E172" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>
@@ -7586,7 +7586,7 @@
       </c>
       <c r="E174" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:08</t>
+          <t xml:space="preserve">2026-09-14 22:13</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
prices: 2026-09-14 22:18 UTC
</commit_message>
<xml_diff>
--- a/docs/herblore_top8.xlsx
+++ b/docs/herblore_top8.xlsx
@@ -97,7 +97,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Last price update: 2026-09-14 22:13 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
+          <t xml:space="preserve">Last price update: 2026-09-14 22:18 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
         </is>
       </c>
     </row>
@@ -3978,7 +3978,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4062,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4146,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -4209,7 +4209,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -4377,7 +4377,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4608,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4713,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -4734,7 +4734,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -4902,7 +4902,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -4923,7 +4923,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -4965,7 +4965,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -5238,7 +5238,7 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5259,7 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -5322,7 +5322,7 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -5406,7 +5406,7 @@
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -5427,7 +5427,7 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5469,7 @@
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -5553,7 +5553,7 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -5574,7 +5574,7 @@
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -5595,7 +5595,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5637,7 @@
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5679,7 @@
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -5763,7 +5763,7 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -5931,7 +5931,7 @@
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -5952,7 +5952,7 @@
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -5973,7 +5973,7 @@
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -5994,7 +5994,7 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -6015,7 +6015,7 @@
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -6057,7 +6057,7 @@
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6120,7 @@
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6141,7 @@
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -6162,7 +6162,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -6225,7 +6225,7 @@
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -6246,7 +6246,7 @@
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6267,7 @@
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6288,7 @@
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6372,7 @@
       </c>
       <c r="E116" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -6393,7 +6393,7 @@
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -6414,7 +6414,7 @@
       </c>
       <c r="E118" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -6456,7 +6456,7 @@
       </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="E121" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="E124" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -6582,7 +6582,7 @@
       </c>
       <c r="E126" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -6666,7 +6666,7 @@
       </c>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -6687,7 +6687,7 @@
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -6729,7 +6729,7 @@
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -6750,7 +6750,7 @@
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -6792,7 +6792,7 @@
       </c>
       <c r="E136" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -6813,7 +6813,7 @@
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -6834,7 +6834,7 @@
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="E140" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -6897,7 +6897,7 @@
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -6918,7 +6918,7 @@
       </c>
       <c r="E142" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -6939,7 +6939,7 @@
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -6960,7 +6960,7 @@
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -6981,7 +6981,7 @@
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -7002,7 +7002,7 @@
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7023,7 @@
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -7044,7 +7044,7 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -7086,7 +7086,7 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -7107,7 +7107,7 @@
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -7128,7 +7128,7 @@
       </c>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7149,7 @@
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -7170,7 +7170,7 @@
       </c>
       <c r="E154" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -7229,7 +7229,7 @@
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="E158" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -7292,7 +7292,7 @@
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -7355,7 +7355,7 @@
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="E164" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -7397,7 +7397,7 @@
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7418,7 @@
       </c>
       <c r="E166" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7439,7 @@
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -7460,7 +7460,7 @@
       </c>
       <c r="E168" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -7481,7 +7481,7 @@
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -7502,7 +7502,7 @@
       </c>
       <c r="E170" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -7523,7 +7523,7 @@
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -7544,7 +7544,7 @@
       </c>
       <c r="E172" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>
@@ -7586,7 +7586,7 @@
       </c>
       <c r="E174" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:13</t>
+          <t xml:space="preserve">2026-09-14 22:18</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
prices: 2026-09-14 22:23 UTC
</commit_message>
<xml_diff>
--- a/docs/herblore_top8.xlsx
+++ b/docs/herblore_top8.xlsx
@@ -97,7 +97,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Last price update: 2026-09-14 22:18 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
+          <t xml:space="preserve">Last price update: 2026-09-14 22:23 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
         </is>
       </c>
     </row>
@@ -3978,7 +3978,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4062,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4146,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -4209,7 +4209,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -4377,7 +4377,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4608,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4713,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -4734,7 +4734,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -4902,7 +4902,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -4923,7 +4923,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -4965,7 +4965,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -5238,7 +5238,7 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5259,7 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -5322,7 +5322,7 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -5406,7 +5406,7 @@
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -5427,7 +5427,7 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5469,7 @@
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -5553,7 +5553,7 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -5574,7 +5574,7 @@
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -5595,7 +5595,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5637,7 @@
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5679,7 @@
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -5763,7 +5763,7 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -5931,7 +5931,7 @@
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -5952,7 +5952,7 @@
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -5973,7 +5973,7 @@
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -5994,7 +5994,7 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -6015,7 +6015,7 @@
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -6057,7 +6057,7 @@
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6120,7 @@
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6141,7 @@
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -6162,7 +6162,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -6225,7 +6225,7 @@
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -6246,7 +6246,7 @@
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6267,7 @@
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6288,7 @@
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6372,7 @@
       </c>
       <c r="E116" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -6393,7 +6393,7 @@
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -6414,7 +6414,7 @@
       </c>
       <c r="E118" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -6456,7 +6456,7 @@
       </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="E121" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="E124" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -6582,7 +6582,7 @@
       </c>
       <c r="E126" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -6666,7 +6666,7 @@
       </c>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -6687,7 +6687,7 @@
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -6729,7 +6729,7 @@
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -6750,7 +6750,7 @@
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -6792,7 +6792,7 @@
       </c>
       <c r="E136" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -6813,7 +6813,7 @@
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -6834,7 +6834,7 @@
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="E140" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -6897,7 +6897,7 @@
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -6918,7 +6918,7 @@
       </c>
       <c r="E142" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -6939,7 +6939,7 @@
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -6960,7 +6960,7 @@
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -6981,7 +6981,7 @@
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -7002,7 +7002,7 @@
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7023,7 @@
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -7044,7 +7044,7 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -7086,7 +7086,7 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -7107,7 +7107,7 @@
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -7128,7 +7128,7 @@
       </c>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7149,7 @@
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -7170,7 +7170,7 @@
       </c>
       <c r="E154" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -7229,7 +7229,7 @@
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="E158" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -7292,7 +7292,7 @@
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -7355,7 +7355,7 @@
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="E164" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -7397,7 +7397,7 @@
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7418,7 @@
       </c>
       <c r="E166" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7439,7 @@
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -7460,7 +7460,7 @@
       </c>
       <c r="E168" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -7481,7 +7481,7 @@
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -7502,7 +7502,7 @@
       </c>
       <c r="E170" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -7523,7 +7523,7 @@
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -7544,7 +7544,7 @@
       </c>
       <c r="E172" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>
@@ -7586,7 +7586,7 @@
       </c>
       <c r="E174" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:18</t>
+          <t xml:space="preserve">2026-09-14 22:23</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
prices: 2026-09-14 22:28 UTC
</commit_message>
<xml_diff>
--- a/docs/herblore_top8.xlsx
+++ b/docs/herblore_top8.xlsx
@@ -97,7 +97,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Last price update: 2026-09-14 22:23 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
+          <t xml:space="preserve">Last price update: 2026-09-14 22:28 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
         </is>
       </c>
     </row>
@@ -3978,7 +3978,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4062,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4146,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -4209,7 +4209,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -4377,7 +4377,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4608,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4713,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -4734,7 +4734,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -4902,7 +4902,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -4923,7 +4923,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -4965,7 +4965,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -5238,7 +5238,7 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5259,7 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -5322,7 +5322,7 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -5406,7 +5406,7 @@
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -5427,7 +5427,7 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5469,7 @@
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -5553,7 +5553,7 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -5574,7 +5574,7 @@
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -5595,7 +5595,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5637,7 @@
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5679,7 @@
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -5763,7 +5763,7 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -5931,7 +5931,7 @@
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -5952,7 +5952,7 @@
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -5973,7 +5973,7 @@
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -5994,7 +5994,7 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -6015,7 +6015,7 @@
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -6057,7 +6057,7 @@
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6120,7 @@
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6141,7 @@
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -6162,7 +6162,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -6225,7 +6225,7 @@
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -6246,7 +6246,7 @@
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6267,7 @@
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6288,7 @@
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6372,7 @@
       </c>
       <c r="E116" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -6393,7 +6393,7 @@
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -6414,7 +6414,7 @@
       </c>
       <c r="E118" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -6456,7 +6456,7 @@
       </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="E121" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="E124" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -6582,7 +6582,7 @@
       </c>
       <c r="E126" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -6666,7 +6666,7 @@
       </c>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -6687,7 +6687,7 @@
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -6729,7 +6729,7 @@
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -6750,7 +6750,7 @@
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -6792,7 +6792,7 @@
       </c>
       <c r="E136" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -6813,7 +6813,7 @@
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -6834,7 +6834,7 @@
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="E140" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -6897,7 +6897,7 @@
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -6918,7 +6918,7 @@
       </c>
       <c r="E142" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -6939,7 +6939,7 @@
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -6960,7 +6960,7 @@
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -6981,7 +6981,7 @@
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -7002,7 +7002,7 @@
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7023,7 @@
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -7044,7 +7044,7 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -7086,7 +7086,7 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -7107,7 +7107,7 @@
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -7128,7 +7128,7 @@
       </c>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7149,7 @@
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -7170,7 +7170,7 @@
       </c>
       <c r="E154" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -7229,7 +7229,7 @@
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="E158" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -7292,7 +7292,7 @@
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -7355,7 +7355,7 @@
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="E164" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -7397,7 +7397,7 @@
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7418,7 @@
       </c>
       <c r="E166" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7439,7 @@
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -7460,7 +7460,7 @@
       </c>
       <c r="E168" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -7481,7 +7481,7 @@
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -7502,7 +7502,7 @@
       </c>
       <c r="E170" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -7523,7 +7523,7 @@
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -7544,7 +7544,7 @@
       </c>
       <c r="E172" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>
@@ -7586,7 +7586,7 @@
       </c>
       <c r="E174" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:23</t>
+          <t xml:space="preserve">2026-09-14 22:28</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
prices: 2026-09-14 22:33 UTC
</commit_message>
<xml_diff>
--- a/docs/herblore_top8.xlsx
+++ b/docs/herblore_top8.xlsx
@@ -97,7 +97,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Last price update: 2026-09-14 22:28 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
+          <t xml:space="preserve">Last price update: 2026-09-14 22:33 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
         </is>
       </c>
     </row>
@@ -3978,7 +3978,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4062,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4146,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -4209,7 +4209,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -4377,7 +4377,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4608,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4713,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -4734,7 +4734,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -4902,7 +4902,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -4923,7 +4923,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -4965,7 +4965,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -5238,7 +5238,7 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5259,7 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -5322,7 +5322,7 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -5406,7 +5406,7 @@
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -5427,7 +5427,7 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5469,7 @@
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -5553,7 +5553,7 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -5574,7 +5574,7 @@
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -5595,7 +5595,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5637,7 @@
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5679,7 @@
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -5763,7 +5763,7 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -5931,7 +5931,7 @@
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -5952,7 +5952,7 @@
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -5973,7 +5973,7 @@
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -5994,7 +5994,7 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -6015,7 +6015,7 @@
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -6057,7 +6057,7 @@
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6120,7 @@
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6141,7 @@
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -6162,7 +6162,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -6225,7 +6225,7 @@
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -6246,7 +6246,7 @@
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6267,7 @@
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6288,7 @@
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6372,7 @@
       </c>
       <c r="E116" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -6393,7 +6393,7 @@
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -6414,7 +6414,7 @@
       </c>
       <c r="E118" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -6456,7 +6456,7 @@
       </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="E121" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="E124" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -6582,7 +6582,7 @@
       </c>
       <c r="E126" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -6666,7 +6666,7 @@
       </c>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -6687,7 +6687,7 @@
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -6729,7 +6729,7 @@
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -6750,7 +6750,7 @@
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -6792,7 +6792,7 @@
       </c>
       <c r="E136" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -6813,7 +6813,7 @@
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -6834,7 +6834,7 @@
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="E140" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -6897,7 +6897,7 @@
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -6918,7 +6918,7 @@
       </c>
       <c r="E142" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -6939,7 +6939,7 @@
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -6960,7 +6960,7 @@
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -6981,7 +6981,7 @@
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -7002,7 +7002,7 @@
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7023,7 @@
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -7044,7 +7044,7 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -7086,7 +7086,7 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -7107,7 +7107,7 @@
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -7128,7 +7128,7 @@
       </c>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7149,7 @@
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -7170,7 +7170,7 @@
       </c>
       <c r="E154" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -7229,7 +7229,7 @@
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="E158" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -7292,7 +7292,7 @@
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -7355,7 +7355,7 @@
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="E164" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -7397,7 +7397,7 @@
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7418,7 @@
       </c>
       <c r="E166" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7439,7 @@
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -7460,7 +7460,7 @@
       </c>
       <c r="E168" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -7481,7 +7481,7 @@
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -7502,7 +7502,7 @@
       </c>
       <c r="E170" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -7523,7 +7523,7 @@
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -7544,7 +7544,7 @@
       </c>
       <c r="E172" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>
@@ -7586,7 +7586,7 @@
       </c>
       <c r="E174" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:28</t>
+          <t xml:space="preserve">2026-09-14 22:33</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
prices: 2026-09-14 22:38 UTC
</commit_message>
<xml_diff>
--- a/docs/herblore_top8.xlsx
+++ b/docs/herblore_top8.xlsx
@@ -97,7 +97,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Last price update: 2026-09-14 22:33 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
+          <t xml:space="preserve">Last price update: 2026-09-14 22:38 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
         </is>
       </c>
     </row>
@@ -3978,7 +3978,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4062,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4146,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -4209,7 +4209,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -4377,7 +4377,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4608,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4713,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -4734,7 +4734,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -4902,7 +4902,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -4923,7 +4923,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -4965,7 +4965,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -5238,7 +5238,7 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5259,7 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -5322,7 +5322,7 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -5406,7 +5406,7 @@
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -5427,7 +5427,7 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5469,7 @@
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -5553,7 +5553,7 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -5574,7 +5574,7 @@
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -5595,7 +5595,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5637,7 @@
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5679,7 @@
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -5763,7 +5763,7 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -5931,7 +5931,7 @@
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -5952,7 +5952,7 @@
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -5973,7 +5973,7 @@
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -5994,7 +5994,7 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -6015,7 +6015,7 @@
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -6057,7 +6057,7 @@
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6120,7 @@
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6141,7 @@
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -6162,7 +6162,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -6225,7 +6225,7 @@
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -6246,7 +6246,7 @@
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6267,7 @@
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6288,7 @@
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6372,7 @@
       </c>
       <c r="E116" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -6393,7 +6393,7 @@
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -6414,7 +6414,7 @@
       </c>
       <c r="E118" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -6456,7 +6456,7 @@
       </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="E121" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="E124" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -6582,7 +6582,7 @@
       </c>
       <c r="E126" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -6666,7 +6666,7 @@
       </c>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -6687,7 +6687,7 @@
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -6729,7 +6729,7 @@
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -6750,7 +6750,7 @@
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -6792,7 +6792,7 @@
       </c>
       <c r="E136" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -6813,7 +6813,7 @@
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -6834,7 +6834,7 @@
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="E140" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -6897,7 +6897,7 @@
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -6918,7 +6918,7 @@
       </c>
       <c r="E142" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -6939,7 +6939,7 @@
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -6960,7 +6960,7 @@
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -6981,7 +6981,7 @@
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -7002,7 +7002,7 @@
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7023,7 @@
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -7044,7 +7044,7 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -7086,7 +7086,7 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -7107,7 +7107,7 @@
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -7128,7 +7128,7 @@
       </c>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7149,7 @@
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -7170,7 +7170,7 @@
       </c>
       <c r="E154" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -7229,7 +7229,7 @@
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="E158" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -7292,7 +7292,7 @@
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -7355,7 +7355,7 @@
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="E164" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -7397,7 +7397,7 @@
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7418,7 @@
       </c>
       <c r="E166" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7439,7 @@
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -7460,7 +7460,7 @@
       </c>
       <c r="E168" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -7481,7 +7481,7 @@
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -7502,7 +7502,7 @@
       </c>
       <c r="E170" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -7523,7 +7523,7 @@
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -7544,7 +7544,7 @@
       </c>
       <c r="E172" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>
@@ -7586,7 +7586,7 @@
       </c>
       <c r="E174" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:33</t>
+          <t xml:space="preserve">2026-09-14 22:38</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
prices: 2026-09-14 22:43 UTC
</commit_message>
<xml_diff>
--- a/docs/herblore_top8.xlsx
+++ b/docs/herblore_top8.xlsx
@@ -97,7 +97,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Last price update: 2026-09-14 22:38 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
+          <t xml:space="preserve">Last price update: 2026-09-14 22:43 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
         </is>
       </c>
     </row>
@@ -3978,7 +3978,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4062,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4146,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -4209,7 +4209,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -4377,7 +4377,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4608,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4713,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -4734,7 +4734,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -4902,7 +4902,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -4923,7 +4923,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -4965,7 +4965,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -5238,7 +5238,7 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5259,7 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -5322,7 +5322,7 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -5406,7 +5406,7 @@
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -5427,7 +5427,7 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5469,7 @@
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -5553,7 +5553,7 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -5574,7 +5574,7 @@
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -5595,7 +5595,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5637,7 @@
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5679,7 @@
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -5763,7 +5763,7 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -5931,7 +5931,7 @@
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -5952,7 +5952,7 @@
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -5973,7 +5973,7 @@
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -5994,7 +5994,7 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -6015,7 +6015,7 @@
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -6057,7 +6057,7 @@
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6120,7 @@
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6141,7 @@
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -6162,7 +6162,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -6225,7 +6225,7 @@
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -6246,7 +6246,7 @@
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6267,7 @@
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6288,7 @@
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6372,7 @@
       </c>
       <c r="E116" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -6393,7 +6393,7 @@
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -6414,7 +6414,7 @@
       </c>
       <c r="E118" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -6456,7 +6456,7 @@
       </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="E121" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="E124" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -6582,7 +6582,7 @@
       </c>
       <c r="E126" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -6666,7 +6666,7 @@
       </c>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -6687,7 +6687,7 @@
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -6729,7 +6729,7 @@
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -6750,7 +6750,7 @@
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -6792,7 +6792,7 @@
       </c>
       <c r="E136" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -6813,7 +6813,7 @@
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -6834,7 +6834,7 @@
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="E140" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -6897,7 +6897,7 @@
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -6918,7 +6918,7 @@
       </c>
       <c r="E142" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -6939,7 +6939,7 @@
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -6960,7 +6960,7 @@
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -6981,7 +6981,7 @@
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -7002,7 +7002,7 @@
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7023,7 @@
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -7044,7 +7044,7 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -7086,7 +7086,7 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -7107,7 +7107,7 @@
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -7128,7 +7128,7 @@
       </c>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7149,7 @@
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -7170,7 +7170,7 @@
       </c>
       <c r="E154" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -7229,7 +7229,7 @@
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="E158" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -7292,7 +7292,7 @@
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -7355,7 +7355,7 @@
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="E164" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -7397,7 +7397,7 @@
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7418,7 @@
       </c>
       <c r="E166" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7439,7 @@
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -7460,7 +7460,7 @@
       </c>
       <c r="E168" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -7481,7 +7481,7 @@
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -7502,7 +7502,7 @@
       </c>
       <c r="E170" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -7523,7 +7523,7 @@
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -7544,7 +7544,7 @@
       </c>
       <c r="E172" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>
@@ -7586,7 +7586,7 @@
       </c>
       <c r="E174" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:38</t>
+          <t xml:space="preserve">2026-09-14 22:43</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
prices: 2026-09-14 22:48 UTC
</commit_message>
<xml_diff>
--- a/docs/herblore_top8.xlsx
+++ b/docs/herblore_top8.xlsx
@@ -97,7 +97,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Last price update: 2026-09-14 22:43 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
+          <t xml:space="preserve">Last price update: 2026-09-14 22:48 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
         </is>
       </c>
     </row>
@@ -3978,7 +3978,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4062,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4146,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -4209,7 +4209,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -4377,7 +4377,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4608,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4713,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -4734,7 +4734,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -4902,7 +4902,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -4923,7 +4923,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -4965,7 +4965,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -5238,7 +5238,7 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5259,7 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -5322,7 +5322,7 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -5406,7 +5406,7 @@
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -5427,7 +5427,7 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5469,7 @@
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -5553,7 +5553,7 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -5574,7 +5574,7 @@
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -5595,7 +5595,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5637,7 @@
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5679,7 @@
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -5763,7 +5763,7 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -5931,7 +5931,7 @@
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -5952,7 +5952,7 @@
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -5973,7 +5973,7 @@
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -5994,7 +5994,7 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -6015,7 +6015,7 @@
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -6057,7 +6057,7 @@
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6120,7 @@
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6141,7 @@
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -6162,7 +6162,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -6225,7 +6225,7 @@
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -6246,7 +6246,7 @@
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6267,7 @@
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6288,7 @@
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6372,7 @@
       </c>
       <c r="E116" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -6393,7 +6393,7 @@
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -6414,7 +6414,7 @@
       </c>
       <c r="E118" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -6456,7 +6456,7 @@
       </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="E121" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="E124" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -6582,7 +6582,7 @@
       </c>
       <c r="E126" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -6666,7 +6666,7 @@
       </c>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -6687,7 +6687,7 @@
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -6729,7 +6729,7 @@
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -6750,7 +6750,7 @@
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -6792,7 +6792,7 @@
       </c>
       <c r="E136" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -6813,7 +6813,7 @@
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -6834,7 +6834,7 @@
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="E140" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -6897,7 +6897,7 @@
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -6918,7 +6918,7 @@
       </c>
       <c r="E142" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -6939,7 +6939,7 @@
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -6960,7 +6960,7 @@
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -6981,7 +6981,7 @@
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -7002,7 +7002,7 @@
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7023,7 @@
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -7044,7 +7044,7 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -7086,7 +7086,7 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -7107,7 +7107,7 @@
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -7128,7 +7128,7 @@
       </c>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7149,7 @@
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -7170,7 +7170,7 @@
       </c>
       <c r="E154" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -7229,7 +7229,7 @@
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="E158" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -7292,7 +7292,7 @@
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -7355,7 +7355,7 @@
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="E164" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -7397,7 +7397,7 @@
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7418,7 @@
       </c>
       <c r="E166" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7439,7 @@
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -7460,7 +7460,7 @@
       </c>
       <c r="E168" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -7481,7 +7481,7 @@
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -7502,7 +7502,7 @@
       </c>
       <c r="E170" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -7523,7 +7523,7 @@
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -7544,7 +7544,7 @@
       </c>
       <c r="E172" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>
@@ -7586,7 +7586,7 @@
       </c>
       <c r="E174" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:43</t>
+          <t xml:space="preserve">2026-09-14 22:48</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
prices: 2026-09-14 22:53 UTC
</commit_message>
<xml_diff>
--- a/docs/herblore_top8.xlsx
+++ b/docs/herblore_top8.xlsx
@@ -97,7 +97,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Last price update: 2026-09-14 22:48 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
+          <t xml:space="preserve">Last price update: 2026-09-14 22:53 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
         </is>
       </c>
     </row>
@@ -3978,7 +3978,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4062,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4146,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -4209,7 +4209,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -4377,7 +4377,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4608,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4713,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -4734,7 +4734,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -4902,7 +4902,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -4923,7 +4923,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -4965,7 +4965,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -5238,7 +5238,7 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5259,7 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -5322,7 +5322,7 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -5406,7 +5406,7 @@
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -5427,7 +5427,7 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5469,7 @@
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -5553,7 +5553,7 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -5574,7 +5574,7 @@
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -5595,7 +5595,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5637,7 @@
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5679,7 @@
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -5763,7 +5763,7 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -5931,7 +5931,7 @@
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -5952,7 +5952,7 @@
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -5973,7 +5973,7 @@
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -5994,7 +5994,7 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -6015,7 +6015,7 @@
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -6057,7 +6057,7 @@
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6120,7 @@
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6141,7 @@
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -6162,7 +6162,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -6225,7 +6225,7 @@
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -6246,7 +6246,7 @@
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6267,7 @@
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6288,7 @@
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6372,7 @@
       </c>
       <c r="E116" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -6393,7 +6393,7 @@
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -6414,7 +6414,7 @@
       </c>
       <c r="E118" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -6456,7 +6456,7 @@
       </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="E121" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="E124" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -6582,7 +6582,7 @@
       </c>
       <c r="E126" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -6666,7 +6666,7 @@
       </c>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -6687,7 +6687,7 @@
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -6729,7 +6729,7 @@
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -6750,7 +6750,7 @@
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -6792,7 +6792,7 @@
       </c>
       <c r="E136" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -6813,7 +6813,7 @@
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -6834,7 +6834,7 @@
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="E140" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -6897,7 +6897,7 @@
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -6918,7 +6918,7 @@
       </c>
       <c r="E142" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -6939,7 +6939,7 @@
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -6960,7 +6960,7 @@
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -6981,7 +6981,7 @@
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -7002,7 +7002,7 @@
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7023,7 @@
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -7044,7 +7044,7 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -7086,7 +7086,7 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -7107,7 +7107,7 @@
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -7128,7 +7128,7 @@
       </c>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7149,7 @@
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -7170,7 +7170,7 @@
       </c>
       <c r="E154" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -7229,7 +7229,7 @@
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="E158" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -7292,7 +7292,7 @@
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -7355,7 +7355,7 @@
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="E164" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -7397,7 +7397,7 @@
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7418,7 @@
       </c>
       <c r="E166" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7439,7 @@
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -7460,7 +7460,7 @@
       </c>
       <c r="E168" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -7481,7 +7481,7 @@
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -7502,7 +7502,7 @@
       </c>
       <c r="E170" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -7523,7 +7523,7 @@
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -7544,7 +7544,7 @@
       </c>
       <c r="E172" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>
@@ -7586,7 +7586,7 @@
       </c>
       <c r="E174" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:48</t>
+          <t xml:space="preserve">2026-09-14 22:53</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
prices: 2026-09-14 22:58 UTC
</commit_message>
<xml_diff>
--- a/docs/herblore_top8.xlsx
+++ b/docs/herblore_top8.xlsx
@@ -97,7 +97,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Last price update: 2026-09-14 22:53 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
+          <t xml:space="preserve">Last price update: 2026-09-14 22:58 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
         </is>
       </c>
     </row>
@@ -3978,7 +3978,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4062,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4146,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -4209,7 +4209,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -4377,7 +4377,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4608,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4713,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -4734,7 +4734,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -4902,7 +4902,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -4923,7 +4923,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -4965,7 +4965,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -5238,7 +5238,7 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5259,7 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -5322,7 +5322,7 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -5406,7 +5406,7 @@
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -5427,7 +5427,7 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5469,7 @@
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -5553,7 +5553,7 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -5574,7 +5574,7 @@
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -5595,7 +5595,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5637,7 @@
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5679,7 @@
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -5763,7 +5763,7 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -5931,7 +5931,7 @@
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -5952,7 +5952,7 @@
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -5973,7 +5973,7 @@
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -5994,7 +5994,7 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -6015,7 +6015,7 @@
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -6057,7 +6057,7 @@
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6120,7 @@
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6141,7 @@
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -6162,7 +6162,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -6225,7 +6225,7 @@
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -6246,7 +6246,7 @@
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6267,7 @@
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6288,7 @@
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6372,7 @@
       </c>
       <c r="E116" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -6393,7 +6393,7 @@
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -6414,7 +6414,7 @@
       </c>
       <c r="E118" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -6456,7 +6456,7 @@
       </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="E121" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="E124" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -6582,7 +6582,7 @@
       </c>
       <c r="E126" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -6666,7 +6666,7 @@
       </c>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -6687,7 +6687,7 @@
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -6729,7 +6729,7 @@
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -6750,7 +6750,7 @@
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -6792,7 +6792,7 @@
       </c>
       <c r="E136" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -6813,7 +6813,7 @@
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -6834,7 +6834,7 @@
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="E140" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -6897,7 +6897,7 @@
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -6918,7 +6918,7 @@
       </c>
       <c r="E142" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -6939,7 +6939,7 @@
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -6960,7 +6960,7 @@
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -6981,7 +6981,7 @@
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -7002,7 +7002,7 @@
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7023,7 @@
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -7044,7 +7044,7 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -7086,7 +7086,7 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -7107,7 +7107,7 @@
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -7128,7 +7128,7 @@
       </c>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7149,7 @@
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -7170,7 +7170,7 @@
       </c>
       <c r="E154" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -7229,7 +7229,7 @@
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="E158" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -7292,7 +7292,7 @@
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -7355,7 +7355,7 @@
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="E164" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -7397,7 +7397,7 @@
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7418,7 @@
       </c>
       <c r="E166" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7439,7 @@
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -7460,7 +7460,7 @@
       </c>
       <c r="E168" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -7481,7 +7481,7 @@
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -7502,7 +7502,7 @@
       </c>
       <c r="E170" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -7523,7 +7523,7 @@
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -7544,7 +7544,7 @@
       </c>
       <c r="E172" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>
@@ -7586,7 +7586,7 @@
       </c>
       <c r="E174" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:53</t>
+          <t xml:space="preserve">2026-09-14 22:58</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
prices: 2026-09-14 23:03 UTC
</commit_message>
<xml_diff>
--- a/docs/herblore_top8.xlsx
+++ b/docs/herblore_top8.xlsx
@@ -97,7 +97,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Last price update: 2026-09-14 22:58 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
+          <t xml:space="preserve">Last price update: 2026-09-14 23:03 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
         </is>
       </c>
     </row>
@@ -3978,7 +3978,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4062,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4146,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -4209,7 +4209,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -4377,7 +4377,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4608,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4713,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -4734,7 +4734,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -4902,7 +4902,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -4923,7 +4923,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -4965,7 +4965,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -5238,7 +5238,7 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5259,7 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -5322,7 +5322,7 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -5406,7 +5406,7 @@
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -5427,7 +5427,7 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5469,7 @@
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -5553,7 +5553,7 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -5574,7 +5574,7 @@
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -5595,7 +5595,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5637,7 @@
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5679,7 @@
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -5763,7 +5763,7 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -5931,7 +5931,7 @@
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -5952,7 +5952,7 @@
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -5973,7 +5973,7 @@
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -5994,7 +5994,7 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -6015,7 +6015,7 @@
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -6057,7 +6057,7 @@
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6120,7 @@
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6141,7 @@
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -6162,7 +6162,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -6225,7 +6225,7 @@
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -6246,7 +6246,7 @@
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6267,7 @@
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6288,7 @@
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6372,7 @@
       </c>
       <c r="E116" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -6393,7 +6393,7 @@
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -6414,7 +6414,7 @@
       </c>
       <c r="E118" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -6456,7 +6456,7 @@
       </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="E121" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="E124" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -6582,7 +6582,7 @@
       </c>
       <c r="E126" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -6666,7 +6666,7 @@
       </c>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -6687,7 +6687,7 @@
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -6729,7 +6729,7 @@
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -6750,7 +6750,7 @@
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -6792,7 +6792,7 @@
       </c>
       <c r="E136" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -6813,7 +6813,7 @@
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -6834,7 +6834,7 @@
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="E140" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -6897,7 +6897,7 @@
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -6918,7 +6918,7 @@
       </c>
       <c r="E142" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -6939,7 +6939,7 @@
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -6960,7 +6960,7 @@
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -6981,7 +6981,7 @@
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -7002,7 +7002,7 @@
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7023,7 @@
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -7044,7 +7044,7 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -7086,7 +7086,7 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -7107,7 +7107,7 @@
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -7128,7 +7128,7 @@
       </c>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7149,7 @@
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -7170,7 +7170,7 @@
       </c>
       <c r="E154" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -7229,7 +7229,7 @@
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="E158" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -7292,7 +7292,7 @@
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -7355,7 +7355,7 @@
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="E164" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -7397,7 +7397,7 @@
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7418,7 @@
       </c>
       <c r="E166" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7439,7 @@
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -7460,7 +7460,7 @@
       </c>
       <c r="E168" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -7481,7 +7481,7 @@
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -7502,7 +7502,7 @@
       </c>
       <c r="E170" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -7523,7 +7523,7 @@
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -7544,7 +7544,7 @@
       </c>
       <c r="E172" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>
@@ -7586,7 +7586,7 @@
       </c>
       <c r="E174" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 22:58</t>
+          <t xml:space="preserve">2026-09-14 23:03</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
prices: 2026-09-14 23:08 UTC
</commit_message>
<xml_diff>
--- a/docs/herblore_top8.xlsx
+++ b/docs/herblore_top8.xlsx
@@ -97,7 +97,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Last price update: 2026-09-14 23:03 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
+          <t xml:space="preserve">Last price update: 2026-09-14 23:08 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
         </is>
       </c>
     </row>
@@ -3978,7 +3978,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4062,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4146,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -4209,7 +4209,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -4377,7 +4377,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4608,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4713,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -4734,7 +4734,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -4902,7 +4902,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -4923,7 +4923,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -4965,7 +4965,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -5238,7 +5238,7 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5259,7 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -5322,7 +5322,7 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -5406,7 +5406,7 @@
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -5427,7 +5427,7 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5469,7 @@
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -5553,7 +5553,7 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -5574,7 +5574,7 @@
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -5595,7 +5595,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5637,7 @@
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5679,7 @@
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -5763,7 +5763,7 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -5931,7 +5931,7 @@
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -5952,7 +5952,7 @@
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -5973,7 +5973,7 @@
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -5994,7 +5994,7 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -6015,7 +6015,7 @@
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -6057,7 +6057,7 @@
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6120,7 @@
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6141,7 @@
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -6162,7 +6162,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -6225,7 +6225,7 @@
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -6246,7 +6246,7 @@
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6267,7 @@
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6288,7 @@
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6372,7 @@
       </c>
       <c r="E116" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -6393,7 +6393,7 @@
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -6414,7 +6414,7 @@
       </c>
       <c r="E118" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -6456,7 +6456,7 @@
       </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="E121" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="E124" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -6582,7 +6582,7 @@
       </c>
       <c r="E126" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -6666,7 +6666,7 @@
       </c>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -6687,7 +6687,7 @@
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -6729,7 +6729,7 @@
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -6750,7 +6750,7 @@
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -6792,7 +6792,7 @@
       </c>
       <c r="E136" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -6813,7 +6813,7 @@
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -6834,7 +6834,7 @@
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="E140" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -6897,7 +6897,7 @@
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -6918,7 +6918,7 @@
       </c>
       <c r="E142" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -6939,7 +6939,7 @@
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -6960,7 +6960,7 @@
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -6981,7 +6981,7 @@
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -7002,7 +7002,7 @@
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7023,7 @@
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -7044,7 +7044,7 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -7086,7 +7086,7 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -7107,7 +7107,7 @@
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -7128,7 +7128,7 @@
       </c>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7149,7 @@
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -7170,7 +7170,7 @@
       </c>
       <c r="E154" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -7229,7 +7229,7 @@
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="E158" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -7292,7 +7292,7 @@
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -7355,7 +7355,7 @@
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="E164" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -7397,7 +7397,7 @@
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7418,7 @@
       </c>
       <c r="E166" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7439,7 @@
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -7460,7 +7460,7 @@
       </c>
       <c r="E168" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -7481,7 +7481,7 @@
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -7502,7 +7502,7 @@
       </c>
       <c r="E170" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -7523,7 +7523,7 @@
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -7544,7 +7544,7 @@
       </c>
       <c r="E172" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>
@@ -7586,7 +7586,7 @@
       </c>
       <c r="E174" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:03</t>
+          <t xml:space="preserve">2026-09-14 23:08</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
prices: 2026-09-14 23:13 UTC
</commit_message>
<xml_diff>
--- a/docs/herblore_top8.xlsx
+++ b/docs/herblore_top8.xlsx
@@ -97,7 +97,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Last price update: 2026-09-14 23:08 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
+          <t xml:space="preserve">Last price update: 2026-09-14 23:13 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
         </is>
       </c>
     </row>
@@ -3978,7 +3978,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4062,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4146,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -4209,7 +4209,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -4377,7 +4377,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4608,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4713,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -4734,7 +4734,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -4902,7 +4902,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -4923,7 +4923,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -4965,7 +4965,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -5238,7 +5238,7 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5259,7 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -5322,7 +5322,7 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -5406,7 +5406,7 @@
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -5427,7 +5427,7 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5469,7 @@
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -5553,7 +5553,7 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -5574,7 +5574,7 @@
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -5595,7 +5595,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5637,7 @@
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5679,7 @@
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -5763,7 +5763,7 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -5931,7 +5931,7 @@
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -5952,7 +5952,7 @@
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -5973,7 +5973,7 @@
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -5994,7 +5994,7 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -6015,7 +6015,7 @@
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -6057,7 +6057,7 @@
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6120,7 @@
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6141,7 @@
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -6162,7 +6162,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -6225,7 +6225,7 @@
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -6246,7 +6246,7 @@
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6267,7 @@
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6288,7 @@
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6372,7 @@
       </c>
       <c r="E116" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -6393,7 +6393,7 @@
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -6414,7 +6414,7 @@
       </c>
       <c r="E118" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -6456,7 +6456,7 @@
       </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="E121" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="E124" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -6582,7 +6582,7 @@
       </c>
       <c r="E126" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -6666,7 +6666,7 @@
       </c>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -6687,7 +6687,7 @@
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -6729,7 +6729,7 @@
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -6750,7 +6750,7 @@
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -6792,7 +6792,7 @@
       </c>
       <c r="E136" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -6813,7 +6813,7 @@
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -6834,7 +6834,7 @@
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="E140" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -6897,7 +6897,7 @@
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -6918,7 +6918,7 @@
       </c>
       <c r="E142" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -6939,7 +6939,7 @@
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -6960,7 +6960,7 @@
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -6981,7 +6981,7 @@
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -7002,7 +7002,7 @@
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7023,7 @@
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -7044,7 +7044,7 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -7086,7 +7086,7 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -7107,7 +7107,7 @@
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -7128,7 +7128,7 @@
       </c>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7149,7 @@
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -7170,7 +7170,7 @@
       </c>
       <c r="E154" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -7229,7 +7229,7 @@
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="E158" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -7292,7 +7292,7 @@
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -7355,7 +7355,7 @@
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="E164" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -7397,7 +7397,7 @@
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7418,7 @@
       </c>
       <c r="E166" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7439,7 @@
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -7460,7 +7460,7 @@
       </c>
       <c r="E168" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -7481,7 +7481,7 @@
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -7502,7 +7502,7 @@
       </c>
       <c r="E170" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -7523,7 +7523,7 @@
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -7544,7 +7544,7 @@
       </c>
       <c r="E172" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>
@@ -7586,7 +7586,7 @@
       </c>
       <c r="E174" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:08</t>
+          <t xml:space="preserve">2026-09-14 23:13</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
prices: 2026-09-14 23:18 UTC
</commit_message>
<xml_diff>
--- a/docs/herblore_top8.xlsx
+++ b/docs/herblore_top8.xlsx
@@ -97,7 +97,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Last price update: 2026-09-14 23:13 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
+          <t xml:space="preserve">Last price update: 2026-09-14 23:18 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
         </is>
       </c>
     </row>
@@ -3978,7 +3978,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4062,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4146,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -4209,7 +4209,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -4377,7 +4377,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4608,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4713,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -4734,7 +4734,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -4902,7 +4902,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -4923,7 +4923,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -4965,7 +4965,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -5238,7 +5238,7 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5259,7 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -5322,7 +5322,7 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -5406,7 +5406,7 @@
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -5427,7 +5427,7 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5469,7 @@
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -5553,7 +5553,7 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -5574,7 +5574,7 @@
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -5595,7 +5595,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5637,7 @@
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5679,7 @@
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -5763,7 +5763,7 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -5931,7 +5931,7 @@
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -5952,7 +5952,7 @@
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -5973,7 +5973,7 @@
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -5994,7 +5994,7 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -6015,7 +6015,7 @@
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -6057,7 +6057,7 @@
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6120,7 @@
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6141,7 @@
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -6162,7 +6162,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -6225,7 +6225,7 @@
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -6246,7 +6246,7 @@
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6267,7 @@
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6288,7 @@
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6372,7 @@
       </c>
       <c r="E116" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -6393,7 +6393,7 @@
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -6414,7 +6414,7 @@
       </c>
       <c r="E118" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -6456,7 +6456,7 @@
       </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="E121" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="E124" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -6582,7 +6582,7 @@
       </c>
       <c r="E126" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -6666,7 +6666,7 @@
       </c>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -6687,7 +6687,7 @@
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -6729,7 +6729,7 @@
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -6750,7 +6750,7 @@
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -6792,7 +6792,7 @@
       </c>
       <c r="E136" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -6813,7 +6813,7 @@
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -6834,7 +6834,7 @@
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="E140" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -6897,7 +6897,7 @@
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -6918,7 +6918,7 @@
       </c>
       <c r="E142" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -6939,7 +6939,7 @@
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -6960,7 +6960,7 @@
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -6981,7 +6981,7 @@
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -7002,7 +7002,7 @@
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7023,7 @@
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -7044,7 +7044,7 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -7086,7 +7086,7 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -7107,7 +7107,7 @@
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -7128,7 +7128,7 @@
       </c>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7149,7 @@
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -7170,7 +7170,7 @@
       </c>
       <c r="E154" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -7229,7 +7229,7 @@
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="E158" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -7292,7 +7292,7 @@
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -7355,7 +7355,7 @@
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="E164" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -7397,7 +7397,7 @@
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7418,7 @@
       </c>
       <c r="E166" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7439,7 @@
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -7460,7 +7460,7 @@
       </c>
       <c r="E168" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -7481,7 +7481,7 @@
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -7502,7 +7502,7 @@
       </c>
       <c r="E170" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -7523,7 +7523,7 @@
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -7544,7 +7544,7 @@
       </c>
       <c r="E172" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>
@@ -7586,7 +7586,7 @@
       </c>
       <c r="E174" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:13</t>
+          <t xml:space="preserve">2026-09-14 23:18</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
prices: 2026-09-14 23:23 UTC
</commit_message>
<xml_diff>
--- a/docs/herblore_top8.xlsx
+++ b/docs/herblore_top8.xlsx
@@ -97,7 +97,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Last price update: 2026-09-14 23:18 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
+          <t xml:space="preserve">Last price update: 2026-09-14 23:23 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
         </is>
       </c>
     </row>
@@ -3978,7 +3978,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4062,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4146,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -4209,7 +4209,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -4377,7 +4377,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4608,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4713,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -4734,7 +4734,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -4902,7 +4902,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -4923,7 +4923,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -4965,7 +4965,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -5238,7 +5238,7 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5259,7 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -5322,7 +5322,7 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -5406,7 +5406,7 @@
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -5427,7 +5427,7 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5469,7 @@
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -5553,7 +5553,7 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -5574,7 +5574,7 @@
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -5595,7 +5595,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5637,7 @@
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5679,7 @@
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -5763,7 +5763,7 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -5931,7 +5931,7 @@
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -5952,7 +5952,7 @@
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -5973,7 +5973,7 @@
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -5994,7 +5994,7 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -6015,7 +6015,7 @@
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -6057,7 +6057,7 @@
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6120,7 @@
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6141,7 @@
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -6162,7 +6162,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -6225,7 +6225,7 @@
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -6246,7 +6246,7 @@
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6267,7 @@
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6288,7 @@
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6372,7 @@
       </c>
       <c r="E116" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -6393,7 +6393,7 @@
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -6414,7 +6414,7 @@
       </c>
       <c r="E118" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -6456,7 +6456,7 @@
       </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="E121" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="E124" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -6582,7 +6582,7 @@
       </c>
       <c r="E126" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -6666,7 +6666,7 @@
       </c>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -6687,7 +6687,7 @@
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -6729,7 +6729,7 @@
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -6750,7 +6750,7 @@
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -6792,7 +6792,7 @@
       </c>
       <c r="E136" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -6813,7 +6813,7 @@
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -6834,7 +6834,7 @@
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="E140" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -6897,7 +6897,7 @@
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -6918,7 +6918,7 @@
       </c>
       <c r="E142" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -6939,7 +6939,7 @@
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -6960,7 +6960,7 @@
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -6981,7 +6981,7 @@
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -7002,7 +7002,7 @@
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7023,7 @@
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -7044,7 +7044,7 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -7086,7 +7086,7 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -7107,7 +7107,7 @@
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -7128,7 +7128,7 @@
       </c>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7149,7 @@
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -7170,7 +7170,7 @@
       </c>
       <c r="E154" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -7229,7 +7229,7 @@
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="E158" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -7292,7 +7292,7 @@
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -7355,7 +7355,7 @@
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="E164" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -7397,7 +7397,7 @@
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7418,7 @@
       </c>
       <c r="E166" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7439,7 @@
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -7460,7 +7460,7 @@
       </c>
       <c r="E168" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -7481,7 +7481,7 @@
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -7502,7 +7502,7 @@
       </c>
       <c r="E170" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -7523,7 +7523,7 @@
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -7544,7 +7544,7 @@
       </c>
       <c r="E172" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>
@@ -7586,7 +7586,7 @@
       </c>
       <c r="E174" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:18</t>
+          <t xml:space="preserve">2026-09-14 23:23</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
prices: 2026-09-14 23:28 UTC
</commit_message>
<xml_diff>
--- a/docs/herblore_top8.xlsx
+++ b/docs/herblore_top8.xlsx
@@ -97,7 +97,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Last price update: 2026-09-14 23:23 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
+          <t xml:space="preserve">Last price update: 2026-09-14 23:28 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
         </is>
       </c>
     </row>
@@ -3978,7 +3978,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4062,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4146,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -4209,7 +4209,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -4377,7 +4377,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4608,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4713,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -4734,7 +4734,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -4902,7 +4902,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -4923,7 +4923,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -4965,7 +4965,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -5238,7 +5238,7 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5259,7 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -5322,7 +5322,7 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -5406,7 +5406,7 @@
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -5427,7 +5427,7 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5469,7 @@
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -5553,7 +5553,7 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -5574,7 +5574,7 @@
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -5595,7 +5595,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5637,7 @@
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5679,7 @@
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -5763,7 +5763,7 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -5931,7 +5931,7 @@
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -5952,7 +5952,7 @@
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -5973,7 +5973,7 @@
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -5994,7 +5994,7 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -6015,7 +6015,7 @@
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -6057,7 +6057,7 @@
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6120,7 @@
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6141,7 @@
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -6162,7 +6162,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -6225,7 +6225,7 @@
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -6246,7 +6246,7 @@
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6267,7 @@
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6288,7 @@
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6372,7 @@
       </c>
       <c r="E116" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -6393,7 +6393,7 @@
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -6414,7 +6414,7 @@
       </c>
       <c r="E118" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -6456,7 +6456,7 @@
       </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="E121" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="E124" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -6582,7 +6582,7 @@
       </c>
       <c r="E126" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -6666,7 +6666,7 @@
       </c>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -6687,7 +6687,7 @@
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -6729,7 +6729,7 @@
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -6750,7 +6750,7 @@
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -6792,7 +6792,7 @@
       </c>
       <c r="E136" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -6813,7 +6813,7 @@
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -6834,7 +6834,7 @@
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="E140" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -6897,7 +6897,7 @@
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -6918,7 +6918,7 @@
       </c>
       <c r="E142" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -6939,7 +6939,7 @@
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -6960,7 +6960,7 @@
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -6981,7 +6981,7 @@
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -7002,7 +7002,7 @@
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7023,7 @@
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -7044,7 +7044,7 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -7086,7 +7086,7 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -7107,7 +7107,7 @@
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -7128,7 +7128,7 @@
       </c>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7149,7 @@
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -7170,7 +7170,7 @@
       </c>
       <c r="E154" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -7229,7 +7229,7 @@
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="E158" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -7292,7 +7292,7 @@
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -7355,7 +7355,7 @@
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="E164" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -7397,7 +7397,7 @@
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7418,7 @@
       </c>
       <c r="E166" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7439,7 @@
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -7460,7 +7460,7 @@
       </c>
       <c r="E168" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -7481,7 +7481,7 @@
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -7502,7 +7502,7 @@
       </c>
       <c r="E170" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -7523,7 +7523,7 @@
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -7544,7 +7544,7 @@
       </c>
       <c r="E172" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>
@@ -7586,7 +7586,7 @@
       </c>
       <c r="E174" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:23</t>
+          <t xml:space="preserve">2026-09-14 23:28</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
prices: 2026-09-14 23:33 UTC
</commit_message>
<xml_diff>
--- a/docs/herblore_top8.xlsx
+++ b/docs/herblore_top8.xlsx
@@ -97,7 +97,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Last price update: 2026-09-14 23:28 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
+          <t xml:space="preserve">Last price update: 2026-09-14 23:33 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
         </is>
       </c>
     </row>
@@ -3978,7 +3978,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4062,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4146,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -4209,7 +4209,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -4377,7 +4377,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4608,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4713,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -4734,7 +4734,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -4902,7 +4902,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -4923,7 +4923,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -4965,7 +4965,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -5238,7 +5238,7 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5259,7 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -5322,7 +5322,7 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -5406,7 +5406,7 @@
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -5427,7 +5427,7 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5469,7 @@
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -5553,7 +5553,7 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -5574,7 +5574,7 @@
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -5595,7 +5595,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5637,7 @@
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5679,7 @@
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -5763,7 +5763,7 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -5931,7 +5931,7 @@
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -5952,7 +5952,7 @@
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -5973,7 +5973,7 @@
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -5994,7 +5994,7 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -6015,7 +6015,7 @@
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -6057,7 +6057,7 @@
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6120,7 @@
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6141,7 @@
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -6162,7 +6162,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -6225,7 +6225,7 @@
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -6246,7 +6246,7 @@
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6267,7 @@
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6288,7 @@
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6372,7 @@
       </c>
       <c r="E116" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -6393,7 +6393,7 @@
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -6414,7 +6414,7 @@
       </c>
       <c r="E118" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -6456,7 +6456,7 @@
       </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="E121" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="E124" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -6582,7 +6582,7 @@
       </c>
       <c r="E126" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -6666,7 +6666,7 @@
       </c>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -6687,7 +6687,7 @@
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -6729,7 +6729,7 @@
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -6750,7 +6750,7 @@
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -6792,7 +6792,7 @@
       </c>
       <c r="E136" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -6813,7 +6813,7 @@
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -6834,7 +6834,7 @@
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="E140" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -6897,7 +6897,7 @@
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -6918,7 +6918,7 @@
       </c>
       <c r="E142" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -6939,7 +6939,7 @@
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -6960,7 +6960,7 @@
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -6981,7 +6981,7 @@
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -7002,7 +7002,7 @@
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7023,7 @@
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -7044,7 +7044,7 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -7086,7 +7086,7 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -7107,7 +7107,7 @@
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -7128,7 +7128,7 @@
       </c>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7149,7 @@
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -7170,7 +7170,7 @@
       </c>
       <c r="E154" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -7229,7 +7229,7 @@
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="E158" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -7292,7 +7292,7 @@
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -7355,7 +7355,7 @@
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="E164" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -7397,7 +7397,7 @@
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7418,7 @@
       </c>
       <c r="E166" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7439,7 @@
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -7460,7 +7460,7 @@
       </c>
       <c r="E168" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -7481,7 +7481,7 @@
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -7502,7 +7502,7 @@
       </c>
       <c r="E170" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -7523,7 +7523,7 @@
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -7544,7 +7544,7 @@
       </c>
       <c r="E172" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>
@@ -7586,7 +7586,7 @@
       </c>
       <c r="E174" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:28</t>
+          <t xml:space="preserve">2026-09-14 23:33</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
prices: 2026-09-14 23:38 UTC
</commit_message>
<xml_diff>
--- a/docs/herblore_top8.xlsx
+++ b/docs/herblore_top8.xlsx
@@ -97,7 +97,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Last price update: 2026-09-14 23:33 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
+          <t xml:space="preserve">Last price update: 2026-09-14 23:38 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
         </is>
       </c>
     </row>
@@ -3978,7 +3978,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4062,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4146,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -4209,7 +4209,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -4377,7 +4377,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4608,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4713,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -4734,7 +4734,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -4902,7 +4902,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -4923,7 +4923,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -4965,7 +4965,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -5238,7 +5238,7 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5259,7 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -5322,7 +5322,7 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -5406,7 +5406,7 @@
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -5427,7 +5427,7 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5469,7 @@
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -5553,7 +5553,7 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -5574,7 +5574,7 @@
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -5595,7 +5595,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5637,7 @@
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5679,7 @@
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -5763,7 +5763,7 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -5931,7 +5931,7 @@
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -5952,7 +5952,7 @@
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -5973,7 +5973,7 @@
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -5994,7 +5994,7 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -6015,7 +6015,7 @@
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -6057,7 +6057,7 @@
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6120,7 @@
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6141,7 @@
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -6162,7 +6162,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -6225,7 +6225,7 @@
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -6246,7 +6246,7 @@
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6267,7 @@
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6288,7 @@
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6372,7 @@
       </c>
       <c r="E116" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -6393,7 +6393,7 @@
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -6414,7 +6414,7 @@
       </c>
       <c r="E118" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -6456,7 +6456,7 @@
       </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="E121" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="E124" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -6582,7 +6582,7 @@
       </c>
       <c r="E126" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -6666,7 +6666,7 @@
       </c>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -6687,7 +6687,7 @@
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -6729,7 +6729,7 @@
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -6750,7 +6750,7 @@
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -6792,7 +6792,7 @@
       </c>
       <c r="E136" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -6813,7 +6813,7 @@
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -6834,7 +6834,7 @@
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="E140" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -6897,7 +6897,7 @@
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -6918,7 +6918,7 @@
       </c>
       <c r="E142" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -6939,7 +6939,7 @@
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -6960,7 +6960,7 @@
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -6981,7 +6981,7 @@
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -7002,7 +7002,7 @@
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7023,7 @@
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -7044,7 +7044,7 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -7086,7 +7086,7 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -7107,7 +7107,7 @@
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -7128,7 +7128,7 @@
       </c>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7149,7 @@
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -7170,7 +7170,7 @@
       </c>
       <c r="E154" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -7229,7 +7229,7 @@
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="E158" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -7292,7 +7292,7 @@
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -7355,7 +7355,7 @@
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="E164" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -7397,7 +7397,7 @@
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7418,7 @@
       </c>
       <c r="E166" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7439,7 @@
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -7460,7 +7460,7 @@
       </c>
       <c r="E168" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -7481,7 +7481,7 @@
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -7502,7 +7502,7 @@
       </c>
       <c r="E170" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -7523,7 +7523,7 @@
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -7544,7 +7544,7 @@
       </c>
       <c r="E172" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>
@@ -7586,7 +7586,7 @@
       </c>
       <c r="E174" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:33</t>
+          <t xml:space="preserve">2026-09-14 23:38</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
prices: 2026-09-14 23:43 UTC
</commit_message>
<xml_diff>
--- a/docs/herblore_top8.xlsx
+++ b/docs/herblore_top8.xlsx
@@ -97,7 +97,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Last price update: 2026-09-14 23:38 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
+          <t xml:space="preserve">Last price update: 2026-09-14 23:43 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
         </is>
       </c>
     </row>
@@ -3978,7 +3978,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4062,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4146,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -4209,7 +4209,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -4377,7 +4377,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4608,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4713,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -4734,7 +4734,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -4902,7 +4902,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -4923,7 +4923,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -4965,7 +4965,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -5238,7 +5238,7 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5259,7 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -5322,7 +5322,7 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -5406,7 +5406,7 @@
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -5427,7 +5427,7 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5469,7 @@
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -5553,7 +5553,7 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -5574,7 +5574,7 @@
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -5595,7 +5595,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5637,7 @@
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5679,7 @@
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -5763,7 +5763,7 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -5931,7 +5931,7 @@
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -5952,7 +5952,7 @@
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -5973,7 +5973,7 @@
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -5994,7 +5994,7 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -6015,7 +6015,7 @@
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -6057,7 +6057,7 @@
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6120,7 @@
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6141,7 @@
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -6162,7 +6162,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -6225,7 +6225,7 @@
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -6246,7 +6246,7 @@
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6267,7 @@
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6288,7 @@
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6372,7 @@
       </c>
       <c r="E116" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -6393,7 +6393,7 @@
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -6414,7 +6414,7 @@
       </c>
       <c r="E118" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -6456,7 +6456,7 @@
       </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="E121" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="E124" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -6582,7 +6582,7 @@
       </c>
       <c r="E126" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -6666,7 +6666,7 @@
       </c>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -6687,7 +6687,7 @@
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -6729,7 +6729,7 @@
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -6750,7 +6750,7 @@
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -6792,7 +6792,7 @@
       </c>
       <c r="E136" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -6813,7 +6813,7 @@
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -6834,7 +6834,7 @@
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="E140" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -6897,7 +6897,7 @@
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -6918,7 +6918,7 @@
       </c>
       <c r="E142" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -6939,7 +6939,7 @@
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -6960,7 +6960,7 @@
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -6981,7 +6981,7 @@
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -7002,7 +7002,7 @@
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7023,7 @@
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -7044,7 +7044,7 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -7086,7 +7086,7 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -7107,7 +7107,7 @@
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -7128,7 +7128,7 @@
       </c>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7149,7 @@
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -7170,7 +7170,7 @@
       </c>
       <c r="E154" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -7229,7 +7229,7 @@
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="E158" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -7292,7 +7292,7 @@
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -7355,7 +7355,7 @@
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="E164" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -7397,7 +7397,7 @@
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7418,7 @@
       </c>
       <c r="E166" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7439,7 @@
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -7460,7 +7460,7 @@
       </c>
       <c r="E168" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -7481,7 +7481,7 @@
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -7502,7 +7502,7 @@
       </c>
       <c r="E170" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -7523,7 +7523,7 @@
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -7544,7 +7544,7 @@
       </c>
       <c r="E172" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>
@@ -7586,7 +7586,7 @@
       </c>
       <c r="E174" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:38</t>
+          <t xml:space="preserve">2026-09-14 23:43</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
prices: 2026-09-14 23:48 UTC
</commit_message>
<xml_diff>
--- a/docs/herblore_top8.xlsx
+++ b/docs/herblore_top8.xlsx
@@ -97,7 +97,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Last price update: 2026-09-14 23:43 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
+          <t xml:space="preserve">Last price update: 2026-09-14 23:48 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
         </is>
       </c>
     </row>
@@ -3978,7 +3978,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4062,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4146,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -4209,7 +4209,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -4377,7 +4377,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4608,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4713,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -4734,7 +4734,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -4902,7 +4902,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -4923,7 +4923,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -4965,7 +4965,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -5238,7 +5238,7 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5259,7 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -5322,7 +5322,7 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -5406,7 +5406,7 @@
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -5427,7 +5427,7 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5469,7 @@
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -5553,7 +5553,7 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -5574,7 +5574,7 @@
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -5595,7 +5595,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5637,7 @@
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5679,7 @@
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -5763,7 +5763,7 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -5931,7 +5931,7 @@
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -5952,7 +5952,7 @@
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -5973,7 +5973,7 @@
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -5994,7 +5994,7 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -6015,7 +6015,7 @@
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -6057,7 +6057,7 @@
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6120,7 @@
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6141,7 @@
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -6162,7 +6162,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -6225,7 +6225,7 @@
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -6246,7 +6246,7 @@
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6267,7 @@
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6288,7 @@
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6372,7 @@
       </c>
       <c r="E116" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -6393,7 +6393,7 @@
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -6414,7 +6414,7 @@
       </c>
       <c r="E118" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -6456,7 +6456,7 @@
       </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="E121" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="E124" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -6582,7 +6582,7 @@
       </c>
       <c r="E126" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -6666,7 +6666,7 @@
       </c>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -6687,7 +6687,7 @@
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -6729,7 +6729,7 @@
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -6750,7 +6750,7 @@
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -6792,7 +6792,7 @@
       </c>
       <c r="E136" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -6813,7 +6813,7 @@
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -6834,7 +6834,7 @@
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="E140" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -6897,7 +6897,7 @@
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -6918,7 +6918,7 @@
       </c>
       <c r="E142" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -6939,7 +6939,7 @@
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -6960,7 +6960,7 @@
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -6981,7 +6981,7 @@
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -7002,7 +7002,7 @@
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7023,7 @@
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -7044,7 +7044,7 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -7086,7 +7086,7 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -7107,7 +7107,7 @@
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -7128,7 +7128,7 @@
       </c>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7149,7 @@
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -7170,7 +7170,7 @@
       </c>
       <c r="E154" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -7229,7 +7229,7 @@
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="E158" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -7292,7 +7292,7 @@
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -7355,7 +7355,7 @@
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="E164" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -7397,7 +7397,7 @@
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7418,7 @@
       </c>
       <c r="E166" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7439,7 @@
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -7460,7 +7460,7 @@
       </c>
       <c r="E168" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -7481,7 +7481,7 @@
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -7502,7 +7502,7 @@
       </c>
       <c r="E170" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -7523,7 +7523,7 @@
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -7544,7 +7544,7 @@
       </c>
       <c r="E172" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>
@@ -7586,7 +7586,7 @@
       </c>
       <c r="E174" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:43</t>
+          <t xml:space="preserve">2026-09-14 23:48</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
prices: 2026-09-14 23:53 UTC
</commit_message>
<xml_diff>
--- a/docs/herblore_top8.xlsx
+++ b/docs/herblore_top8.xlsx
@@ -97,7 +97,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Last price update: 2026-09-14 23:48 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
+          <t xml:space="preserve">Last price update: 2026-09-14 23:53 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
         </is>
       </c>
     </row>
@@ -3978,7 +3978,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4062,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4146,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -4209,7 +4209,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -4377,7 +4377,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4608,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4713,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -4734,7 +4734,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -4902,7 +4902,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -4923,7 +4923,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -4965,7 +4965,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -5238,7 +5238,7 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5259,7 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -5322,7 +5322,7 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -5406,7 +5406,7 @@
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -5427,7 +5427,7 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5469,7 @@
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -5553,7 +5553,7 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -5574,7 +5574,7 @@
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -5595,7 +5595,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5637,7 @@
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5679,7 @@
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -5763,7 +5763,7 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -5931,7 +5931,7 @@
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -5952,7 +5952,7 @@
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -5973,7 +5973,7 @@
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -5994,7 +5994,7 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -6015,7 +6015,7 @@
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -6057,7 +6057,7 @@
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6120,7 @@
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6141,7 @@
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -6162,7 +6162,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -6225,7 +6225,7 @@
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -6246,7 +6246,7 @@
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6267,7 @@
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6288,7 @@
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6372,7 @@
       </c>
       <c r="E116" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -6393,7 +6393,7 @@
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -6414,7 +6414,7 @@
       </c>
       <c r="E118" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -6456,7 +6456,7 @@
       </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="E121" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="E124" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -6582,7 +6582,7 @@
       </c>
       <c r="E126" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -6666,7 +6666,7 @@
       </c>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -6687,7 +6687,7 @@
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -6729,7 +6729,7 @@
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -6750,7 +6750,7 @@
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -6792,7 +6792,7 @@
       </c>
       <c r="E136" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -6813,7 +6813,7 @@
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -6834,7 +6834,7 @@
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="E140" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -6897,7 +6897,7 @@
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -6918,7 +6918,7 @@
       </c>
       <c r="E142" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -6939,7 +6939,7 @@
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -6960,7 +6960,7 @@
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -6981,7 +6981,7 @@
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -7002,7 +7002,7 @@
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7023,7 @@
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -7044,7 +7044,7 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -7086,7 +7086,7 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -7107,7 +7107,7 @@
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -7128,7 +7128,7 @@
       </c>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7149,7 @@
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -7170,7 +7170,7 @@
       </c>
       <c r="E154" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -7229,7 +7229,7 @@
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="E158" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -7292,7 +7292,7 @@
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -7355,7 +7355,7 @@
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="E164" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -7397,7 +7397,7 @@
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7418,7 @@
       </c>
       <c r="E166" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7439,7 @@
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -7460,7 +7460,7 @@
       </c>
       <c r="E168" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -7481,7 +7481,7 @@
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -7502,7 +7502,7 @@
       </c>
       <c r="E170" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -7523,7 +7523,7 @@
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -7544,7 +7544,7 @@
       </c>
       <c r="E172" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>
@@ -7586,7 +7586,7 @@
       </c>
       <c r="E174" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:48</t>
+          <t xml:space="preserve">2026-09-14 23:53</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
prices: 2026-09-14 23:58 UTC
</commit_message>
<xml_diff>
--- a/docs/herblore_top8.xlsx
+++ b/docs/herblore_top8.xlsx
@@ -97,7 +97,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Last price update: 2026-09-14 23:53 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
+          <t xml:space="preserve">Last price update: 2026-09-14 23:58 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
         </is>
       </c>
     </row>
@@ -3978,7 +3978,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4062,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4146,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -4209,7 +4209,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -4377,7 +4377,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4608,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4713,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -4734,7 +4734,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -4902,7 +4902,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -4923,7 +4923,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -4965,7 +4965,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -5238,7 +5238,7 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5259,7 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -5322,7 +5322,7 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -5406,7 +5406,7 @@
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -5427,7 +5427,7 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5469,7 @@
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -5553,7 +5553,7 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -5574,7 +5574,7 @@
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -5595,7 +5595,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5637,7 @@
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5679,7 @@
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -5763,7 +5763,7 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -5931,7 +5931,7 @@
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -5952,7 +5952,7 @@
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -5973,7 +5973,7 @@
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -5994,7 +5994,7 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -6015,7 +6015,7 @@
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -6057,7 +6057,7 @@
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6120,7 @@
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6141,7 @@
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -6162,7 +6162,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -6225,7 +6225,7 @@
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -6246,7 +6246,7 @@
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6267,7 @@
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6288,7 @@
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6372,7 @@
       </c>
       <c r="E116" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -6393,7 +6393,7 @@
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -6414,7 +6414,7 @@
       </c>
       <c r="E118" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -6456,7 +6456,7 @@
       </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="E121" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="E124" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -6582,7 +6582,7 @@
       </c>
       <c r="E126" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -6666,7 +6666,7 @@
       </c>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -6687,7 +6687,7 @@
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -6729,7 +6729,7 @@
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -6750,7 +6750,7 @@
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -6792,7 +6792,7 @@
       </c>
       <c r="E136" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -6813,7 +6813,7 @@
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -6834,7 +6834,7 @@
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="E140" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -6897,7 +6897,7 @@
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -6918,7 +6918,7 @@
       </c>
       <c r="E142" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -6939,7 +6939,7 @@
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -6960,7 +6960,7 @@
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -6981,7 +6981,7 @@
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -7002,7 +7002,7 @@
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7023,7 @@
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -7044,7 +7044,7 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -7086,7 +7086,7 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -7107,7 +7107,7 @@
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -7128,7 +7128,7 @@
       </c>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7149,7 @@
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -7170,7 +7170,7 @@
       </c>
       <c r="E154" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -7229,7 +7229,7 @@
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="E158" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -7292,7 +7292,7 @@
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -7355,7 +7355,7 @@
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="E164" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -7397,7 +7397,7 @@
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7418,7 @@
       </c>
       <c r="E166" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7439,7 @@
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -7460,7 +7460,7 @@
       </c>
       <c r="E168" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -7481,7 +7481,7 @@
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -7502,7 +7502,7 @@
       </c>
       <c r="E170" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -7523,7 +7523,7 @@
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -7544,7 +7544,7 @@
       </c>
       <c r="E172" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>
@@ -7586,7 +7586,7 @@
       </c>
       <c r="E174" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:53</t>
+          <t xml:space="preserve">2026-09-14 23:58</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
prices: 2026-09-15 00:03 UTC
</commit_message>
<xml_diff>
--- a/docs/herblore_top8.xlsx
+++ b/docs/herblore_top8.xlsx
@@ -97,7 +97,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Last price update: 2026-09-14 23:58 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
+          <t xml:space="preserve">Last price update: 2026-09-15 00:03 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
         </is>
       </c>
     </row>
@@ -3978,7 +3978,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4062,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4146,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -4209,7 +4209,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -4377,7 +4377,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4608,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4713,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -4734,7 +4734,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -4902,7 +4902,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -4923,7 +4923,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -4965,7 +4965,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -5238,7 +5238,7 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5259,7 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -5322,7 +5322,7 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -5406,7 +5406,7 @@
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -5427,7 +5427,7 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5469,7 @@
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -5553,7 +5553,7 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -5574,7 +5574,7 @@
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -5595,7 +5595,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5637,7 @@
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5679,7 @@
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -5763,7 +5763,7 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -5931,7 +5931,7 @@
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -5952,7 +5952,7 @@
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -5973,7 +5973,7 @@
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -5994,7 +5994,7 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -6015,7 +6015,7 @@
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -6057,7 +6057,7 @@
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6120,7 @@
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6141,7 @@
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -6162,7 +6162,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -6225,7 +6225,7 @@
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -6246,7 +6246,7 @@
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6267,7 @@
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6288,7 @@
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6372,7 @@
       </c>
       <c r="E116" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -6393,7 +6393,7 @@
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -6414,7 +6414,7 @@
       </c>
       <c r="E118" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -6456,7 +6456,7 @@
       </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="E121" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="E124" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -6582,7 +6582,7 @@
       </c>
       <c r="E126" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -6666,7 +6666,7 @@
       </c>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -6687,7 +6687,7 @@
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -6729,7 +6729,7 @@
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -6750,7 +6750,7 @@
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -6792,7 +6792,7 @@
       </c>
       <c r="E136" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -6813,7 +6813,7 @@
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -6834,7 +6834,7 @@
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="E140" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -6897,7 +6897,7 @@
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -6918,7 +6918,7 @@
       </c>
       <c r="E142" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -6939,7 +6939,7 @@
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -6960,7 +6960,7 @@
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -6981,7 +6981,7 @@
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -7002,7 +7002,7 @@
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7023,7 @@
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -7044,7 +7044,7 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -7086,7 +7086,7 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -7107,7 +7107,7 @@
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -7128,7 +7128,7 @@
       </c>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7149,7 @@
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -7170,7 +7170,7 @@
       </c>
       <c r="E154" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -7229,7 +7229,7 @@
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="E158" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -7292,7 +7292,7 @@
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -7355,7 +7355,7 @@
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="E164" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -7397,7 +7397,7 @@
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7418,7 @@
       </c>
       <c r="E166" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7439,7 @@
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -7460,7 +7460,7 @@
       </c>
       <c r="E168" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -7481,7 +7481,7 @@
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -7502,7 +7502,7 @@
       </c>
       <c r="E170" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -7523,7 +7523,7 @@
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -7544,7 +7544,7 @@
       </c>
       <c r="E172" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>
@@ -7586,7 +7586,7 @@
       </c>
       <c r="E174" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-14 23:58</t>
+          <t xml:space="preserve">2026-09-15 00:03</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
prices: 2026-09-15 00:08 UTC
</commit_message>
<xml_diff>
--- a/docs/herblore_top8.xlsx
+++ b/docs/herblore_top8.xlsx
@@ -97,7 +97,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Last price update: 2026-09-15 00:03 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
+          <t xml:space="preserve">Last price update: 2026-09-15 00:08 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
         </is>
       </c>
     </row>
@@ -3978,7 +3978,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4062,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4146,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -4209,7 +4209,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -4377,7 +4377,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4608,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4713,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -4734,7 +4734,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -4902,7 +4902,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -4923,7 +4923,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -4965,7 +4965,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -5238,7 +5238,7 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5259,7 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -5322,7 +5322,7 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -5406,7 +5406,7 @@
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -5427,7 +5427,7 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5469,7 @@
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -5553,7 +5553,7 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -5574,7 +5574,7 @@
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -5595,7 +5595,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5637,7 @@
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5679,7 @@
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -5763,7 +5763,7 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -5931,7 +5931,7 @@
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -5952,7 +5952,7 @@
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -5973,7 +5973,7 @@
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -5994,7 +5994,7 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -6015,7 +6015,7 @@
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -6057,7 +6057,7 @@
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6120,7 @@
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6141,7 @@
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -6162,7 +6162,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -6225,7 +6225,7 @@
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -6246,7 +6246,7 @@
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6267,7 @@
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6288,7 @@
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6372,7 @@
       </c>
       <c r="E116" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -6393,7 +6393,7 @@
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -6414,7 +6414,7 @@
       </c>
       <c r="E118" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -6456,7 +6456,7 @@
       </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="E121" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="E124" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -6582,7 +6582,7 @@
       </c>
       <c r="E126" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -6666,7 +6666,7 @@
       </c>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -6687,7 +6687,7 @@
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -6729,7 +6729,7 @@
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -6750,7 +6750,7 @@
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -6792,7 +6792,7 @@
       </c>
       <c r="E136" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -6813,7 +6813,7 @@
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -6834,7 +6834,7 @@
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="E140" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -6897,7 +6897,7 @@
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -6918,7 +6918,7 @@
       </c>
       <c r="E142" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -6939,7 +6939,7 @@
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -6960,7 +6960,7 @@
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -6981,7 +6981,7 @@
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -7002,7 +7002,7 @@
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7023,7 @@
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -7044,7 +7044,7 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -7086,7 +7086,7 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -7107,7 +7107,7 @@
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -7128,7 +7128,7 @@
       </c>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7149,7 @@
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -7170,7 +7170,7 @@
       </c>
       <c r="E154" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -7229,7 +7229,7 @@
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="E158" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -7292,7 +7292,7 @@
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -7355,7 +7355,7 @@
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="E164" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -7397,7 +7397,7 @@
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7418,7 @@
       </c>
       <c r="E166" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7439,7 @@
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -7460,7 +7460,7 @@
       </c>
       <c r="E168" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -7481,7 +7481,7 @@
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -7502,7 +7502,7 @@
       </c>
       <c r="E170" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -7523,7 +7523,7 @@
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -7544,7 +7544,7 @@
       </c>
       <c r="E172" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>
@@ -7586,7 +7586,7 @@
       </c>
       <c r="E174" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:03</t>
+          <t xml:space="preserve">2026-09-15 00:08</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
prices: 2026-09-15 00:13 UTC
</commit_message>
<xml_diff>
--- a/docs/herblore_top8.xlsx
+++ b/docs/herblore_top8.xlsx
@@ -97,7 +97,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Last price update: 2026-09-15 00:08 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
+          <t xml:space="preserve">Last price update: 2026-09-15 00:13 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
         </is>
       </c>
     </row>
@@ -3978,7 +3978,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4062,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4146,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -4209,7 +4209,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -4377,7 +4377,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4608,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4713,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -4734,7 +4734,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -4902,7 +4902,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -4923,7 +4923,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -4965,7 +4965,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -5238,7 +5238,7 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5259,7 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -5322,7 +5322,7 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -5406,7 +5406,7 @@
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -5427,7 +5427,7 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5469,7 @@
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -5553,7 +5553,7 @@
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -5574,7 +5574,7 @@
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -5595,7 +5595,7 @@
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5637,7 @@
       </c>
       <c r="E81" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5679,7 @@
       </c>
       <c r="E83" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -5742,7 +5742,7 @@
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -5763,7 +5763,7 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -5931,7 +5931,7 @@
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -5952,7 +5952,7 @@
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -5973,7 +5973,7 @@
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -5994,7 +5994,7 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -6015,7 +6015,7 @@
       </c>
       <c r="E99" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -6057,7 +6057,7 @@
       </c>
       <c r="E101" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6120,7 @@
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6141,7 @@
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -6162,7 +6162,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -6225,7 +6225,7 @@
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -6246,7 +6246,7 @@
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6267,7 @@
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6288,7 @@
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="E113" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6372,7 @@
       </c>
       <c r="E116" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -6393,7 +6393,7 @@
       </c>
       <c r="E117" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -6414,7 +6414,7 @@
       </c>
       <c r="E118" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="E119" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -6456,7 +6456,7 @@
       </c>
       <c r="E120" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="E121" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -6498,7 +6498,7 @@
       </c>
       <c r="E122" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="E124" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -6561,7 +6561,7 @@
       </c>
       <c r="E125" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -6582,7 +6582,7 @@
       </c>
       <c r="E126" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="E127" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -6645,7 +6645,7 @@
       </c>
       <c r="E129" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -6666,7 +6666,7 @@
       </c>
       <c r="E130" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -6687,7 +6687,7 @@
       </c>
       <c r="E131" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="E132" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -6729,7 +6729,7 @@
       </c>
       <c r="E133" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -6750,7 +6750,7 @@
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
       </c>
       <c r="E135" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -6792,7 +6792,7 @@
       </c>
       <c r="E136" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -6813,7 +6813,7 @@
       </c>
       <c r="E137" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -6834,7 +6834,7 @@
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="E139" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="E140" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -6897,7 +6897,7 @@
       </c>
       <c r="E141" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -6918,7 +6918,7 @@
       </c>
       <c r="E142" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -6939,7 +6939,7 @@
       </c>
       <c r="E143" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -6960,7 +6960,7 @@
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -6981,7 +6981,7 @@
       </c>
       <c r="E145" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -7002,7 +7002,7 @@
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7023,7 @@
       </c>
       <c r="E147" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -7044,7 +7044,7 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="E149" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -7086,7 +7086,7 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -7107,7 +7107,7 @@
       </c>
       <c r="E151" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -7128,7 +7128,7 @@
       </c>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7149,7 @@
       </c>
       <c r="E153" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -7170,7 +7170,7 @@
       </c>
       <c r="E154" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -7229,7 +7229,7 @@
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="E158" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -7292,7 +7292,7 @@
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -7355,7 +7355,7 @@
       </c>
       <c r="E163" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="E164" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -7397,7 +7397,7 @@
       </c>
       <c r="E165" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -7418,7 +7418,7 @@
       </c>
       <c r="E166" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7439,7 @@
       </c>
       <c r="E167" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -7460,7 +7460,7 @@
       </c>
       <c r="E168" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -7481,7 +7481,7 @@
       </c>
       <c r="E169" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -7502,7 +7502,7 @@
       </c>
       <c r="E170" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -7523,7 +7523,7 @@
       </c>
       <c r="E171" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -7544,7 +7544,7 @@
       </c>
       <c r="E172" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="E173" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>
@@ -7586,7 +7586,7 @@
       </c>
       <c r="E174" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:08</t>
+          <t xml:space="preserve">2026-09-15 00:13</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
prices: 2026-09-15 00:18 UTC
</commit_message>
<xml_diff>
--- a/docs/herblore_top8.xlsx
+++ b/docs/herblore_top8.xlsx
@@ -97,7 +97,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Last price update: 2026-09-15 00:13 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
+          <t xml:space="preserve">Last price update: 2026-09-15 00:18 UTC — auto-refreshes every 5 minutes (server.mjs). Source: wiki median GE price (buy=sell=median).</t>
         </is>
       </c>
     </row>
@@ -3978,7 +3978,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -4062,7 +4062,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4146,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -4209,7 +4209,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -4377,7 +4377,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -4419,7 +4419,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4608,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4713,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -4734,7 +4734,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -4902,7 +4902,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -4923,7 +4923,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -4965,7 +4965,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -5238,7 +5238,7 @@
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5259,7 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -5322,7 +5322,7 @@
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-15 00:13</t>
+          <t xml:space="preserve">2026-09-15 00:18</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t xml:space="prese